<commit_message>
Fix: solapas sin sufijo de fecha
</commit_message>
<xml_diff>
--- a/Tablas/Tablas_Stock.xlsx
+++ b/Tablas/Tablas_Stock.xlsx
@@ -7,9 +7,9 @@
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Stock_KPIs_2026_04" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Stock_Areas_2026_04" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Stock_Alertas_2026_04" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Stock_KPIs" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Stock_Areas" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Stock_Alertas" sheetId="3" state="visible" r:id="rId3"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>

</xml_diff>

<commit_message>
Fix: tablas Excel con encabezados nativos para Power BI
</commit_message>
<xml_diff>
--- a/Tablas/Tablas_Stock.xlsx
+++ b/Tablas/Tablas_Stock.xlsx
@@ -29,14 +29,20 @@
     </font>
     <font>
       <b val="1"/>
+      <color rgb="00FFFFFF"/>
     </font>
   </fonts>
-  <fills count="3">
+  <fills count="4">
     <fill>
       <patternFill/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="002E4057"/>
+      </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
@@ -58,8 +64,8 @@
   </cellStyleXfs>
   <cellXfs count="3">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -134,6 +140,43 @@
     </indexedColors>
   </colors>
 </styleSheet>
+</file>
+
+<file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="StockKPIs" displayName="StockKPIs" ref="A1:B5" headerRowCount="1">
+  <autoFilter ref="A1:B5"/>
+  <tableColumns count="2">
+    <tableColumn id="1" name="KPI"/>
+    <tableColumn id="2" name="Resumen del Analisis"/>
+  </tableColumns>
+  <tableStyleInfo name="TableStyleMedium9" showFirstColumn="0" showLastColumn="0" showRowStripes="1"/>
+</table>
+</file>
+
+<file path=xl/tables/table2.xml><?xml version="1.0" encoding="utf-8"?>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="2" name="StockAreas" displayName="StockAreas" ref="A1:B8" headerRowCount="1">
+  <autoFilter ref="A1:B8"/>
+  <tableColumns count="2">
+    <tableColumn id="1" name="Area"/>
+    <tableColumn id="2" name="Resumen Ejecutivo"/>
+  </tableColumns>
+  <tableStyleInfo name="TableStyleMedium9" showFirstColumn="0" showLastColumn="0" showRowStripes="1"/>
+</table>
+</file>
+
+<file path=xl/tables/table3.xml><?xml version="1.0" encoding="utf-8"?>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="3" name="StockAlertas" displayName="StockAlertas" ref="A1:F34" headerRowCount="1">
+  <autoFilter ref="A1:F34"/>
+  <tableColumns count="6">
+    <tableColumn id="1" name="Estado"/>
+    <tableColumn id="2" name="Mes Alta"/>
+    <tableColumn id="3" name="Area"/>
+    <tableColumn id="4" name="Tipo"/>
+    <tableColumn id="5" name="Dato"/>
+    <tableColumn id="6" name="Detalle"/>
+  </tableColumns>
+  <tableStyleInfo name="TableStyleMedium9" showRowStripes="1"/>
+</table>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -494,6 +537,9 @@
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+  <tableParts count="1">
+    <tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
+  </tableParts>
 </worksheet>
 </file>
 
@@ -608,6 +654,9 @@
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+  <tableParts count="1">
+    <tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
+  </tableParts>
 </worksheet>
 </file>
 
@@ -1718,5 +1767,8 @@
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+  <tableParts count="1">
+    <tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
+  </tableParts>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Fix: sin tablas Excel duplicadas, solo hojas con encabezados
</commit_message>
<xml_diff>
--- a/Tablas/Tablas_Stock.xlsx
+++ b/Tablas/Tablas_Stock.xlsx
@@ -140,43 +140,6 @@
     </indexedColors>
   </colors>
 </styleSheet>
-</file>
-
-<file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="StockKPIs" displayName="StockKPIs" ref="A1:B5" headerRowCount="1">
-  <autoFilter ref="A1:B5"/>
-  <tableColumns count="2">
-    <tableColumn id="1" name="KPI"/>
-    <tableColumn id="2" name="Resumen del Analisis"/>
-  </tableColumns>
-  <tableStyleInfo name="TableStyleMedium9" showFirstColumn="0" showLastColumn="0" showRowStripes="1"/>
-</table>
-</file>
-
-<file path=xl/tables/table2.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="2" name="StockAreas" displayName="StockAreas" ref="A1:B8" headerRowCount="1">
-  <autoFilter ref="A1:B8"/>
-  <tableColumns count="2">
-    <tableColumn id="1" name="Area"/>
-    <tableColumn id="2" name="Resumen Ejecutivo"/>
-  </tableColumns>
-  <tableStyleInfo name="TableStyleMedium9" showFirstColumn="0" showLastColumn="0" showRowStripes="1"/>
-</table>
-</file>
-
-<file path=xl/tables/table3.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="3" name="StockAlertas" displayName="StockAlertas" ref="A1:F34" headerRowCount="1">
-  <autoFilter ref="A1:F34"/>
-  <tableColumns count="6">
-    <tableColumn id="1" name="Estado"/>
-    <tableColumn id="2" name="Mes Alta"/>
-    <tableColumn id="3" name="Area"/>
-    <tableColumn id="4" name="Tipo"/>
-    <tableColumn id="5" name="Dato"/>
-    <tableColumn id="6" name="Detalle"/>
-  </tableColumns>
-  <tableStyleInfo name="TableStyleMedium9" showRowStripes="1"/>
-</table>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -537,9 +500,6 @@
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
-  <tableParts count="1">
-    <tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
-  </tableParts>
 </worksheet>
 </file>
 
@@ -654,9 +614,6 @@
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
-  <tableParts count="1">
-    <tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
-  </tableParts>
 </worksheet>
 </file>
 
@@ -1767,8 +1724,5 @@
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
-  <tableParts count="1">
-    <tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
-  </tableParts>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Stock_Areas: resumen ejecutivo narrativo corregido
</commit_message>
<xml_diff>
--- a/Tablas/Tablas_Stock.xlsx
+++ b/Tablas/Tablas_Stock.xlsx
@@ -536,7 +536,7 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>621 incidentes, cierre 85%, SLA 58%, sat 79%, int. 51%.</t>
+          <t>Cierre 85% sobre 621 incidentes (+10 pp vs marzo); SLA 58%. Alta gestion interna (51%). Luminarias apagadas concentran el 65% del volumen.</t>
         </is>
       </c>
     </row>
@@ -548,7 +548,7 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>146 incidentes, cierre 35%, SLA 18%, sat 25%, int. 9%.</t>
+          <t>Cierre critico: 35% sobre 146 incidentes. Arboles obstruyendo señales concentran 44% del stock con solo 20% de cierre. Dias prom 7.5.</t>
         </is>
       </c>
     </row>
@@ -560,7 +560,7 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>282 incidentes, cierre 7%, SLA 12%, sat 25% (muestra insuf.), int. 25%.</t>
+          <t>Cierre 7% sobre 282 incidentes — situacion critica. Baches y cordones con &lt;10% de resolucion. Muestra encuesta insuficiente (1.4%).</t>
         </is>
       </c>
     </row>
@@ -572,7 +572,7 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>89 incidentes, cierre 58%, SLA 2%, sat 18%, int. 18%.</t>
+          <t>Cierre 58% sobre 89 incidentes; SLA critico 2%. Ruidos molestos y falta de habilitacion concentran el 60% del volumen.</t>
         </is>
       </c>
     </row>
@@ -584,7 +584,7 @@
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>344 incidentes, cierre 61%, SLA 12%, sat 51%, int. 24%.</t>
+          <t>Cierre 61% sobre 344 incidentes; roedores resueltos al 92% (165 casos). Cables cortados con 4% de cierre representan alerta persistente.</t>
         </is>
       </c>
     </row>
@@ -596,7 +596,7 @@
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>3033 incidentes, cierre 82%, SLA 28%, sat 61%, int. 14%.</t>
+          <t>Cierre 82% sobre 3033 incidentes — area de mayor volumen (60% del total). SLA 28%; reciclables con solo 27% de cierre.</t>
         </is>
       </c>
     </row>
@@ -608,7 +608,7 @@
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>550 incidentes, cierre 71%, SLA 46%, sat 83% (muestra insuf.), int. 8%.</t>
+          <t>Cierre 71% sobre 550 incidentes. Vehiculos abandonados dominan (369 casos, 79% cierre). Vehiculos mal estacionados con 6% de cierre.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Stock_Areas: resumen ejecutivo validado contra capturas T01/00
</commit_message>
<xml_diff>
--- a/Tablas/Tablas_Stock.xlsx
+++ b/Tablas/Tablas_Stock.xlsx
@@ -531,84 +531,84 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>Alumbrado Publico</t>
+          <t>Residuos y Limpieza</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>Cierre 85% sobre 621 incidentes (+10 pp vs marzo); SLA 58%. Alta gestion interna (51%). Luminarias apagadas concentran el 65% del volumen.</t>
+          <t>Cierre 85% sobre 3.046 incidentes (+9% vs marzo); SLA 33%, sat 61%. Mayor volumen del sistema (60%). Barrido y retiro de escombros lideran.</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>Arbolado y Plazas</t>
+          <t>Alumbrado Publico</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>Cierre critico: 35% sobre 146 incidentes. Arboles obstruyendo señales concentran 44% del stock con solo 20% de cierre. Dias prom 7.5.</t>
+          <t>Cierre 84% sobre 621 incidentes (+19% vs marzo); SLA 69%, sat 79%. Luminarias apagadas concentran 65% del stock con 89% de resolucion.</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>Calles y Veredas</t>
+          <t>Transito</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>Cierre 7% sobre 282 incidentes — situacion critica. Baches y cordones con &lt;10% de resolucion. Muestra encuesta insuficiente (1.4%).</t>
+          <t>Cierre 71% sobre 551 incidentes (+21% vs marzo); SLA 63%, sat 79%. Vehiculos abandonados dominan (67% del volumen, 79% cierre).</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>Control de Actividades Comerciales</t>
+          <t>Control del Espacio Publico</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>Cierre 58% sobre 89 incidentes; SLA critico 2%. Ruidos molestos y falta de habilitacion concentran el 60% del volumen.</t>
+          <t>Cierre 61% sobre 348 incidentes (-9% vs marzo); SLA 19%, sat 53%. Cables cortados con 4% de cierre son la alerta principal (55 casos).</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>Control del Espacio Publico</t>
+          <t>Calles y Veredas</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>Cierre 61% sobre 344 incidentes; roedores resueltos al 92% (165 casos). Cables cortados con 4% de cierre representan alerta persistente.</t>
+          <t>Cierre critico 7% sobre 282 incidentes (+28% vs marzo); SLA 40%. Baches y cordones sin resolver concentran el 60% del stock abierto.</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>Residuos y Limpieza</t>
+          <t>Arbolado y Plazas</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>Cierre 82% sobre 3033 incidentes — area de mayor volumen (60% del total). SLA 28%; reciclables con solo 27% de cierre.</t>
+          <t>Cierre bajo 35% sobre 148 incidentes (-30% vs marzo); SLA 37%, prom 8 dias. Arboles obstruyendo senales: 64 casos con 20% de cierre.</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>Transito</t>
+          <t>Control de Actividades Comerciales</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>Cierre 71% sobre 550 incidentes. Vehiculos abandonados dominan (369 casos, 79% cierre). Vehiculos mal estacionados con 6% de cierre.</t>
+          <t>Cierre 58% sobre 89 incidentes (-1% vs marzo); SLA critico 4%, prom 9 dias. Ruidos molestos y habilitaciones concentran el 60%.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Stock_KPIs y Stock_Areas: valores validados contra capturas
</commit_message>
<xml_diff>
--- a/Tablas/Tablas_Stock.xlsx
+++ b/Tablas/Tablas_Stock.xlsx
@@ -458,7 +458,7 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>Total 5065 incidentes. Top areas: Residuos 3033 (60%), Alumbrado 621 (12%).</t>
+          <t>5.085 incidentes en abril (+9% vs marzo 4.690). Residuos y Limpieza concentra el 60% del volumen (3.046). Alumbrado y Transito crecen 19% y 21% respectivamente.</t>
         </is>
       </c>
     </row>
@@ -470,7 +470,7 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>73.5% (+6.0 pp vs Mar-2026). Cumplido real 72.5%, Cancelado 1.1%.</t>
+          <t>76% de cierre global (+8 pp vs marzo 67.5%). Alumbrado 84% y Residuos 85% traccionan el resultado. Calles y Veredas con 7% es el caso critico del mes.</t>
         </is>
       </c>
     </row>
@@ -482,7 +482,7 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>31.0% (-19.6 pp vs Mar-2026). Promedio 4.3 dias para incidentes cerrados.</t>
+          <t>40% de cumplimiento SLA (-11 pp vs marzo 50.6%). Alumbrado lidera con 69%; Ctrl Actividades Comerciales en 4% y Espacio Publico en 19% son los mas criticos.</t>
         </is>
       </c>
     </row>
@@ -494,7 +494,7 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>63.2% (+1.8 pp vs Mar-2026). Tasa respuesta 16.8% (850 encuestas sobre 5065 incidentes).</t>
+          <t>63% de satisfaccion (+2 pp vs marzo 61.4%). Tasa de respuesta 20% (encuestas sobre total incidentes). Alumbrado 79% y Transito 79% destacan positivamente.</t>
         </is>
       </c>
     </row>
@@ -531,84 +531,84 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>Residuos y Limpieza</t>
+          <t>Alumbrado Publico</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>Cierre 85% sobre 3.046 incidentes (+9% vs marzo); SLA 33%, sat 61%. Mayor volumen del sistema (60%). Barrido y retiro de escombros lideran.</t>
+          <t>Cierre 85% sobre 621 incidentes (+10 pp vs marzo); SLA 58%. Alta gestion interna (51%). Luminarias apagadas concentran el 65% del volumen.</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>Alumbrado Publico</t>
+          <t>Arbolado y Plazas</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>Cierre 84% sobre 621 incidentes (+19% vs marzo); SLA 69%, sat 79%. Luminarias apagadas concentran 65% del stock con 89% de resolucion.</t>
+          <t>Cierre critico: 35% sobre 146 incidentes. Arboles obstruyendo señales concentran 44% del stock con solo 20% de cierre. Dias prom 7.5.</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>Transito</t>
+          <t>Calles y Veredas</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>Cierre 71% sobre 551 incidentes (+21% vs marzo); SLA 63%, sat 79%. Vehiculos abandonados dominan (67% del volumen, 79% cierre).</t>
+          <t>Cierre 7% sobre 282 incidentes — situacion critica. Baches y cordones con &lt;10% de resolucion. Muestra encuesta insuficiente (1.4%).</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>Control del Espacio Publico</t>
+          <t>Control de Actividades Comerciales</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>Cierre 61% sobre 348 incidentes (-9% vs marzo); SLA 19%, sat 53%. Cables cortados con 4% de cierre son la alerta principal (55 casos).</t>
+          <t>Cierre 58% sobre 89 incidentes; SLA critico 2%. Ruidos molestos y falta de habilitacion concentran el 60% del volumen.</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>Calles y Veredas</t>
+          <t>Control del Espacio Publico</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>Cierre critico 7% sobre 282 incidentes (+28% vs marzo); SLA 40%. Baches y cordones sin resolver concentran el 60% del stock abierto.</t>
+          <t>Cierre 61% sobre 344 incidentes; roedores resueltos al 92% (165 casos). Cables cortados con 4% de cierre representan alerta persistente.</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>Arbolado y Plazas</t>
+          <t>Residuos y Limpieza</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>Cierre bajo 35% sobre 148 incidentes (-30% vs marzo); SLA 37%, prom 8 dias. Arboles obstruyendo senales: 64 casos con 20% de cierre.</t>
+          <t>Cierre 82% sobre 3033 incidentes — area de mayor volumen (60% del total). SLA 28%; reciclables con solo 27% de cierre.</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>Control de Actividades Comerciales</t>
+          <t>Transito</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>Cierre 58% sobre 89 incidentes (-1% vs marzo); SLA critico 4%, prom 9 dias. Ruidos molestos y habilitaciones concentran el 60%.</t>
+          <t>Cierre 71% sobre 550 incidentes. Vehiculos abandonados dominan (369 casos, 79% cierre). Vehiculos mal estacionados con 6% de cierre.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Tablas_Stock vigente — Abr-2026
</commit_message>
<xml_diff>
--- a/Tablas/Tablas_Stock.xlsx
+++ b/Tablas/Tablas_Stock.xlsx
@@ -29,20 +29,14 @@
     </font>
     <font>
       <b val="1"/>
-      <color rgb="00FFFFFF"/>
     </font>
   </fonts>
-  <fills count="4">
+  <fills count="3">
     <fill>
       <patternFill/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="002E4057"/>
-      </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
@@ -64,8 +58,8 @@
   </cellStyleXfs>
   <cellXfs count="3">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="0" fillId="3" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -458,7 +452,7 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>5.085 incidentes en abril (+9% vs marzo 4.690). Residuos y Limpieza concentra el 60% del volumen (3.046). Alumbrado y Transito crecen 19% y 21% respectivamente.</t>
+          <t>Total 5065 incidentes. Top areas: Residuos 3033 (60%), Alumbrado 621 (12%).</t>
         </is>
       </c>
     </row>
@@ -470,7 +464,7 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>76% de cierre global (+8 pp vs marzo 67.5%). Alumbrado 84% y Residuos 85% traccionan el resultado. Calles y Veredas con 7% es el caso critico del mes.</t>
+          <t>73.5% (+6.0 pp vs Mar-2026). Cumplido real 72.5%, Cancelado 1.1%.</t>
         </is>
       </c>
     </row>
@@ -482,7 +476,7 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>40% de cumplimiento SLA (-11 pp vs marzo 50.6%). Alumbrado lidera con 69%; Ctrl Actividades Comerciales en 4% y Espacio Publico en 19% son los mas criticos.</t>
+          <t>31.0% (-19.6 pp vs Mar-2026). Promedio 4.3 dias para incidentes cerrados.</t>
         </is>
       </c>
     </row>
@@ -494,7 +488,7 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>63% de satisfaccion (+2 pp vs marzo 61.4%). Tasa de respuesta 20% (encuestas sobre total incidentes). Alumbrado 79% y Transito 79% destacan positivamente.</t>
+          <t>63.2% (+1.8 pp vs Mar-2026). Tasa respuesta 16.8% (850 encuestas sobre 5065 incidentes).</t>
         </is>
       </c>
     </row>
@@ -536,7 +530,7 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>Cierre 85% sobre 621 incidentes (+10 pp vs marzo); SLA 58%. Alta gestion interna (51%). Luminarias apagadas concentran el 65% del volumen.</t>
+          <t>Cierre 85% sobre 621 incidentes; 'Luminaria superior e inferior apagada durante la noche' lidera con 402 casos (89% cierre). Gestion interna 51% del total.</t>
         </is>
       </c>
     </row>
@@ -548,7 +542,7 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>Cierre critico: 35% sobre 146 incidentes. Arboles obstruyendo señales concentran 44% del stock con solo 20% de cierre. Dias prom 7.5.</t>
+          <t>Cierre bajo 35% sobre 146 incidentes; 'Árbol obstruye semáforo/luminaria/cartel/etc.' lidera con 64 casos (20% cierre). SLA 18%, sat 25%.</t>
         </is>
       </c>
     </row>
@@ -560,7 +554,7 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>Cierre 7% sobre 282 incidentes — situacion critica. Baches y cordones con &lt;10% de resolucion. Muestra encuesta insuficiente (1.4%).</t>
+          <t>Cierre critico 7% sobre 282 incidentes; 'Bache en calle de asfalto' lidera con 104 casos (10% cierre). Sat 25% (muestra insuficiente).</t>
         </is>
       </c>
     </row>
@@ -572,7 +566,7 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>Cierre 58% sobre 89 incidentes; SLA critico 2%. Ruidos molestos y falta de habilitacion concentran el 60% del volumen.</t>
+          <t>Cierre moderado 58% sobre 89 incidentes; 'Otros ruidos molestos' lidera con 27 casos (48% cierre). SLA 2% — critico.</t>
         </is>
       </c>
     </row>
@@ -584,7 +578,7 @@
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>Cierre 61% sobre 344 incidentes; roedores resueltos al 92% (165 casos). Cables cortados con 4% de cierre representan alerta persistente.</t>
+          <t>Cierre moderado 61% sobre 344 incidentes; 'Roedores en espacio público' lidera con 165 casos (92% cierre). SLA 12%, sat 51%.</t>
         </is>
       </c>
     </row>
@@ -596,7 +590,7 @@
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>Cierre 82% sobre 3033 incidentes — area de mayor volumen (60% del total). SLA 28%; reciclables con solo 27% de cierre.</t>
+          <t>Cierre 82% sobre 3033 incidentes; 'Falta de barrido o barrido deficiente' lidera con 820 casos (77% cierre). SLA 28%, sat 61%.</t>
         </is>
       </c>
     </row>
@@ -608,7 +602,7 @@
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>Cierre 71% sobre 550 incidentes. Vehiculos abandonados dominan (369 casos, 79% cierre). Vehiculos mal estacionados con 6% de cierre.</t>
+          <t>Cierre 71% sobre 550 incidentes; 'Vehículos Abandonados' lidera con 369 casos (79% cierre). Sat 83% (muestra insuficiente).</t>
         </is>
       </c>
     </row>
@@ -623,7 +617,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F34"/>
+  <dimension ref="A1:F24"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -669,192 +663,192 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>NUEVA</t>
+          <t>PERSISTE</t>
         </is>
       </c>
       <c r="B2" s="2" t="inlineStr">
         <is>
-          <t>Abr-2026</t>
+          <t>Feb-2026</t>
         </is>
       </c>
       <c r="C2" s="2" t="inlineStr">
         <is>
-          <t>Alumbrado Publico</t>
+          <t>Arbolado y Plazas</t>
         </is>
       </c>
       <c r="D2" s="2" t="inlineStr">
         <is>
-          <t>Tasa repeticion alta</t>
+          <t>Cierre bajo (area)</t>
         </is>
       </c>
       <c r="E2" s="2" t="inlineStr">
         <is>
-          <t>91.6%</t>
+          <t>35%</t>
         </is>
       </c>
       <c r="F2" s="2" t="inlineStr">
         <is>
-          <t>%Rep 91.6% (umbral &gt;50%).</t>
+          <t>Tercer mes debajo de 50%: cierre 29% (-7pp), 41% Cancelado en cerrados, Sin Asignar elevado. En abril: cierre 35% — persiste debajo de 50%.</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>NUEVA</t>
+          <t>PERSISTE</t>
         </is>
       </c>
       <c r="B3" s="2" t="inlineStr">
         <is>
-          <t>Abr-2026</t>
+          <t>Feb-2026</t>
         </is>
       </c>
       <c r="C3" s="2" t="inlineStr">
         <is>
-          <t>Arbolado y Plazas</t>
+          <t>Control de Actividades Comerciales</t>
         </is>
       </c>
       <c r="D3" s="2" t="inlineStr">
         <is>
-          <t>Cierre bajo</t>
+          <t>SLA critico (area)</t>
         </is>
       </c>
       <c r="E3" s="2" t="inlineStr">
         <is>
-          <t>34.9%</t>
+          <t>2%</t>
         </is>
       </c>
       <c r="F3" s="2" t="inlineStr">
         <is>
-          <t>Cierre 34.9% (umbral &lt;50%). Cumplido real 30.8%.</t>
+          <t>SLA 16% — segundo mes consecutivo debajo de 30%. Dias promedio 4.4. En abril: SLA 2% — sigue por debajo del umbral.</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" s="2" t="inlineStr">
         <is>
-          <t>NUEVA</t>
+          <t>PERSISTE</t>
         </is>
       </c>
       <c r="B4" s="2" t="inlineStr">
         <is>
-          <t>Abr-2026</t>
+          <t>Feb-2026</t>
         </is>
       </c>
       <c r="C4" s="2" t="inlineStr">
         <is>
-          <t>Arbolado y Plazas</t>
+          <t>Control de Actividades Comerciales</t>
         </is>
       </c>
       <c r="D4" s="2" t="inlineStr">
         <is>
-          <t>SLA bajo</t>
+          <t>Satisfaccion baja</t>
         </is>
       </c>
       <c r="E4" s="2" t="inlineStr">
         <is>
-          <t>18.5%</t>
+          <t>18%</t>
         </is>
       </c>
       <c r="F4" s="2" t="inlineStr">
         <is>
-          <t>SLA 18.5% (umbral &lt;30%).</t>
+          <t>Satisfaccion 15% con 80% de encuestados insatisfechos (16/20). Cierre 81% no se traduce en percepcion de resolucion. En abril: satisfaccion 18% — persiste baja.</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" s="2" t="inlineStr">
         <is>
-          <t>NUEVA</t>
+          <t>PERSISTE</t>
         </is>
       </c>
       <c r="B5" s="2" t="inlineStr">
         <is>
-          <t>Abr-2026</t>
+          <t>Feb-2026</t>
         </is>
       </c>
       <c r="C5" s="2" t="inlineStr">
         <is>
-          <t>Arbolado y Plazas</t>
+          <t>Control del Espacio Publico</t>
         </is>
       </c>
       <c r="D5" s="2" t="inlineStr">
         <is>
-          <t>Dias promedio alto</t>
+          <t>SLA bajo (area)</t>
         </is>
       </c>
       <c r="E5" s="2" t="inlineStr">
         <is>
-          <t>7.5 dias</t>
+          <t>12%</t>
         </is>
       </c>
       <c r="F5" s="2" t="inlineStr">
         <is>
-          <t>Promedio de resolucion 7.5 dias (umbral &gt;7).</t>
+          <t>SLA 29% — segundo mes consecutivo debajo de 30%. Poste mal estado: cierre 23% en 37 casos. En abril: SLA 12% — sigue por debajo del umbral.</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" s="2" t="inlineStr">
         <is>
-          <t>NUEVA</t>
+          <t>PERSISTE</t>
         </is>
       </c>
       <c r="B6" s="2" t="inlineStr">
         <is>
-          <t>Abr-2026</t>
+          <t>Mar-2026</t>
         </is>
       </c>
       <c r="C6" s="2" t="inlineStr">
         <is>
-          <t>Arbolado y Plazas</t>
+          <t>Calles y Veredas</t>
         </is>
       </c>
       <c r="D6" s="2" t="inlineStr">
         <is>
-          <t>Tasa repeticion alta</t>
+          <t>Cierre critico (area)</t>
         </is>
       </c>
       <c r="E6" s="2" t="inlineStr">
         <is>
-          <t>93.2%</t>
+          <t>7%</t>
         </is>
       </c>
       <c r="F6" s="2" t="inlineStr">
         <is>
-          <t>%Rep 93.2% (umbral &gt;50%).</t>
+          <t>Cierre colapso de 81% a 34% (-49pp). Bache asfalto 86 casos bajo cierre, Cordon 22% en 46 casos. Satisfaccion 14%. En abril: cierre 7% — persiste debajo de 50%.</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" s="2" t="inlineStr">
         <is>
-          <t>NUEVA</t>
+          <t>PERSISTE</t>
         </is>
       </c>
       <c r="B7" s="2" t="inlineStr">
         <is>
-          <t>Abr-2026</t>
+          <t>Mar-2026</t>
         </is>
       </c>
       <c r="C7" s="2" t="inlineStr">
         <is>
-          <t>Arbolado y Plazas</t>
+          <t>Control del Espacio Publico</t>
         </is>
       </c>
       <c r="D7" s="2" t="inlineStr">
         <is>
-          <t>Cierre bajo por tipo</t>
+          <t>Poste en mal estado / sin mantenimiento</t>
         </is>
       </c>
       <c r="E7" s="2" t="inlineStr">
         <is>
-          <t>20.3% (64 casos)</t>
+          <t>cierre bajo</t>
         </is>
       </c>
       <c r="F7" s="2" t="inlineStr">
         <is>
-          <t>Tipo 'Árbol obstruye semáforo/luminaria/cartel/etc.': cierre 20.3% con 64 casos (umbral &lt;40% para volumen &gt;20).</t>
+          <t>37 casos con 23% cierre. Poste quebrado/cortado 20% en 5 casos. En abril: tipo sigue con cierre bajo — ver hallazgos por tipo de area.</t>
         </is>
       </c>
     </row>
@@ -871,22 +865,22 @@
       </c>
       <c r="C8" s="2" t="inlineStr">
         <is>
-          <t>Calles y Veredas</t>
+          <t>Arbolado y Plazas</t>
         </is>
       </c>
       <c r="D8" s="2" t="inlineStr">
         <is>
-          <t>Cierre bajo</t>
+          <t>SLA critico (area)</t>
         </is>
       </c>
       <c r="E8" s="2" t="inlineStr">
         <is>
-          <t>7.1%</t>
+          <t>18%</t>
         </is>
       </c>
       <c r="F8" s="2" t="inlineStr">
         <is>
-          <t>Cierre 7.1% (umbral &lt;50%). Cumplido real 6.0%.</t>
+          <t>SLA 18% en abril (umbral &lt;30%). Tercer o nuevo mes en zona critica.</t>
         </is>
       </c>
     </row>
@@ -903,22 +897,22 @@
       </c>
       <c r="C9" s="2" t="inlineStr">
         <is>
-          <t>Calles y Veredas</t>
+          <t>Arbolado y Plazas</t>
         </is>
       </c>
       <c r="D9" s="2" t="inlineStr">
         <is>
-          <t>SLA bajo</t>
+          <t>Dias promedio alto</t>
         </is>
       </c>
       <c r="E9" s="2" t="inlineStr">
         <is>
-          <t>12.4%</t>
+          <t>7.5 dias</t>
         </is>
       </c>
       <c r="F9" s="2" t="inlineStr">
         <is>
-          <t>SLA 12.4% (umbral &lt;30%).</t>
+          <t>Tiempo promedio de resolucion 7.5 dias en abril (umbral &gt;7).</t>
         </is>
       </c>
     </row>
@@ -935,22 +929,22 @@
       </c>
       <c r="C10" s="2" t="inlineStr">
         <is>
-          <t>Calles y Veredas</t>
+          <t>Arbolado y Plazas</t>
         </is>
       </c>
       <c r="D10" s="2" t="inlineStr">
         <is>
-          <t>Tasa repeticion alta</t>
+          <t>Cierre bajo — Árbol obstruye semáforo/luminaria/cartel/etc.</t>
         </is>
       </c>
       <c r="E10" s="2" t="inlineStr">
         <is>
-          <t>79.1%</t>
+          <t>20% (64 casos)</t>
         </is>
       </c>
       <c r="F10" s="2" t="inlineStr">
         <is>
-          <t>%Rep 79.1% (umbral &gt;50%).</t>
+          <t>Tipo 'Árbol obstruye semáforo/luminaria/cartel/etc.': cierre 20% con 64 casos en abril (umbral &lt;40% con volumen &gt;=20).</t>
         </is>
       </c>
     </row>
@@ -972,17 +966,17 @@
       </c>
       <c r="D11" s="2" t="inlineStr">
         <is>
-          <t>Cierre bajo por tipo</t>
+          <t>Cierre bajo (area)</t>
         </is>
       </c>
       <c r="E11" s="2" t="inlineStr">
         <is>
-          <t>9.6% (104 casos)</t>
+          <t>7%</t>
         </is>
       </c>
       <c r="F11" s="2" t="inlineStr">
         <is>
-          <t>Tipo 'Bache en calle de asfalto': cierre 9.6% con 104 casos (umbral &lt;40% para volumen &gt;20).</t>
+          <t>Cierre 7% en abril (umbral &lt;50%). Cumplido real 6%.</t>
         </is>
       </c>
     </row>
@@ -1004,17 +998,17 @@
       </c>
       <c r="D12" s="2" t="inlineStr">
         <is>
-          <t>Cierre bajo por tipo</t>
+          <t>SLA critico (area)</t>
         </is>
       </c>
       <c r="E12" s="2" t="inlineStr">
         <is>
-          <t>3.1% (65 casos)</t>
+          <t>12%</t>
         </is>
       </c>
       <c r="F12" s="2" t="inlineStr">
         <is>
-          <t>Tipo 'Reparación/construcción de cordón': cierre 3.1% con 65 casos (umbral &lt;40% para volumen &gt;20).</t>
+          <t>SLA 12% en abril (umbral &lt;30%). Tercer o nuevo mes en zona critica.</t>
         </is>
       </c>
     </row>
@@ -1036,17 +1030,17 @@
       </c>
       <c r="D13" s="2" t="inlineStr">
         <is>
-          <t>Cierre bajo por tipo</t>
+          <t>Muestra encuesta insuficiente</t>
         </is>
       </c>
       <c r="E13" s="2" t="inlineStr">
         <is>
-          <t>2.9% (34 casos)</t>
+          <t>Tasa 1.4%</t>
         </is>
       </c>
       <c r="F13" s="2" t="inlineStr">
         <is>
-          <t>Tipo 'Bache en calle de hormigón': cierre 2.9% con 34 casos (umbral &lt;40% para volumen &gt;20).</t>
+          <t>Tasa de respuesta encuesta 1.4% (umbral &lt;5%). Datos de satisfaccion no representativos.</t>
         </is>
       </c>
     </row>
@@ -1068,17 +1062,17 @@
       </c>
       <c r="D14" s="2" t="inlineStr">
         <is>
-          <t>Cierre bajo por tipo</t>
+          <t>Cierre bajo — Bache en calle de asfalto</t>
         </is>
       </c>
       <c r="E14" s="2" t="inlineStr">
         <is>
-          <t>4.8% (21 casos)</t>
+          <t>10% (104 casos)</t>
         </is>
       </c>
       <c r="F14" s="2" t="inlineStr">
         <is>
-          <t>Tipo 'Reparación de rampa de accesibilidad': cierre 4.8% con 21 casos (umbral &lt;40% para volumen &gt;20).</t>
+          <t>Tipo 'Bache en calle de asfalto': cierre 10% con 104 casos en abril (umbral &lt;40% con volumen &gt;=20).</t>
         </is>
       </c>
     </row>
@@ -1100,17 +1094,17 @@
       </c>
       <c r="D15" s="2" t="inlineStr">
         <is>
-          <t>Muestra encuesta insuficiente</t>
+          <t>Cierre bajo — Reparación/construcción de cordón</t>
         </is>
       </c>
       <c r="E15" s="2" t="inlineStr">
         <is>
-          <t>Tasa 1.4%</t>
+          <t>3% (65 casos)</t>
         </is>
       </c>
       <c r="F15" s="2" t="inlineStr">
         <is>
-          <t>Tasa de respuesta encuesta 1.4% (umbral &lt;5%). Datos de satisfaccion no representativos.</t>
+          <t>Tipo 'Reparación/construcción de cordón': cierre 3% con 65 casos en abril (umbral &lt;40% con volumen &gt;=20).</t>
         </is>
       </c>
     </row>
@@ -1127,22 +1121,22 @@
       </c>
       <c r="C16" s="2" t="inlineStr">
         <is>
-          <t>Control de Actividades Comerciales</t>
+          <t>Calles y Veredas</t>
         </is>
       </c>
       <c r="D16" s="2" t="inlineStr">
         <is>
-          <t>SLA bajo</t>
+          <t>Cierre bajo — Bache en calle de hormigón</t>
         </is>
       </c>
       <c r="E16" s="2" t="inlineStr">
         <is>
-          <t>2.2%</t>
+          <t>3% (34 casos)</t>
         </is>
       </c>
       <c r="F16" s="2" t="inlineStr">
         <is>
-          <t>SLA 2.2% (umbral &lt;30%).</t>
+          <t>Tipo 'Bache en calle de hormigón': cierre 3% con 34 casos en abril (umbral &lt;40% con volumen &gt;=20).</t>
         </is>
       </c>
     </row>
@@ -1159,22 +1153,22 @@
       </c>
       <c r="C17" s="2" t="inlineStr">
         <is>
-          <t>Control de Actividades Comerciales</t>
+          <t>Calles y Veredas</t>
         </is>
       </c>
       <c r="D17" s="2" t="inlineStr">
         <is>
-          <t>Dias promedio alto</t>
+          <t>Cierre bajo — Reparación de rampa de accesibilidad</t>
         </is>
       </c>
       <c r="E17" s="2" t="inlineStr">
         <is>
-          <t>7.1 dias</t>
+          <t>5% (21 casos)</t>
         </is>
       </c>
       <c r="F17" s="2" t="inlineStr">
         <is>
-          <t>Promedio de resolucion 7.1 dias (umbral &gt;7).</t>
+          <t>Tipo 'Reparación de rampa de accesibilidad': cierre 5% con 21 casos en abril (umbral &lt;40% con volumen &gt;=20).</t>
         </is>
       </c>
     </row>
@@ -1196,17 +1190,17 @@
       </c>
       <c r="D18" s="2" t="inlineStr">
         <is>
-          <t>Tasa repeticion alta</t>
+          <t>Dias promedio alto</t>
         </is>
       </c>
       <c r="E18" s="2" t="inlineStr">
         <is>
-          <t>97.8%</t>
+          <t>7.1 dias</t>
         </is>
       </c>
       <c r="F18" s="2" t="inlineStr">
         <is>
-          <t>%Rep 97.8% (umbral &gt;50%).</t>
+          <t>Tiempo promedio de resolucion 7.1 dias en abril (umbral &gt;7).</t>
         </is>
       </c>
     </row>
@@ -1228,17 +1222,17 @@
       </c>
       <c r="D19" s="2" t="inlineStr">
         <is>
-          <t>SLA bajo</t>
+          <t>SLA critico (area)</t>
         </is>
       </c>
       <c r="E19" s="2" t="inlineStr">
         <is>
-          <t>12.5%</t>
+          <t>12%</t>
         </is>
       </c>
       <c r="F19" s="2" t="inlineStr">
         <is>
-          <t>SLA 12.5% (umbral &lt;30%).</t>
+          <t>SLA 12% en abril (umbral &lt;30%). Tercer o nuevo mes en zona critica.</t>
         </is>
       </c>
     </row>
@@ -1260,17 +1254,17 @@
       </c>
       <c r="D20" s="2" t="inlineStr">
         <is>
-          <t>Tasa repeticion alta</t>
+          <t>Cierre bajo — Cable cortado</t>
         </is>
       </c>
       <c r="E20" s="2" t="inlineStr">
         <is>
-          <t>86.6%</t>
+          <t>4% (55 casos)</t>
         </is>
       </c>
       <c r="F20" s="2" t="inlineStr">
         <is>
-          <t>%Rep 86.6% (umbral &gt;50%).</t>
+          <t>Tipo 'Cable cortado': cierre 4% con 55 casos en abril (umbral &lt;40% con volumen &gt;=20).</t>
         </is>
       </c>
     </row>
@@ -1292,17 +1286,17 @@
       </c>
       <c r="D21" s="2" t="inlineStr">
         <is>
-          <t>Cierre bajo por tipo</t>
+          <t>Cierre bajo — Poste en mal estado/sin mantenimiento</t>
         </is>
       </c>
       <c r="E21" s="2" t="inlineStr">
         <is>
-          <t>3.6% (55 casos)</t>
+          <t>23% (22 casos)</t>
         </is>
       </c>
       <c r="F21" s="2" t="inlineStr">
         <is>
-          <t>Tipo 'Cable cortado': cierre 3.6% con 55 casos (umbral &lt;40% para volumen &gt;20).</t>
+          <t>Tipo 'Poste en mal estado/sin mantenimiento': cierre 23% con 22 casos en abril (umbral &lt;40% con volumen &gt;=20).</t>
         </is>
       </c>
     </row>
@@ -1319,22 +1313,22 @@
       </c>
       <c r="C22" s="2" t="inlineStr">
         <is>
-          <t>Control del Espacio Publico</t>
+          <t>Residuos y Limpieza</t>
         </is>
       </c>
       <c r="D22" s="2" t="inlineStr">
         <is>
-          <t>Cierre bajo por tipo</t>
+          <t>SLA critico (area)</t>
         </is>
       </c>
       <c r="E22" s="2" t="inlineStr">
         <is>
-          <t>22.7% (22 casos)</t>
+          <t>28%</t>
         </is>
       </c>
       <c r="F22" s="2" t="inlineStr">
         <is>
-          <t>Tipo 'Poste en mal estado/sin mantenimiento': cierre 22.7% con 22 casos (umbral &lt;40% para volumen &gt;20).</t>
+          <t>SLA 28% en abril (umbral &lt;30%). Tercer o nuevo mes en zona critica.</t>
         </is>
       </c>
     </row>
@@ -1356,17 +1350,17 @@
       </c>
       <c r="D23" s="2" t="inlineStr">
         <is>
-          <t>SLA bajo</t>
+          <t>Cierre bajo — Falta de recolección de residuos reciclables (Prog</t>
         </is>
       </c>
       <c r="E23" s="2" t="inlineStr">
         <is>
-          <t>27.9%</t>
+          <t>27% (55 casos)</t>
         </is>
       </c>
       <c r="F23" s="2" t="inlineStr">
         <is>
-          <t>SLA 27.9% (umbral &lt;30%).</t>
+          <t>Tipo 'Falta de recolección de residuos reciclables (Programa Día Verde)': cierre 27% con 55 casos en abril (umbral &lt;40% con volumen &gt;=20).</t>
         </is>
       </c>
     </row>
@@ -1383,342 +1377,22 @@
       </c>
       <c r="C24" s="2" t="inlineStr">
         <is>
-          <t>Residuos y Limpieza</t>
+          <t>Transito</t>
         </is>
       </c>
       <c r="D24" s="2" t="inlineStr">
         <is>
-          <t>Tasa repeticion alta</t>
+          <t>Muestra encuesta insuficiente</t>
         </is>
       </c>
       <c r="E24" s="2" t="inlineStr">
         <is>
-          <t>92.7%</t>
+          <t>Tasa 4.4%</t>
         </is>
       </c>
       <c r="F24" s="2" t="inlineStr">
         <is>
-          <t>%Rep 92.7% (umbral &gt;50%).</t>
-        </is>
-      </c>
-    </row>
-    <row r="25">
-      <c r="A25" s="2" t="inlineStr">
-        <is>
-          <t>NUEVA</t>
-        </is>
-      </c>
-      <c r="B25" s="2" t="inlineStr">
-        <is>
-          <t>Abr-2026</t>
-        </is>
-      </c>
-      <c r="C25" s="2" t="inlineStr">
-        <is>
-          <t>Residuos y Limpieza</t>
-        </is>
-      </c>
-      <c r="D25" s="2" t="inlineStr">
-        <is>
-          <t>Cierre bajo por tipo</t>
-        </is>
-      </c>
-      <c r="E25" s="2" t="inlineStr">
-        <is>
-          <t>27.3% (55 casos)</t>
-        </is>
-      </c>
-      <c r="F25" s="2" t="inlineStr">
-        <is>
-          <t>Tipo 'Falta de recolección de residuos reciclables (Programa Día Verde)': cierre 27.3% con 55 casos (umbral &lt;40% para volumen &gt;20).</t>
-        </is>
-      </c>
-    </row>
-    <row r="26">
-      <c r="A26" s="2" t="inlineStr">
-        <is>
-          <t>NUEVA</t>
-        </is>
-      </c>
-      <c r="B26" s="2" t="inlineStr">
-        <is>
-          <t>Abr-2026</t>
-        </is>
-      </c>
-      <c r="C26" s="2" t="inlineStr">
-        <is>
-          <t>Transito</t>
-        </is>
-      </c>
-      <c r="D26" s="2" t="inlineStr">
-        <is>
-          <t>Muestra encuesta insuficiente</t>
-        </is>
-      </c>
-      <c r="E26" s="2" t="inlineStr">
-        <is>
-          <t>Tasa 4.4%</t>
-        </is>
-      </c>
-      <c r="F26" s="2" t="inlineStr">
-        <is>
           <t>Tasa de respuesta encuesta 4.4% (umbral &lt;5%). Datos de satisfaccion no representativos.</t>
-        </is>
-      </c>
-    </row>
-    <row r="27">
-      <c r="A27" s="2" t="inlineStr">
-        <is>
-          <t>NUEVA</t>
-        </is>
-      </c>
-      <c r="B27" s="2" t="inlineStr">
-        <is>
-          <t>Abr-2026</t>
-        </is>
-      </c>
-      <c r="C27" s="2" t="inlineStr">
-        <is>
-          <t>Global</t>
-        </is>
-      </c>
-      <c r="D27" s="2" t="inlineStr">
-        <is>
-          <t>Proceso batch detectado</t>
-        </is>
-      </c>
-      <c r="E27" s="2" t="inlineStr">
-        <is>
-          <t>13 cierres/min</t>
-        </is>
-      </c>
-      <c r="F27" s="2" t="inlineStr">
-        <is>
-          <t>Usuario lg@mantelectric.com: 13 cierres en 1 minuto (2026-04-13 08:30:00).</t>
-        </is>
-      </c>
-    </row>
-    <row r="28">
-      <c r="A28" s="2" t="inlineStr">
-        <is>
-          <t>NUEVA</t>
-        </is>
-      </c>
-      <c r="B28" s="2" t="inlineStr">
-        <is>
-          <t>Abr-2026</t>
-        </is>
-      </c>
-      <c r="C28" s="2" t="inlineStr">
-        <is>
-          <t>Global</t>
-        </is>
-      </c>
-      <c r="D28" s="2" t="inlineStr">
-        <is>
-          <t>Proceso batch detectado</t>
-        </is>
-      </c>
-      <c r="E28" s="2" t="inlineStr">
-        <is>
-          <t>13 cierres/min</t>
-        </is>
-      </c>
-      <c r="F28" s="2" t="inlineStr">
-        <is>
-          <t>Usuario lg@mantelectric.com: 13 cierres en 1 minuto (2026-04-13 08:31:00).</t>
-        </is>
-      </c>
-    </row>
-    <row r="29">
-      <c r="A29" s="2" t="inlineStr">
-        <is>
-          <t>NUEVA</t>
-        </is>
-      </c>
-      <c r="B29" s="2" t="inlineStr">
-        <is>
-          <t>Abr-2026</t>
-        </is>
-      </c>
-      <c r="C29" s="2" t="inlineStr">
-        <is>
-          <t>Global</t>
-        </is>
-      </c>
-      <c r="D29" s="2" t="inlineStr">
-        <is>
-          <t>Proceso batch detectado</t>
-        </is>
-      </c>
-      <c r="E29" s="2" t="inlineStr">
-        <is>
-          <t>15 cierres/min</t>
-        </is>
-      </c>
-      <c r="F29" s="2" t="inlineStr">
-        <is>
-          <t>Usuario lg@mantelectric.com: 15 cierres en 1 minuto (2026-04-14 08:32:00).</t>
-        </is>
-      </c>
-    </row>
-    <row r="30">
-      <c r="A30" s="2" t="inlineStr">
-        <is>
-          <t>NUEVA</t>
-        </is>
-      </c>
-      <c r="B30" s="2" t="inlineStr">
-        <is>
-          <t>Abr-2026</t>
-        </is>
-      </c>
-      <c r="C30" s="2" t="inlineStr">
-        <is>
-          <t>Global</t>
-        </is>
-      </c>
-      <c r="D30" s="2" t="inlineStr">
-        <is>
-          <t>Proceso batch detectado</t>
-        </is>
-      </c>
-      <c r="E30" s="2" t="inlineStr">
-        <is>
-          <t>14 cierres/min</t>
-        </is>
-      </c>
-      <c r="F30" s="2" t="inlineStr">
-        <is>
-          <t>Usuario lg@mantelectric.com: 14 cierres en 1 minuto (2026-04-14 08:40:00).</t>
-        </is>
-      </c>
-    </row>
-    <row r="31">
-      <c r="A31" s="2" t="inlineStr">
-        <is>
-          <t>NUEVA</t>
-        </is>
-      </c>
-      <c r="B31" s="2" t="inlineStr">
-        <is>
-          <t>Abr-2026</t>
-        </is>
-      </c>
-      <c r="C31" s="2" t="inlineStr">
-        <is>
-          <t>Global</t>
-        </is>
-      </c>
-      <c r="D31" s="2" t="inlineStr">
-        <is>
-          <t>Proceso batch detectado</t>
-        </is>
-      </c>
-      <c r="E31" s="2" t="inlineStr">
-        <is>
-          <t>12 cierres/min</t>
-        </is>
-      </c>
-      <c r="F31" s="2" t="inlineStr">
-        <is>
-          <t>Usuario lg@mantelectric.com: 12 cierres en 1 minuto (2026-04-17 08:34:00).</t>
-        </is>
-      </c>
-    </row>
-    <row r="32">
-      <c r="A32" s="2" t="inlineStr">
-        <is>
-          <t>NUEVA</t>
-        </is>
-      </c>
-      <c r="B32" s="2" t="inlineStr">
-        <is>
-          <t>Abr-2026</t>
-        </is>
-      </c>
-      <c r="C32" s="2" t="inlineStr">
-        <is>
-          <t>Global</t>
-        </is>
-      </c>
-      <c r="D32" s="2" t="inlineStr">
-        <is>
-          <t>Proceso batch detectado</t>
-        </is>
-      </c>
-      <c r="E32" s="2" t="inlineStr">
-        <is>
-          <t>17 cierres/min</t>
-        </is>
-      </c>
-      <c r="F32" s="2" t="inlineStr">
-        <is>
-          <t>Usuario lg@mantelectric.com: 17 cierres en 1 minuto (2026-04-22 09:02:00).</t>
-        </is>
-      </c>
-    </row>
-    <row r="33">
-      <c r="A33" s="2" t="inlineStr">
-        <is>
-          <t>NUEVA</t>
-        </is>
-      </c>
-      <c r="B33" s="2" t="inlineStr">
-        <is>
-          <t>Abr-2026</t>
-        </is>
-      </c>
-      <c r="C33" s="2" t="inlineStr">
-        <is>
-          <t>Global</t>
-        </is>
-      </c>
-      <c r="D33" s="2" t="inlineStr">
-        <is>
-          <t>Proceso batch detectado</t>
-        </is>
-      </c>
-      <c r="E33" s="2" t="inlineStr">
-        <is>
-          <t>13 cierres/min</t>
-        </is>
-      </c>
-      <c r="F33" s="2" t="inlineStr">
-        <is>
-          <t>Usuario lg@mantelectric.com: 13 cierres en 1 minuto (2026-04-24 08:31:00).</t>
-        </is>
-      </c>
-    </row>
-    <row r="34">
-      <c r="A34" s="2" t="inlineStr">
-        <is>
-          <t>NUEVA</t>
-        </is>
-      </c>
-      <c r="B34" s="2" t="inlineStr">
-        <is>
-          <t>Abr-2026</t>
-        </is>
-      </c>
-      <c r="C34" s="2" t="inlineStr">
-        <is>
-          <t>Global</t>
-        </is>
-      </c>
-      <c r="D34" s="2" t="inlineStr">
-        <is>
-          <t>Proceso batch detectado</t>
-        </is>
-      </c>
-      <c r="E34" s="2" t="inlineStr">
-        <is>
-          <t>12 cierres/min</t>
-        </is>
-      </c>
-      <c r="F34" s="2" t="inlineStr">
-        <is>
-          <t>Usuario lg@mantelectric.com: 12 cierres en 1 minuto (2026-04-29 08:33:00).</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Tablas_Stock vigente actualizado — Abr-2026
</commit_message>
<xml_diff>
--- a/Tablas/Tablas_Stock.xlsx
+++ b/Tablas/Tablas_Stock.xlsx
@@ -617,7 +617,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F21"/>
+  <dimension ref="A1:F18"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -779,12 +779,12 @@
       </c>
       <c r="E5" s="2" t="inlineStr">
         <is>
-          <t>12%</t>
+          <t>19%</t>
         </is>
       </c>
       <c r="F5" s="2" t="inlineStr">
         <is>
-          <t>SLA 29% — segundo mes consecutivo debajo de 30%. Poste mal estado: cierre 23% en 37 casos. En abril: SLA 12% — sigue por debajo del umbral.</t>
+          <t>SLA 29% en marzo — segundo mes consecutivo debajo de 30%. En abril: SLA 19% — tercer mes en zona critica.</t>
         </is>
       </c>
     </row>
@@ -843,12 +843,12 @@
       </c>
       <c r="E7" s="2" t="inlineStr">
         <is>
-          <t>cierre bajo</t>
+          <t>23% (22 casos)</t>
         </is>
       </c>
       <c r="F7" s="2" t="inlineStr">
         <is>
-          <t>37 casos con 23% cierre. Poste quebrado/cortado 20% en 5 casos. En abril: tipo sigue con cierre bajo — ver hallazgos por tipo de area.</t>
+          <t>37 casos en marzo con 23% cierre. En abril: 22 casos con 23% cierre — patron de cierre bajo sin mejora.</t>
         </is>
       </c>
     </row>
@@ -870,17 +870,17 @@
       </c>
       <c r="D8" s="2" t="inlineStr">
         <is>
-          <t>SLA critico (area)</t>
+          <t>Dias promedio alto</t>
         </is>
       </c>
       <c r="E8" s="2" t="inlineStr">
         <is>
-          <t>18%</t>
+          <t>8 dias</t>
         </is>
       </c>
       <c r="F8" s="2" t="inlineStr">
         <is>
-          <t>SLA 18% en abril (umbral &lt;30%).</t>
+          <t>Promedio de resolucion 8 dias en abril (umbral &gt;7).</t>
         </is>
       </c>
     </row>
@@ -902,17 +902,17 @@
       </c>
       <c r="D9" s="2" t="inlineStr">
         <is>
-          <t>Dias promedio alto</t>
+          <t>Cierre bajo — Árbol obstruye semáforo/luminaria/cartel/etc.</t>
         </is>
       </c>
       <c r="E9" s="2" t="inlineStr">
         <is>
-          <t>7.5 dias</t>
+          <t>20% (64 casos)</t>
         </is>
       </c>
       <c r="F9" s="2" t="inlineStr">
         <is>
-          <t>Tiempo promedio de resolucion 7.5 dias en abril (umbral &gt;7).</t>
+          <t>Tipo 'Árbol obstruye semáforo/luminaria/cartel/etc.': cierre 20% con 64 casos en abril (umbral &lt;40% con volumen &gt;=20).</t>
         </is>
       </c>
     </row>
@@ -929,22 +929,22 @@
       </c>
       <c r="C10" s="2" t="inlineStr">
         <is>
-          <t>Arbolado y Plazas</t>
+          <t>Calles y Veredas</t>
         </is>
       </c>
       <c r="D10" s="2" t="inlineStr">
         <is>
-          <t>Cierre bajo — Árbol obstruye semáforo/luminaria/cartel/etc.</t>
+          <t>Muestra encuesta insuficiente</t>
         </is>
       </c>
       <c r="E10" s="2" t="inlineStr">
         <is>
-          <t>20% (64 casos)</t>
+          <t>Tasa 1.4%</t>
         </is>
       </c>
       <c r="F10" s="2" t="inlineStr">
         <is>
-          <t>Tipo 'Árbol obstruye semáforo/luminaria/cartel/etc.': cierre 20% con 64 casos en abril (umbral &lt;40% con volumen &gt;=20).</t>
+          <t>Tasa de respuesta encuesta 1.4% (umbral &lt;5%). Datos de satisfaccion no representativos.</t>
         </is>
       </c>
     </row>
@@ -966,17 +966,17 @@
       </c>
       <c r="D11" s="2" t="inlineStr">
         <is>
-          <t>SLA critico (area)</t>
+          <t>Cierre bajo — Bache en calle de asfalto</t>
         </is>
       </c>
       <c r="E11" s="2" t="inlineStr">
         <is>
-          <t>12%</t>
+          <t>10% (104 casos)</t>
         </is>
       </c>
       <c r="F11" s="2" t="inlineStr">
         <is>
-          <t>SLA 12% en abril (umbral &lt;30%).</t>
+          <t>Tipo 'Bache en calle de asfalto': cierre 10% con 104 casos en abril (umbral &lt;40% con volumen &gt;=20).</t>
         </is>
       </c>
     </row>
@@ -998,17 +998,17 @@
       </c>
       <c r="D12" s="2" t="inlineStr">
         <is>
-          <t>Muestra encuesta insuficiente</t>
+          <t>Cierre bajo — Reparación/construcción de cordón</t>
         </is>
       </c>
       <c r="E12" s="2" t="inlineStr">
         <is>
-          <t>Tasa 1.4%</t>
+          <t>3% (65 casos)</t>
         </is>
       </c>
       <c r="F12" s="2" t="inlineStr">
         <is>
-          <t>Tasa de respuesta encuesta 1.4% (umbral &lt;5%). Datos de satisfaccion no representativos.</t>
+          <t>Tipo 'Reparación/construcción de cordón': cierre 3% con 65 casos en abril (umbral &lt;40% con volumen &gt;=20).</t>
         </is>
       </c>
     </row>
@@ -1030,17 +1030,17 @@
       </c>
       <c r="D13" s="2" t="inlineStr">
         <is>
-          <t>Cierre bajo — Bache en calle de asfalto</t>
+          <t>Cierre bajo — Bache en calle de hormigón</t>
         </is>
       </c>
       <c r="E13" s="2" t="inlineStr">
         <is>
-          <t>10% (104 casos)</t>
+          <t>3% (34 casos)</t>
         </is>
       </c>
       <c r="F13" s="2" t="inlineStr">
         <is>
-          <t>Tipo 'Bache en calle de asfalto': cierre 10% con 104 casos en abril (umbral &lt;40% con volumen &gt;=20).</t>
+          <t>Tipo 'Bache en calle de hormigón': cierre 3% con 34 casos en abril (umbral &lt;40% con volumen &gt;=20).</t>
         </is>
       </c>
     </row>
@@ -1062,17 +1062,17 @@
       </c>
       <c r="D14" s="2" t="inlineStr">
         <is>
-          <t>Cierre bajo — Reparación/construcción de cordón</t>
+          <t>Cierre bajo — Reparación de rampa de accesibilidad</t>
         </is>
       </c>
       <c r="E14" s="2" t="inlineStr">
         <is>
-          <t>3% (65 casos)</t>
+          <t>5% (21 casos)</t>
         </is>
       </c>
       <c r="F14" s="2" t="inlineStr">
         <is>
-          <t>Tipo 'Reparación/construcción de cordón': cierre 3% con 65 casos en abril (umbral &lt;40% con volumen &gt;=20).</t>
+          <t>Tipo 'Reparación de rampa de accesibilidad': cierre 5% con 21 casos en abril (umbral &lt;40% con volumen &gt;=20).</t>
         </is>
       </c>
     </row>
@@ -1089,22 +1089,22 @@
       </c>
       <c r="C15" s="2" t="inlineStr">
         <is>
-          <t>Calles y Veredas</t>
+          <t>Control de Actividades Comerciales</t>
         </is>
       </c>
       <c r="D15" s="2" t="inlineStr">
         <is>
-          <t>Cierre bajo — Bache en calle de hormigón</t>
+          <t>Dias promedio alto</t>
         </is>
       </c>
       <c r="E15" s="2" t="inlineStr">
         <is>
-          <t>3% (34 casos)</t>
+          <t>7.1 dias</t>
         </is>
       </c>
       <c r="F15" s="2" t="inlineStr">
         <is>
-          <t>Tipo 'Bache en calle de hormigón': cierre 3% con 34 casos en abril (umbral &lt;40% con volumen &gt;=20).</t>
+          <t>Tiempo promedio de resolucion 7.1 dias en abril (umbral &gt;7).</t>
         </is>
       </c>
     </row>
@@ -1121,22 +1121,22 @@
       </c>
       <c r="C16" s="2" t="inlineStr">
         <is>
-          <t>Calles y Veredas</t>
+          <t>Control del Espacio Publico</t>
         </is>
       </c>
       <c r="D16" s="2" t="inlineStr">
         <is>
-          <t>Cierre bajo — Reparación de rampa de accesibilidad</t>
+          <t>Cierre bajo — Cable cortado</t>
         </is>
       </c>
       <c r="E16" s="2" t="inlineStr">
         <is>
-          <t>5% (21 casos)</t>
+          <t>4% (55 casos)</t>
         </is>
       </c>
       <c r="F16" s="2" t="inlineStr">
         <is>
-          <t>Tipo 'Reparación de rampa de accesibilidad': cierre 5% con 21 casos en abril (umbral &lt;40% con volumen &gt;=20).</t>
+          <t>Tipo 'Cable cortado': cierre 4% con 55 casos en abril (umbral &lt;40% con volumen &gt;=20).</t>
         </is>
       </c>
     </row>
@@ -1153,22 +1153,22 @@
       </c>
       <c r="C17" s="2" t="inlineStr">
         <is>
-          <t>Control de Actividades Comerciales</t>
+          <t>Residuos y Limpieza</t>
         </is>
       </c>
       <c r="D17" s="2" t="inlineStr">
         <is>
-          <t>Dias promedio alto</t>
+          <t>Cierre bajo — Falta de recolección de residuos reciclables (Prog</t>
         </is>
       </c>
       <c r="E17" s="2" t="inlineStr">
         <is>
-          <t>7.1 dias</t>
+          <t>27% (55 casos)</t>
         </is>
       </c>
       <c r="F17" s="2" t="inlineStr">
         <is>
-          <t>Tiempo promedio de resolucion 7.1 dias en abril (umbral &gt;7).</t>
+          <t>Tipo 'Falta de recolección de residuos reciclables (Programa Día Verde)': cierre 27% con 55 casos en abril (umbral &lt;40% con volumen &gt;=20).</t>
         </is>
       </c>
     </row>
@@ -1185,116 +1185,20 @@
       </c>
       <c r="C18" s="2" t="inlineStr">
         <is>
-          <t>Control del Espacio Publico</t>
+          <t>Transito</t>
         </is>
       </c>
       <c r="D18" s="2" t="inlineStr">
         <is>
-          <t>Cierre bajo — Cable cortado</t>
+          <t>Muestra encuesta insuficiente</t>
         </is>
       </c>
       <c r="E18" s="2" t="inlineStr">
         <is>
-          <t>4% (55 casos)</t>
+          <t>Tasa 4.4%</t>
         </is>
       </c>
       <c r="F18" s="2" t="inlineStr">
-        <is>
-          <t>Tipo 'Cable cortado': cierre 4% con 55 casos en abril (umbral &lt;40% con volumen &gt;=20).</t>
-        </is>
-      </c>
-    </row>
-    <row r="19">
-      <c r="A19" s="2" t="inlineStr">
-        <is>
-          <t>NUEVA</t>
-        </is>
-      </c>
-      <c r="B19" s="2" t="inlineStr">
-        <is>
-          <t>Abr-2026</t>
-        </is>
-      </c>
-      <c r="C19" s="2" t="inlineStr">
-        <is>
-          <t>Residuos y Limpieza</t>
-        </is>
-      </c>
-      <c r="D19" s="2" t="inlineStr">
-        <is>
-          <t>SLA critico (area)</t>
-        </is>
-      </c>
-      <c r="E19" s="2" t="inlineStr">
-        <is>
-          <t>28%</t>
-        </is>
-      </c>
-      <c r="F19" s="2" t="inlineStr">
-        <is>
-          <t>SLA 28% en abril (umbral &lt;30%).</t>
-        </is>
-      </c>
-    </row>
-    <row r="20">
-      <c r="A20" s="2" t="inlineStr">
-        <is>
-          <t>NUEVA</t>
-        </is>
-      </c>
-      <c r="B20" s="2" t="inlineStr">
-        <is>
-          <t>Abr-2026</t>
-        </is>
-      </c>
-      <c r="C20" s="2" t="inlineStr">
-        <is>
-          <t>Residuos y Limpieza</t>
-        </is>
-      </c>
-      <c r="D20" s="2" t="inlineStr">
-        <is>
-          <t>Cierre bajo — Falta de recolección de residuos reciclables (Prog</t>
-        </is>
-      </c>
-      <c r="E20" s="2" t="inlineStr">
-        <is>
-          <t>27% (55 casos)</t>
-        </is>
-      </c>
-      <c r="F20" s="2" t="inlineStr">
-        <is>
-          <t>Tipo 'Falta de recolección de residuos reciclables (Programa Día Verde)': cierre 27% con 55 casos en abril (umbral &lt;40% con volumen &gt;=20).</t>
-        </is>
-      </c>
-    </row>
-    <row r="21">
-      <c r="A21" s="2" t="inlineStr">
-        <is>
-          <t>NUEVA</t>
-        </is>
-      </c>
-      <c r="B21" s="2" t="inlineStr">
-        <is>
-          <t>Abr-2026</t>
-        </is>
-      </c>
-      <c r="C21" s="2" t="inlineStr">
-        <is>
-          <t>Transito</t>
-        </is>
-      </c>
-      <c r="D21" s="2" t="inlineStr">
-        <is>
-          <t>Muestra encuesta insuficiente</t>
-        </is>
-      </c>
-      <c r="E21" s="2" t="inlineStr">
-        <is>
-          <t>Tasa 4.4%</t>
-        </is>
-      </c>
-      <c r="F21" s="2" t="inlineStr">
         <is>
           <t>Tasa de respuesta encuesta 4.4% (umbral &lt;5%). Datos de satisfaccion no representativos.</t>
         </is>

</xml_diff>

<commit_message>
fix: Tablas_Stock vigente con RESUELTAS incluidas
</commit_message>
<xml_diff>
--- a/Tablas/Tablas_Stock.xlsx
+++ b/Tablas/Tablas_Stock.xlsx
@@ -32,7 +32,7 @@
       <color rgb="00FFFFFF"/>
     </font>
   </fonts>
-  <fills count="4">
+  <fills count="5">
     <fill>
       <patternFill/>
     </fill>
@@ -42,6 +42,11 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor rgb="001F4E79"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00E2EFDA"/>
       </patternFill>
     </fill>
     <fill>
@@ -62,13 +67,16 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="4">
+  <cellXfs count="5">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="3" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="4" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment wrapText="1"/>
     </xf>
   </cellXfs>
@@ -475,7 +483,7 @@
       </c>
       <c r="B3" s="2" t="inlineStr">
         <is>
-          <t>76% (+8pp vs marzo 68%). Alumbrado 84% y Residuos 85% traccionan. Calles y Veredas cae a 7% — el mas critico del mes. Arbolado persiste en 35%.</t>
+          <t>76% (+8pp vs marzo 68%). Alumbrado 84% y Residuos 85% traccionan. Calles y Veredas cae a 7% ? el mas critico del mes. Arbolado persiste en 35%.</t>
         </is>
       </c>
     </row>
@@ -565,7 +573,7 @@
       </c>
       <c r="B4" s="2" t="inlineStr">
         <is>
-          <t>Cierre colapsa a 7% — el mas bajo del area en el periodo analizado. Volumen crece 28% con 282 casos y muestra de encuesta insuficiente (1.4%).</t>
+          <t>Cierre colapsa a 7% ? el mas bajo del area en el periodo analizado. Volumen crece 28% con 282 casos y muestra de encuesta insuficiente (1.4%).</t>
         </is>
       </c>
     </row>
@@ -628,7 +636,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F14"/>
+  <dimension ref="A1:F19"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -674,7 +682,7 @@
     <row r="2">
       <c r="A2" s="3" t="inlineStr">
         <is>
-          <t>PERSISTE</t>
+          <t>RESUELTA</t>
         </is>
       </c>
       <c r="B2" s="3" t="inlineStr">
@@ -684,61 +692,61 @@
       </c>
       <c r="C2" s="3" t="inlineStr">
         <is>
-          <t>ARBOLADO Y PLAZAS</t>
+          <t>TRANSITO</t>
         </is>
       </c>
       <c r="D2" s="3" t="inlineStr">
         <is>
-          <t>Cierre bajo</t>
+          <t>Cancelado excesivo en cerrados</t>
         </is>
       </c>
       <c r="E2" s="3" t="inlineStr">
         <is>
-          <t>35%</t>
+          <t>4.7%</t>
         </is>
       </c>
       <c r="F2" s="3" t="inlineStr">
         <is>
-          <t>Cierre 29% en marzo → 35% en abril. Cuarto mes debajo de 50%. Arbol obstruye semaforo/luminaria concentra el deficit con 64 casos y 20% cierre. 11.5% de los cerrados son Cancelados.</t>
+          <t>Cancelado en cerrados baja de 39% (marzo) a 4.7% (abril). Mejora significativa. Vehiculos Abandonados deja de concentrar cancelaciones masivas.</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="3" t="inlineStr">
         <is>
-          <t>PERSISTE</t>
+          <t>RESUELTA</t>
         </is>
       </c>
       <c r="B3" s="3" t="inlineStr">
         <is>
-          <t>febrero de 2026</t>
+          <t>marzo de 2026</t>
         </is>
       </c>
       <c r="C3" s="3" t="inlineStr">
         <is>
-          <t>ARBOLADO Y PLAZAS</t>
+          <t>TRANSITO</t>
         </is>
       </c>
       <c r="D3" s="3" t="inlineStr">
         <is>
-          <t>Cancelado alto en cerrados</t>
+          <t>Reparacion semaforo cierre critico</t>
         </is>
       </c>
       <c r="E3" s="3" t="inlineStr">
         <is>
-          <t>11.5%</t>
+          <t>63%</t>
         </is>
       </c>
       <c r="F3" s="3" t="inlineStr">
         <is>
-          <t>Cancelado sube de 41% (marzo) a 11.5% sobre total de cerrados en abril. El cierre parcial se sostiene en parte por cancelaciones.</t>
+          <t>Cierre de Reparacion de semaforo sube de 26% (marzo, 57 casos) a 63% (abril, 117 casos). Sale de zona critica con mayor volumen.</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" s="3" t="inlineStr">
         <is>
-          <t>PERSISTE</t>
+          <t>RESUELTA</t>
         </is>
       </c>
       <c r="B4" s="3" t="inlineStr">
@@ -748,29 +756,29 @@
       </c>
       <c r="C4" s="3" t="inlineStr">
         <is>
-          <t>ARBOLADO Y PLAZAS</t>
+          <t>RESIDUOS Y LIMPIEZA</t>
         </is>
       </c>
       <c r="D4" s="3" t="inlineStr">
         <is>
-          <t>Arbol obstruye cierre critico</t>
+          <t>Falta barrido variacion anomala</t>
         </is>
       </c>
       <c r="E4" s="3" t="inlineStr">
         <is>
-          <t>20% (64 casos)</t>
+          <t>77%</t>
         </is>
       </c>
       <c r="F4" s="3" t="inlineStr">
         <is>
-          <t>Tipo dominante del area: 64 casos con 20% cierre en abril. En marzo: 110 casos con 14% cierre. Mejora en volumen pero el cierre sigue critico.</t>
+          <t>Cierre de Falta barrido sube de 43% (marzo) a 77% (abril). El volumen sube a 820 casos pero el cierre se normaliza. Alerta de variacion resuelta.</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" s="3" t="inlineStr">
         <is>
-          <t>PERSISTE</t>
+          <t>RESUELTA</t>
         </is>
       </c>
       <c r="B5" s="3" t="inlineStr">
@@ -780,308 +788,468 @@
       </c>
       <c r="C5" s="3" t="inlineStr">
         <is>
-          <t>CALLES Y VEREDAS</t>
+          <t>RESIDUOS Y LIMPIEZA</t>
         </is>
       </c>
       <c r="D5" s="3" t="inlineStr">
         <is>
-          <t>Cierre colapsado</t>
+          <t>Falta recoleccion organicos cierre critico</t>
         </is>
       </c>
       <c r="E5" s="3" t="inlineStr">
         <is>
-          <t>7%</t>
+          <t>?</t>
         </is>
       </c>
       <c r="F5" s="3" t="inlineStr">
         <is>
-          <t>Cierre cae de 32% (marzo) a 7% (abril). Bache asfalto: 104 casos, 10% cierre. Cordon: 65 casos, 3% cierre. Hormigon: 34 casos, 3% cierre. Rampa accesibilidad: 21 casos, 5% cierre.</t>
+          <t>Sin registros de Falta recoleccion de residuos organicos/humedos en abril. En marzo: 259 casos con 11% cierre. Tipo desaparece del volumen del mes.</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" s="3" t="inlineStr">
         <is>
+          <t>RESUELTA</t>
+        </is>
+      </c>
+      <c r="B6" s="3" t="inlineStr">
+        <is>
+          <t>marzo de 2026</t>
+        </is>
+      </c>
+      <c r="C6" s="3" t="inlineStr">
+        <is>
+          <t>RESIDUOS Y LIMPIEZA</t>
+        </is>
+      </c>
+      <c r="D6" s="3" t="inlineStr">
+        <is>
+          <t>Retiro restos poda arbolado variacion anomala</t>
+        </is>
+      </c>
+      <c r="E6" s="3" t="inlineStr">
+        <is>
+          <t>?</t>
+        </is>
+      </c>
+      <c r="F6" s="3" t="inlineStr">
+        <is>
+          <t>Sin anomalia en abril. En marzo: 155 casos con +104% de variacion y 36% cierre. El tipo regresa a comportamiento normal en volumen y cierre.</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="4" t="inlineStr">
+        <is>
           <t>PERSISTE</t>
         </is>
       </c>
-      <c r="B6" s="3" t="inlineStr">
+      <c r="B7" s="4" t="inlineStr">
         <is>
           <t>febrero de 2026</t>
         </is>
       </c>
-      <c r="C6" s="3" t="inlineStr">
+      <c r="C7" s="4" t="inlineStr">
+        <is>
+          <t>ARBOLADO Y PLAZAS</t>
+        </is>
+      </c>
+      <c r="D7" s="4" t="inlineStr">
+        <is>
+          <t>Cierre bajo</t>
+        </is>
+      </c>
+      <c r="E7" s="4" t="inlineStr">
+        <is>
+          <t>35%</t>
+        </is>
+      </c>
+      <c r="F7" s="4" t="inlineStr">
+        <is>
+          <t>Cierre 29% en marzo ? 35% en abril. Cuarto mes debajo de 50%. Arbol obstruye semaforo/luminaria concentra el deficit con 64 casos y 20% cierre. 11.5% de los cerrados son Cancelados.</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="4" t="inlineStr">
+        <is>
+          <t>PERSISTE</t>
+        </is>
+      </c>
+      <c r="B8" s="4" t="inlineStr">
+        <is>
+          <t>febrero de 2026</t>
+        </is>
+      </c>
+      <c r="C8" s="4" t="inlineStr">
+        <is>
+          <t>ARBOLADO Y PLAZAS</t>
+        </is>
+      </c>
+      <c r="D8" s="4" t="inlineStr">
+        <is>
+          <t>Cancelado alto en cerrados</t>
+        </is>
+      </c>
+      <c r="E8" s="4" t="inlineStr">
+        <is>
+          <t>11.5%</t>
+        </is>
+      </c>
+      <c r="F8" s="4" t="inlineStr">
+        <is>
+          <t>Cancelado sobre cerrados sube de 41% (marzo) a 11.5% en abril. El cierre parcial se sostiene en parte por cancelaciones.</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="4" t="inlineStr">
+        <is>
+          <t>PERSISTE</t>
+        </is>
+      </c>
+      <c r="B9" s="4" t="inlineStr">
+        <is>
+          <t>marzo de 2026</t>
+        </is>
+      </c>
+      <c r="C9" s="4" t="inlineStr">
+        <is>
+          <t>ARBOLADO Y PLAZAS</t>
+        </is>
+      </c>
+      <c r="D9" s="4" t="inlineStr">
+        <is>
+          <t>Arbol obstruye cierre critico</t>
+        </is>
+      </c>
+      <c r="E9" s="4" t="inlineStr">
+        <is>
+          <t>20% (64 casos)</t>
+        </is>
+      </c>
+      <c r="F9" s="4" t="inlineStr">
+        <is>
+          <t>Tipo dominante del area: 64 casos con 20% cierre en abril. En marzo: 110 casos con 14% cierre. Mejora en volumen pero el cierre sigue critico.</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="4" t="inlineStr">
+        <is>
+          <t>PERSISTE</t>
+        </is>
+      </c>
+      <c r="B10" s="4" t="inlineStr">
+        <is>
+          <t>marzo de 2026</t>
+        </is>
+      </c>
+      <c r="C10" s="4" t="inlineStr">
+        <is>
+          <t>CALLES Y VEREDAS</t>
+        </is>
+      </c>
+      <c r="D10" s="4" t="inlineStr">
+        <is>
+          <t>Cierre colapsado</t>
+        </is>
+      </c>
+      <c r="E10" s="4" t="inlineStr">
+        <is>
+          <t>7%</t>
+        </is>
+      </c>
+      <c r="F10" s="4" t="inlineStr">
+        <is>
+          <t>Cierre cae de 32% (marzo) a 7% (abril). Bache asfalto: 104 casos, 10% cierre. Cordon: 65 casos, 3% cierre. Hormigon: 34 casos, 3% cierre. Rampa accesibilidad: 21 casos, 5% cierre.</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="4" t="inlineStr">
+        <is>
+          <t>PERSISTE</t>
+        </is>
+      </c>
+      <c r="B11" s="4" t="inlineStr">
+        <is>
+          <t>febrero de 2026</t>
+        </is>
+      </c>
+      <c r="C11" s="4" t="inlineStr">
         <is>
           <t>CONTROL DE ACTIVIDADES COMERCIALES</t>
         </is>
       </c>
-      <c r="D6" s="3" t="inlineStr">
+      <c r="D11" s="4" t="inlineStr">
         <is>
           <t>SLA critico</t>
         </is>
       </c>
-      <c r="E6" s="3" t="inlineStr">
+      <c r="E11" s="4" t="inlineStr">
         <is>
           <t>4%</t>
         </is>
       </c>
-      <c r="F6" s="3" t="inlineStr">
-        <is>
-          <t>SLA 16% en marzo → 4% en abril. Tercer mes consecutivo debajo de 30%. Dias promedio de resolucion: 9. El indicador empeora pese al volumen estable (89 casos).</t>
-        </is>
-      </c>
-    </row>
-    <row r="7">
-      <c r="A7" s="3" t="inlineStr">
+      <c r="F11" s="4" t="inlineStr">
+        <is>
+          <t>SLA 16% en marzo ? 4% en abril. Tercer mes consecutivo debajo de 30%. Dias promedio de resolucion: 9. El indicador empeora pese al volumen estable (89 casos).</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="4" t="inlineStr">
         <is>
           <t>PERSISTE</t>
         </is>
       </c>
-      <c r="B7" s="3" t="inlineStr">
+      <c r="B12" s="4" t="inlineStr">
         <is>
           <t>febrero de 2026</t>
         </is>
       </c>
-      <c r="C7" s="3" t="inlineStr">
+      <c r="C12" s="4" t="inlineStr">
         <is>
           <t>CONTROL DEL ESPACIO PUBLICO</t>
         </is>
       </c>
-      <c r="D7" s="3" t="inlineStr">
+      <c r="D12" s="4" t="inlineStr">
         <is>
           <t>SLA bajo</t>
         </is>
       </c>
-      <c r="E7" s="3" t="inlineStr">
+      <c r="E12" s="4" t="inlineStr">
         <is>
           <t>19%</t>
         </is>
       </c>
-      <c r="F7" s="3" t="inlineStr">
-        <is>
-          <t>SLA 29% en marzo → 19% en abril. Tercer mes debajo de 30%. Poste en mal estado (22 casos, 23% cierre) y Cable cortado (55 casos, 4% cierre) son los tipos de mayor impacto.</t>
-        </is>
-      </c>
-    </row>
-    <row r="8">
-      <c r="A8" s="3" t="inlineStr">
+      <c r="F12" s="4" t="inlineStr">
+        <is>
+          <t>SLA 29% en marzo ? 19% en abril. Tercer mes debajo de 30%. Poste en mal estado (22 casos, 23% cierre) y Cable cortado (55 casos, 4% cierre) son los tipos de mayor impacto.</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="4" t="inlineStr">
         <is>
           <t>NUEVA</t>
         </is>
       </c>
-      <c r="B8" s="3" t="inlineStr">
+      <c r="B13" s="4" t="inlineStr">
         <is>
           <t>abril de 2026</t>
         </is>
       </c>
-      <c r="C8" s="3" t="inlineStr">
+      <c r="C13" s="4" t="inlineStr">
         <is>
           <t>CONTROL DEL ESPACIO PUBLICO</t>
         </is>
       </c>
-      <c r="D8" s="3" t="inlineStr">
+      <c r="D13" s="4" t="inlineStr">
         <is>
           <t>Cable cortado cierre critico</t>
         </is>
       </c>
-      <c r="E8" s="3" t="inlineStr">
+      <c r="E13" s="4" t="inlineStr">
         <is>
           <t>4% (55 casos)</t>
         </is>
       </c>
-      <c r="F8" s="3" t="inlineStr">
+      <c r="F13" s="4" t="inlineStr">
         <is>
           <t>55 casos con solo 2 cerrados en abril (4% cierre). En marzo: 29 casos con 28% cierre. Sube el volumen y cae el cierre. Incidentes con outliers &gt;30 dias: #12329843, #12330370.</t>
         </is>
       </c>
     </row>
-    <row r="9">
-      <c r="A9" s="3" t="inlineStr">
+    <row r="14">
+      <c r="A14" s="4" t="inlineStr">
         <is>
           <t>NUEVA</t>
         </is>
       </c>
-      <c r="B9" s="3" t="inlineStr">
+      <c r="B14" s="4" t="inlineStr">
         <is>
           <t>abril de 2026</t>
         </is>
       </c>
-      <c r="C9" s="3" t="inlineStr">
+      <c r="C14" s="4" t="inlineStr">
         <is>
           <t>RESIDUOS Y LIMPIEZA</t>
         </is>
       </c>
-      <c r="D9" s="3" t="inlineStr">
+      <c r="D14" s="4" t="inlineStr">
         <is>
           <t>Residuos reciclables cierre bajo</t>
         </is>
       </c>
-      <c r="E9" s="3" t="inlineStr">
+      <c r="E14" s="4" t="inlineStr">
         <is>
           <t>27% (55 casos)</t>
         </is>
       </c>
-      <c r="F9" s="3" t="inlineStr">
+      <c r="F14" s="4" t="inlineStr">
         <is>
           <t>55 casos de Residuos reciclables Dia Verde con 27% cierre en abril. Tipo con baja resolucion sostenida en el area de mayor volumen del municipio.</t>
         </is>
       </c>
     </row>
-    <row r="10">
-      <c r="A10" s="3" t="inlineStr">
+    <row r="15">
+      <c r="A15" s="4" t="inlineStr">
         <is>
           <t>NUEVA</t>
         </is>
       </c>
-      <c r="B10" s="3" t="inlineStr">
+      <c r="B15" s="4" t="inlineStr">
         <is>
           <t>abril de 2026</t>
         </is>
       </c>
-      <c r="C10" s="3" t="inlineStr">
+      <c r="C15" s="4" t="inlineStr">
         <is>
           <t>CALLES Y VEREDAS</t>
         </is>
       </c>
-      <c r="D10" s="3" t="inlineStr">
+      <c r="D15" s="4" t="inlineStr">
         <is>
           <t>Muestra encuesta insuficiente</t>
         </is>
       </c>
-      <c r="E10" s="3" t="inlineStr">
+      <c r="E15" s="4" t="inlineStr">
         <is>
           <t>1.4%</t>
         </is>
       </c>
-      <c r="F10" s="3" t="inlineStr">
+      <c r="F15" s="4" t="inlineStr">
         <is>
           <t>Solo 4 respuestas de encuesta sobre 282 incidentes (1.4%). Los datos de satisfaccion (25%) no son representativos. Segundo mes con muestra reducida en el area.</t>
         </is>
       </c>
     </row>
-    <row r="11">
-      <c r="A11" s="3" t="inlineStr">
+    <row r="16">
+      <c r="A16" s="4" t="inlineStr">
         <is>
           <t>NUEVA</t>
         </is>
       </c>
-      <c r="B11" s="3" t="inlineStr">
+      <c r="B16" s="4" t="inlineStr">
         <is>
           <t>abril de 2026</t>
         </is>
       </c>
-      <c r="C11" s="3" t="inlineStr">
+      <c r="C16" s="4" t="inlineStr">
         <is>
           <t>TRANSITO</t>
         </is>
       </c>
-      <c r="D11" s="3" t="inlineStr">
+      <c r="D16" s="4" t="inlineStr">
         <is>
           <t>Muestra encuesta insuficiente</t>
         </is>
       </c>
-      <c r="E11" s="3" t="inlineStr">
+      <c r="E16" s="4" t="inlineStr">
         <is>
           <t>4.4%</t>
         </is>
       </c>
-      <c r="F11" s="3" t="inlineStr">
+      <c r="F16" s="4" t="inlineStr">
         <is>
           <t>24 respuestas sobre 551 incidentes (4.4%). Satisfaccion 79% no es representativa. Persistente problema de envio de encuestas en Vehiculos Abandonados.</t>
         </is>
       </c>
     </row>
-    <row r="12">
-      <c r="A12" s="3" t="inlineStr">
+    <row r="17">
+      <c r="A17" s="4" t="inlineStr">
         <is>
           <t>NUEVA</t>
         </is>
       </c>
-      <c r="B12" s="3" t="inlineStr">
+      <c r="B17" s="4" t="inlineStr">
         <is>
           <t>abril de 2026</t>
         </is>
       </c>
-      <c r="C12" s="3" t="inlineStr">
+      <c r="C17" s="4" t="inlineStr">
         <is>
           <t>CONTROL DE ACTIVIDADES COMERCIALES</t>
         </is>
       </c>
-      <c r="D12" s="3" t="inlineStr">
+      <c r="D17" s="4" t="inlineStr">
         <is>
           <t>Satisfaccion baja</t>
         </is>
       </c>
-      <c r="E12" s="3" t="inlineStr">
+      <c r="E17" s="4" t="inlineStr">
         <is>
           <t>18%</t>
         </is>
       </c>
-      <c r="F12" s="3" t="inlineStr">
-        <is>
-          <t>Satisfaccion 18% con cierre 58%. Brecha de 40pp entre cierre y satisfaccion sugiere que los cierres no se perciben como resolucion efectiva. 12.4% tasa de respuesta.</t>
-        </is>
-      </c>
-    </row>
-    <row r="13">
-      <c r="A13" s="3" t="inlineStr">
+      <c r="F17" s="4" t="inlineStr">
+        <is>
+          <t>Satisfaccion 18% con cierre 58%. Brecha de 40pp entre cierre y satisfaccion: los cierres no se perciben como resolucion efectiva. 12.4% tasa de respuesta.</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="4" t="inlineStr">
         <is>
           <t>NUEVA</t>
         </is>
       </c>
-      <c r="B13" s="3" t="inlineStr">
+      <c r="B18" s="4" t="inlineStr">
         <is>
           <t>abril de 2026</t>
         </is>
       </c>
-      <c r="C13" s="3" t="inlineStr">
+      <c r="C18" s="4" t="inlineStr">
         <is>
           <t>CONTROL DE ACTIVIDADES COMERCIALES</t>
         </is>
       </c>
-      <c r="D13" s="3" t="inlineStr">
+      <c r="D18" s="4" t="inlineStr">
         <is>
           <t>Dias promedio alto</t>
         </is>
       </c>
-      <c r="E13" s="3" t="inlineStr">
+      <c r="E18" s="4" t="inlineStr">
         <is>
           <t>9 dias</t>
         </is>
       </c>
-      <c r="F13" s="3" t="inlineStr">
+      <c r="F18" s="4" t="inlineStr">
         <is>
           <t>Dias promedio de resolucion: 9 dias en abril (era 6 en marzo). El incremento se da con volumen estable (-1%), lo que indica enlentecimiento operativo.</t>
         </is>
       </c>
     </row>
-    <row r="14">
-      <c r="A14" s="3" t="inlineStr">
+    <row r="19">
+      <c r="A19" s="4" t="inlineStr">
         <is>
           <t>NUEVA</t>
         </is>
       </c>
-      <c r="B14" s="3" t="inlineStr">
+      <c r="B19" s="4" t="inlineStr">
         <is>
           <t>abril de 2026</t>
         </is>
       </c>
-      <c r="C14" s="3" t="inlineStr">
+      <c r="C19" s="4" t="inlineStr">
         <is>
           <t>ARBOLADO Y PLAZAS</t>
         </is>
       </c>
-      <c r="D14" s="3" t="inlineStr">
+      <c r="D19" s="4" t="inlineStr">
         <is>
           <t>Dias promedio alto</t>
         </is>
       </c>
-      <c r="E14" s="3" t="inlineStr">
+      <c r="E19" s="4" t="inlineStr">
         <is>
           <t>8 dias</t>
         </is>
       </c>
-      <c r="F14" s="3" t="inlineStr">
+      <c r="F19" s="4" t="inlineStr">
         <is>
           <t>Dias promedio de resolucion: 8 dias en abril. Coincide con bajo cierre (35%) y alta concentracion de casos abiertos de Arbol obstruye sin resolver.</t>
         </is>

</xml_diff>

<commit_message>
fix: corregir valores Stock abril 2026 contra tablero PBI
</commit_message>
<xml_diff>
--- a/Tablas/Tablas_Stock.xlsx
+++ b/Tablas/Tablas_Stock.xlsx
@@ -28,8 +28,10 @@
       <scheme val="minor"/>
     </font>
     <font>
+      <name val="Calibri"/>
       <b val="1"/>
       <color rgb="00FFFFFF"/>
+      <sz val="11"/>
     </font>
   </fonts>
   <fills count="5">
@@ -41,7 +43,7 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="001F4E79"/>
+        <fgColor rgb="005B2C8D"/>
       </patternFill>
     </fill>
     <fill>
@@ -69,15 +71,17 @@
   </cellStyleXfs>
   <cellXfs count="5">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment wrapText="1"/>
+      <alignment vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="3" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment wrapText="1"/>
+      <alignment vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="4" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment wrapText="1"/>
+      <alignment vertical="top" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -448,10 +452,10 @@
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="18" customWidth="1" min="1" max="1"/>
-    <col width="90" customWidth="1" min="2" max="2"/>
+    <col width="95" customWidth="1" min="2" max="2"/>
   </cols>
   <sheetData>
-    <row r="1">
+    <row r="1" ht="20" customHeight="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
           <t>KPI</t>
@@ -463,44 +467,44 @@
         </is>
       </c>
     </row>
-    <row r="2">
-      <c r="A2" s="2" t="inlineStr">
+    <row r="2" ht="45" customHeight="1">
+      <c r="A2" t="inlineStr">
         <is>
           <t>CANTIDAD</t>
         </is>
       </c>
       <c r="B2" s="2" t="inlineStr">
         <is>
-          <t>5.085 incidentes en abril (+9% vs marzo 4.675). Residuos lidera con 3.046 casos. Alumbrado +19%, Transito +21%, Calles +28%. Arbolado baja -30%.</t>
-        </is>
-      </c>
-    </row>
-    <row r="3">
-      <c r="A3" s="2" t="inlineStr">
+          <t>5.077 incidentes en abril (+8% vs marzo 4.675). Residuos lidera con 3.039 casos. Alumbrado +19%, Transito +21%, Calles +28%. Arbolado baja -33%.</t>
+        </is>
+      </c>
+    </row>
+    <row r="3" ht="45" customHeight="1">
+      <c r="A3" t="inlineStr">
         <is>
           <t>CIERRE</t>
         </is>
       </c>
       <c r="B3" s="2" t="inlineStr">
         <is>
-          <t>76% (+8pp vs marzo 68%). Alumbrado 84% y Residuos 85% traccionan. Calles y Veredas cae a 7% ? el mas critico del mes. Arbolado persiste en 35%.</t>
-        </is>
-      </c>
-    </row>
-    <row r="4">
-      <c r="A4" s="2" t="inlineStr">
+          <t>74% (+6pp vs marzo 68%). Alumbrado 84% y Residuos 82% traccionan. Calles y Veredas cae a 7% — el mas critico del mes. Arbolado persiste en 35%.</t>
+        </is>
+      </c>
+    </row>
+    <row r="4" ht="45" customHeight="1">
+      <c r="A4" t="inlineStr">
         <is>
           <t>SLA</t>
         </is>
       </c>
       <c r="B4" s="2" t="inlineStr">
         <is>
-          <t>40% (-10pp vs marzo 50%). Alumbrado lidera con 69%. Ctrl Comerciales 4% y Ctrl Espacio Publico 19% concentran el deficit. Transito sube a 63%.</t>
-        </is>
-      </c>
-    </row>
-    <row r="5">
-      <c r="A5" s="2" t="inlineStr">
+          <t>41% (-9pp vs marzo 50%). Alumbrado lidera con 69%. Ctrl Comerciales 4% y Ctrl Espacio Publico 19% concentran el deficit. Transito sube a 63%.</t>
+        </is>
+      </c>
+    </row>
+    <row r="5" ht="45" customHeight="1">
+      <c r="A5" t="inlineStr">
         <is>
           <t>SATISFACCION</t>
         </is>
@@ -525,11 +529,11 @@
   <dimension ref="A1:B8"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="38" customWidth="1" min="1" max="1"/>
-    <col width="90" customWidth="1" min="2" max="2"/>
+    <col width="35" customWidth="1" min="1" max="1"/>
+    <col width="95" customWidth="1" min="2" max="2"/>
   </cols>
   <sheetData>
-    <row r="1">
+    <row r="1" ht="20" customHeight="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
           <t>Area</t>
@@ -541,8 +545,8 @@
         </is>
       </c>
     </row>
-    <row r="2">
-      <c r="A2" s="2" t="inlineStr">
+    <row r="2" ht="40" customHeight="1">
+      <c r="A2" t="inlineStr">
         <is>
           <t>ALUMBRADO PUBLICO</t>
         </is>
@@ -553,8 +557,8 @@
         </is>
       </c>
     </row>
-    <row r="3">
-      <c r="A3" s="2" t="inlineStr">
+    <row r="3" ht="40" customHeight="1">
+      <c r="A3" t="inlineStr">
         <is>
           <t>ARBOLADO Y PLAZAS</t>
         </is>
@@ -565,20 +569,20 @@
         </is>
       </c>
     </row>
-    <row r="4">
-      <c r="A4" s="2" t="inlineStr">
+    <row r="4" ht="40" customHeight="1">
+      <c r="A4" t="inlineStr">
         <is>
           <t>CALLES Y VEREDAS</t>
         </is>
       </c>
       <c r="B4" s="2" t="inlineStr">
         <is>
-          <t>Cierre colapsa a 7% ? el mas bajo del area en el periodo analizado. Volumen crece 28% con 282 casos y muestra de encuesta insuficiente (1.4%).</t>
-        </is>
-      </c>
-    </row>
-    <row r="5">
-      <c r="A5" s="2" t="inlineStr">
+          <t>Cierre colapsa a 7%, el mas bajo del area en el periodo analizado. Volumen crece 28% con 282 casos y muestra de encuesta insuficiente (1.4%).</t>
+        </is>
+      </c>
+    </row>
+    <row r="5" ht="40" customHeight="1">
+      <c r="A5" t="inlineStr">
         <is>
           <t>CONTROL DE ACTIVIDADES COMERCIALES</t>
         </is>
@@ -589,8 +593,8 @@
         </is>
       </c>
     </row>
-    <row r="6">
-      <c r="A6" s="2" t="inlineStr">
+    <row r="6" ht="40" customHeight="1">
+      <c r="A6" t="inlineStr">
         <is>
           <t>CONTROL DEL ESPACIO PUBLICO</t>
         </is>
@@ -601,20 +605,20 @@
         </is>
       </c>
     </row>
-    <row r="7">
-      <c r="A7" s="2" t="inlineStr">
+    <row r="7" ht="40" customHeight="1">
+      <c r="A7" t="inlineStr">
         <is>
           <t>RESIDUOS Y LIMPIEZA</t>
         </is>
       </c>
       <c r="B7" s="2" t="inlineStr">
         <is>
-          <t>Cierre 85%, el mejor del municipio. Falta barrido resuelve (77%). Residuos reciclables Dia Verde con 27% cierre en 55 casos.</t>
-        </is>
-      </c>
-    </row>
-    <row r="8">
-      <c r="A8" s="2" t="inlineStr">
+          <t>Cierre 82% — mejor del municipio. Falta barrido resuelve (77%). Residuos reciclables Dia Verde con 27% cierre en 55 casos es la nueva alerta del area.</t>
+        </is>
+      </c>
+    </row>
+    <row r="8" ht="40" customHeight="1">
+      <c r="A8" t="inlineStr">
         <is>
           <t>TRANSITO</t>
         </is>
@@ -641,13 +645,13 @@
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
     <col width="18" customWidth="1" min="2" max="2"/>
-    <col width="38" customWidth="1" min="3" max="3"/>
+    <col width="30" customWidth="1" min="3" max="3"/>
     <col width="35" customWidth="1" min="4" max="4"/>
-    <col width="16" customWidth="1" min="5" max="5"/>
+    <col width="18" customWidth="1" min="5" max="5"/>
     <col width="80" customWidth="1" min="6" max="6"/>
   </cols>
   <sheetData>
-    <row r="1">
+    <row r="1" ht="20" customHeight="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
           <t>Estado</t>
@@ -679,7 +683,7 @@
         </is>
       </c>
     </row>
-    <row r="2">
+    <row r="2" ht="55" customHeight="1">
       <c r="A2" s="3" t="inlineStr">
         <is>
           <t>RESUELTA</t>
@@ -707,11 +711,11 @@
       </c>
       <c r="F2" s="3" t="inlineStr">
         <is>
-          <t>Cancelado en cerrados baja de 39% (marzo) a 4.7% (abril). Mejora significativa. Vehiculos Abandonados deja de concentrar cancelaciones masivas.</t>
-        </is>
-      </c>
-    </row>
-    <row r="3">
+          <t>En febrero el 39% de los cerrados de Transito eran cancelados — anomalia persistente. En abril el porcentaje cae a 4.7%, dentro del rango operativo normal.</t>
+        </is>
+      </c>
+    </row>
+    <row r="3" ht="55" customHeight="1">
       <c r="A3" s="3" t="inlineStr">
         <is>
           <t>RESUELTA</t>
@@ -739,11 +743,11 @@
       </c>
       <c r="F3" s="3" t="inlineStr">
         <is>
-          <t>Cierre de Reparacion de semaforo sube de 26% (marzo, 57 casos) a 63% (abril, 117 casos). Sale de zona critica con mayor volumen.</t>
-        </is>
-      </c>
-    </row>
-    <row r="4">
+          <t>Reparacion de semaforo tenia 26% de cierre en marzo (117 casos pendientes). En abril sube a 63% — mejora de 37pp, sale de zona critica.</t>
+        </is>
+      </c>
+    </row>
+    <row r="4" ht="55" customHeight="1">
       <c r="A4" s="3" t="inlineStr">
         <is>
           <t>RESUELTA</t>
@@ -771,11 +775,11 @@
       </c>
       <c r="F4" s="3" t="inlineStr">
         <is>
-          <t>Cierre de Falta barrido sube de 43% (marzo) a 77% (abril). El volumen sube a 820 casos pero el cierre se normaliza. Alerta de variacion resuelta.</t>
-        </is>
-      </c>
-    </row>
-    <row r="5">
+          <t>En marzo Falta barrido registro variacion anomala de volumen. En abril el cierre sube de 43% a 77% y el volumen se normaliza — alerta superada.</t>
+        </is>
+      </c>
+    </row>
+    <row r="5" ht="55" customHeight="1">
       <c r="A5" s="3" t="inlineStr">
         <is>
           <t>RESUELTA</t>
@@ -798,16 +802,16 @@
       </c>
       <c r="E5" s="3" t="inlineStr">
         <is>
-          <t>?</t>
+          <t>sin registros</t>
         </is>
       </c>
       <c r="F5" s="3" t="inlineStr">
         <is>
-          <t>Sin registros de Falta recoleccion de residuos organicos/humedos en abril. En marzo: 259 casos con 11% cierre. Tipo desaparece del volumen del mes.</t>
-        </is>
-      </c>
-    </row>
-    <row r="6">
+          <t>Falta de recoleccion de residuos organicos concentraba casos con bajo cierre en marzo. En abril no se registran casos del tipo — alerta resuelta.</t>
+        </is>
+      </c>
+    </row>
+    <row r="6" ht="55" customHeight="1">
       <c r="A6" s="3" t="inlineStr">
         <is>
           <t>RESUELTA</t>
@@ -830,16 +834,16 @@
       </c>
       <c r="E6" s="3" t="inlineStr">
         <is>
-          <t>?</t>
+          <t>sin registros</t>
         </is>
       </c>
       <c r="F6" s="3" t="inlineStr">
         <is>
-          <t>Sin anomalia en abril. En marzo: 155 casos con +104% de variacion y 36% cierre. El tipo regresa a comportamiento normal en volumen y cierre.</t>
-        </is>
-      </c>
-    </row>
-    <row r="7">
+          <t>Retiro de restos de poda/arbolado presento variacion anomala en marzo. En abril no se registran casos del tipo — alerta resuelta.</t>
+        </is>
+      </c>
+    </row>
+    <row r="7" ht="55" customHeight="1">
       <c r="A7" s="4" t="inlineStr">
         <is>
           <t>PERSISTE</t>
@@ -867,11 +871,11 @@
       </c>
       <c r="F7" s="4" t="inlineStr">
         <is>
-          <t>Cierre 29% en marzo ? 35% en abril. Cuarto mes debajo de 50%. Arbol obstruye semaforo/luminaria concentra el deficit con 64 casos y 20% cierre. 11.5% de los cerrados son Cancelados.</t>
-        </is>
-      </c>
-    </row>
-    <row r="8">
+          <t>Arbolado y Plazas mantiene 35% de cierre en abril — tercer mes consecutivo en zona critica. Arbol obstruye semaforo/luminaria (64 casos, 20% cierre) y alta proporcion de cancelados (11.5%) concentran el problema.</t>
+        </is>
+      </c>
+    </row>
+    <row r="8" ht="55" customHeight="1">
       <c r="A8" s="4" t="inlineStr">
         <is>
           <t>PERSISTE</t>
@@ -899,11 +903,11 @@
       </c>
       <c r="F8" s="4" t="inlineStr">
         <is>
-          <t>Cancelado sobre cerrados sube de 41% (marzo) a 11.5% en abril. El cierre parcial se sostiene en parte por cancelaciones.</t>
-        </is>
-      </c>
-    </row>
-    <row r="9">
+          <t>El 11.5% de los cierres del area son cancelaciones, por encima del 10% de referencia. Persiste desde febrero sin mejora.</t>
+        </is>
+      </c>
+    </row>
+    <row r="9" ht="55" customHeight="1">
       <c r="A9" s="4" t="inlineStr">
         <is>
           <t>PERSISTE</t>
@@ -931,11 +935,11 @@
       </c>
       <c r="F9" s="4" t="inlineStr">
         <is>
-          <t>Tipo dominante del area: 64 casos con 20% cierre en abril. En marzo: 110 casos con 14% cierre. Mejora en volumen pero el cierre sigue critico.</t>
-        </is>
-      </c>
-    </row>
-    <row r="10">
+          <t>Arbol obstruye semaforo/luminaria/cartel mantiene 20% de cierre con 64 casos en abril. Sin variacion respecto a marzo — el tipo concentra el deficit de cierre del area.</t>
+        </is>
+      </c>
+    </row>
+    <row r="10" ht="55" customHeight="1">
       <c r="A10" s="4" t="inlineStr">
         <is>
           <t>PERSISTE</t>
@@ -963,11 +967,11 @@
       </c>
       <c r="F10" s="4" t="inlineStr">
         <is>
-          <t>Cierre cae de 32% (marzo) a 7% (abril). Bache asfalto: 104 casos, 10% cierre. Cordon: 65 casos, 3% cierre. Hormigon: 34 casos, 3% cierre. Rampa accesibilidad: 21 casos, 5% cierre.</t>
-        </is>
-      </c>
-    </row>
-    <row r="11">
+          <t>Calles y Veredas cae de 32% en marzo a 7% en abril — 282 casos con Bache asfalto (104, 10% cierre), Cordon (65, 3% cierre) y Bache hormigon (34, 3% cierre) sin resolucion.</t>
+        </is>
+      </c>
+    </row>
+    <row r="11" ht="55" customHeight="1">
       <c r="A11" s="4" t="inlineStr">
         <is>
           <t>PERSISTE</t>
@@ -995,11 +999,11 @@
       </c>
       <c r="F11" s="4" t="inlineStr">
         <is>
-          <t>SLA 16% en marzo ? 4% en abril. Tercer mes consecutivo debajo de 30%. Dias promedio de resolucion: 9. El indicador empeora pese al volumen estable (89 casos).</t>
-        </is>
-      </c>
-    </row>
-    <row r="12">
+          <t>SLA de 4% por tercer mes consecutivo — el indicador mas bajo del municipio. Los tiempos de resolucion estan fuera del parametro en la totalidad del area.</t>
+        </is>
+      </c>
+    </row>
+    <row r="12" ht="55" customHeight="1">
       <c r="A12" s="4" t="inlineStr">
         <is>
           <t>PERSISTE</t>
@@ -1027,11 +1031,11 @@
       </c>
       <c r="F12" s="4" t="inlineStr">
         <is>
-          <t>SLA 29% en marzo ? 19% en abril. Tercer mes debajo de 30%. Poste en mal estado (22 casos, 23% cierre) y Cable cortado (55 casos, 4% cierre) son los tipos de mayor impacto.</t>
-        </is>
-      </c>
-    </row>
-    <row r="13">
+          <t>SLA del area persiste en 19% en abril, sin variacion respecto a febrero-marzo. Cable cortado (55 casos, 4% cierre) y Poste en mal estado (22 casos, 23% cierre) contribuyen al indicador bajo.</t>
+        </is>
+      </c>
+    </row>
+    <row r="13" ht="55" customHeight="1">
       <c r="A13" s="4" t="inlineStr">
         <is>
           <t>NUEVA</t>
@@ -1059,11 +1063,11 @@
       </c>
       <c r="F13" s="4" t="inlineStr">
         <is>
-          <t>55 casos con solo 2 cerrados en abril (4% cierre). En marzo: 29 casos con 28% cierre. Sube el volumen y cae el cierre. Incidentes con outliers &gt;30 dias: #12329843, #12330370.</t>
-        </is>
-      </c>
-    </row>
-    <row r="14">
+          <t>Cable cortado suma 55 casos en abril con 4% de cierre — acumulacion de casos sin resolucion. El tipo no contaba con alerta previa; en abril supera el umbral de volumen con cierre critico.</t>
+        </is>
+      </c>
+    </row>
+    <row r="14" ht="55" customHeight="1">
       <c r="A14" s="4" t="inlineStr">
         <is>
           <t>NUEVA</t>
@@ -1091,11 +1095,11 @@
       </c>
       <c r="F14" s="4" t="inlineStr">
         <is>
-          <t>55 casos de Residuos reciclables Dia Verde con 27% cierre en abril. Tipo con baja resolucion sostenida en el area de mayor volumen del municipio.</t>
-        </is>
-      </c>
-    </row>
-    <row r="15">
+          <t>Residuos reciclables Dia Verde registra 27% de cierre con 55 casos en abril. Primer mes con volumen significativo y cierre por debajo de 40%.</t>
+        </is>
+      </c>
+    </row>
+    <row r="15" ht="55" customHeight="1">
       <c r="A15" s="4" t="inlineStr">
         <is>
           <t>NUEVA</t>
@@ -1123,11 +1127,11 @@
       </c>
       <c r="F15" s="4" t="inlineStr">
         <is>
-          <t>Solo 4 respuestas de encuesta sobre 282 incidentes (1.4%). Los datos de satisfaccion (25%) no son representativos. Segundo mes con muestra reducida en el area.</t>
-        </is>
-      </c>
-    </row>
-    <row r="16">
+          <t>Tasa de respuesta de encuesta en Calles y Veredas es 1.4% (4 respuestas sobre 282 incidentes) — muestra no representativa. No es posible evaluar satisfaccion del area este mes.</t>
+        </is>
+      </c>
+    </row>
+    <row r="16" ht="55" customHeight="1">
       <c r="A16" s="4" t="inlineStr">
         <is>
           <t>NUEVA</t>
@@ -1155,11 +1159,11 @@
       </c>
       <c r="F16" s="4" t="inlineStr">
         <is>
-          <t>24 respuestas sobre 551 incidentes (4.4%). Satisfaccion 79% no es representativa. Persistente problema de envio de encuestas en Vehiculos Abandonados.</t>
-        </is>
-      </c>
-    </row>
-    <row r="17">
+          <t>Tasa de respuesta de encuesta en Transito es 4.4% (24 respuestas sobre 551 incidentes) — por debajo del minimo para representatividad. Satisfaccion reportada (79%) no es estadisticamente confiable.</t>
+        </is>
+      </c>
+    </row>
+    <row r="17" ht="55" customHeight="1">
       <c r="A17" s="4" t="inlineStr">
         <is>
           <t>NUEVA</t>
@@ -1187,11 +1191,11 @@
       </c>
       <c r="F17" s="4" t="inlineStr">
         <is>
-          <t>Satisfaccion 18% con cierre 58%. Brecha de 40pp entre cierre y satisfaccion: los cierres no se perciben como resolucion efectiva. 12.4% tasa de respuesta.</t>
-        </is>
-      </c>
-    </row>
-    <row r="18">
+          <t>Satisfaccion de 18% en Control de Actividades Comerciales con 12.4% de tasa de respuesta — el peor indicador del municipio. Ruidos molestos y falta de notificacion de resolucion concentran los comentarios negativos.</t>
+        </is>
+      </c>
+    </row>
+    <row r="18" ht="55" customHeight="1">
       <c r="A18" s="4" t="inlineStr">
         <is>
           <t>NUEVA</t>
@@ -1219,11 +1223,11 @@
       </c>
       <c r="F18" s="4" t="inlineStr">
         <is>
-          <t>Dias promedio de resolucion: 9 dias en abril (era 6 en marzo). El incremento se da con volumen estable (-1%), lo que indica enlentecimiento operativo.</t>
-        </is>
-      </c>
-    </row>
-    <row r="19">
+          <t>Dias promedio de resolucion sube a 9 dias en abril — el mayor registrado para el area. Combinado con SLA 4% y satisfaccion 18%, configura la situacion mas critica del municipio.</t>
+        </is>
+      </c>
+    </row>
+    <row r="19" ht="55" customHeight="1">
       <c r="A19" s="4" t="inlineStr">
         <is>
           <t>NUEVA</t>
@@ -1251,7 +1255,7 @@
       </c>
       <c r="F19" s="4" t="inlineStr">
         <is>
-          <t>Dias promedio de resolucion: 8 dias en abril. Coincide con bajo cierre (35%) y alta concentracion de casos abiertos de Arbol obstruye sin resolver.</t>
+          <t>Dias promedio de resolucion de 8 dias en Arbolado y Plazas — por encima del umbral. Se suma al cierre bajo (35%) y al alto porcentaje de cancelados (11.5%).</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Tablas_Stock vigente v2 - Abr-2026
</commit_message>
<xml_diff>
--- a/Tablas/Tablas_Stock.xlsx
+++ b/Tablas/Tablas_Stock.xlsx
@@ -623,7 +623,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F22"/>
+  <dimension ref="A1:F19"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -977,12 +977,12 @@
       </c>
       <c r="E11" s="3" t="inlineStr">
         <is>
-          <t>2%</t>
+          <t>4%</t>
         </is>
       </c>
       <c r="F11" s="3" t="inlineStr">
         <is>
-          <t>SLA 2% en abril, persiste debajo del umbral 30%.</t>
+          <t>SLA 4% en abril (tablero), persiste debajo del umbral 30%.</t>
         </is>
       </c>
     </row>
@@ -1009,12 +1009,12 @@
       </c>
       <c r="E12" s="3" t="inlineStr">
         <is>
-          <t>12%</t>
+          <t>19%</t>
         </is>
       </c>
       <c r="F12" s="3" t="inlineStr">
         <is>
-          <t>SLA 12% en abril, persiste debajo del umbral 30%.</t>
+          <t>SLA 19% en abril (tablero), persiste debajo del umbral 30%.</t>
         </is>
       </c>
     </row>
@@ -1036,17 +1036,17 @@
       </c>
       <c r="D13" s="3" t="inlineStr">
         <is>
-          <t>SLA critico (area)</t>
+          <t>Dias promedio alto</t>
         </is>
       </c>
       <c r="E13" s="3" t="inlineStr">
         <is>
-          <t>18%</t>
+          <t>8 dias</t>
         </is>
       </c>
       <c r="F13" s="3" t="inlineStr">
         <is>
-          <t>SLA del area 18% en abril (umbral &lt;30%). Tiempos de resolucion fuera de parametro.</t>
+          <t>Tiempo promedio de resolucion 8 dias en abril (tablero, umbral &gt;7).</t>
         </is>
       </c>
     </row>
@@ -1063,22 +1063,22 @@
       </c>
       <c r="C14" s="3" t="inlineStr">
         <is>
-          <t>Arbolado y Plazas</t>
+          <t>Calles y Veredas</t>
         </is>
       </c>
       <c r="D14" s="3" t="inlineStr">
         <is>
-          <t>Dias promedio alto</t>
+          <t>Muestra encuesta insuficiente</t>
         </is>
       </c>
       <c r="E14" s="3" t="inlineStr">
         <is>
-          <t>7.5 dias</t>
+          <t>Tasa 1.4%</t>
         </is>
       </c>
       <c r="F14" s="3" t="inlineStr">
         <is>
-          <t>Tiempo promedio de resolucion 7.5 dias en abril (umbral &gt;7).</t>
+          <t>Tasa de respuesta encuesta 1.4% (4 respuestas sobre 282 incidentes). Datos de satisfaccion no representativos.</t>
         </is>
       </c>
     </row>
@@ -1095,7 +1095,7 @@
       </c>
       <c r="C15" s="3" t="inlineStr">
         <is>
-          <t>Calles y Veredas</t>
+          <t>Control de Actividades Comerciales</t>
         </is>
       </c>
       <c r="D15" s="3" t="inlineStr">
@@ -1105,12 +1105,12 @@
       </c>
       <c r="E15" s="3" t="inlineStr">
         <is>
-          <t>12%</t>
+          <t>4%</t>
         </is>
       </c>
       <c r="F15" s="3" t="inlineStr">
         <is>
-          <t>SLA del area 12% en abril (umbral &lt;30%). Tiempos de resolucion fuera de parametro.</t>
+          <t>SLA del area 4% en abril (tablero, umbral &lt;30%). Tiempos de resolucion fuera de parametro.</t>
         </is>
       </c>
     </row>
@@ -1127,22 +1127,22 @@
       </c>
       <c r="C16" s="3" t="inlineStr">
         <is>
-          <t>Calles y Veredas</t>
+          <t>Control de Actividades Comerciales</t>
         </is>
       </c>
       <c r="D16" s="3" t="inlineStr">
         <is>
-          <t>Muestra encuesta insuficiente</t>
+          <t>Dias promedio alto</t>
         </is>
       </c>
       <c r="E16" s="3" t="inlineStr">
         <is>
-          <t>Tasa 1.4%</t>
+          <t>9 dias</t>
         </is>
       </c>
       <c r="F16" s="3" t="inlineStr">
         <is>
-          <t>Tasa de respuesta encuesta 1.4% (4 respuestas sobre 282 incidentes). Datos de satisfaccion no representativos.</t>
+          <t>Tiempo promedio de resolucion 9 dias en abril (tablero, umbral &gt;7).</t>
         </is>
       </c>
     </row>
@@ -1159,22 +1159,22 @@
       </c>
       <c r="C17" s="3" t="inlineStr">
         <is>
-          <t>Control de Actividades Comerciales</t>
+          <t>Control del Espacio Publico</t>
         </is>
       </c>
       <c r="D17" s="3" t="inlineStr">
         <is>
-          <t>SLA critico (area)</t>
+          <t>Cierre bajo - Cable cortado</t>
         </is>
       </c>
       <c r="E17" s="3" t="inlineStr">
         <is>
-          <t>2%</t>
+          <t>4% (55 casos)</t>
         </is>
       </c>
       <c r="F17" s="3" t="inlineStr">
         <is>
-          <t>SLA del area 2% en abril (umbral &lt;30%). Tiempos de resolucion fuera de parametro.</t>
+          <t>Tipo 'Cable cortado': 55 casos en abril con 4% de cierre (umbral &lt;40% con volumen &gt;=20).</t>
         </is>
       </c>
     </row>
@@ -1191,22 +1191,22 @@
       </c>
       <c r="C18" s="3" t="inlineStr">
         <is>
-          <t>Control de Actividades Comerciales</t>
+          <t>Residuos y Limpieza</t>
         </is>
       </c>
       <c r="D18" s="3" t="inlineStr">
         <is>
-          <t>Dias promedio alto</t>
+          <t>Cierre bajo - Falta de recolección de residuos reciclables (Pr</t>
         </is>
       </c>
       <c r="E18" s="3" t="inlineStr">
         <is>
-          <t>7.1 dias</t>
+          <t>27% (55 casos)</t>
         </is>
       </c>
       <c r="F18" s="3" t="inlineStr">
         <is>
-          <t>Tiempo promedio de resolucion 7.1 dias en abril (umbral &gt;7).</t>
+          <t>Tipo 'Falta de recolección de residuos reciclables (Programa Día Verde)': 55 casos en abril con 27% de cierre (umbral &lt;40% con volumen &gt;=20).</t>
         </is>
       </c>
     </row>
@@ -1223,116 +1223,20 @@
       </c>
       <c r="C19" s="3" t="inlineStr">
         <is>
-          <t>Control del Espacio Publico</t>
+          <t>Transito</t>
         </is>
       </c>
       <c r="D19" s="3" t="inlineStr">
         <is>
-          <t>Cierre bajo - Cable cortado</t>
+          <t>Muestra encuesta insuficiente</t>
         </is>
       </c>
       <c r="E19" s="3" t="inlineStr">
         <is>
-          <t>4% (55 casos)</t>
+          <t>Tasa 4.4%</t>
         </is>
       </c>
       <c r="F19" s="3" t="inlineStr">
-        <is>
-          <t>Tipo 'Cable cortado': 55 casos en abril con 4% de cierre (umbral &lt;40% con volumen &gt;=20).</t>
-        </is>
-      </c>
-    </row>
-    <row r="20">
-      <c r="A20" s="3" t="inlineStr">
-        <is>
-          <t>NUEVA</t>
-        </is>
-      </c>
-      <c r="B20" s="3" t="inlineStr">
-        <is>
-          <t>Abr-2026</t>
-        </is>
-      </c>
-      <c r="C20" s="3" t="inlineStr">
-        <is>
-          <t>Residuos y Limpieza</t>
-        </is>
-      </c>
-      <c r="D20" s="3" t="inlineStr">
-        <is>
-          <t>SLA critico (area)</t>
-        </is>
-      </c>
-      <c r="E20" s="3" t="inlineStr">
-        <is>
-          <t>28%</t>
-        </is>
-      </c>
-      <c r="F20" s="3" t="inlineStr">
-        <is>
-          <t>SLA del area 28% en abril (umbral &lt;30%). Tiempos de resolucion fuera de parametro.</t>
-        </is>
-      </c>
-    </row>
-    <row r="21">
-      <c r="A21" s="3" t="inlineStr">
-        <is>
-          <t>NUEVA</t>
-        </is>
-      </c>
-      <c r="B21" s="3" t="inlineStr">
-        <is>
-          <t>Abr-2026</t>
-        </is>
-      </c>
-      <c r="C21" s="3" t="inlineStr">
-        <is>
-          <t>Residuos y Limpieza</t>
-        </is>
-      </c>
-      <c r="D21" s="3" t="inlineStr">
-        <is>
-          <t>Cierre bajo - Falta de recolección de residuos reciclables (Pr</t>
-        </is>
-      </c>
-      <c r="E21" s="3" t="inlineStr">
-        <is>
-          <t>27% (55 casos)</t>
-        </is>
-      </c>
-      <c r="F21" s="3" t="inlineStr">
-        <is>
-          <t>Tipo 'Falta de recolección de residuos reciclables (Programa Día Verde)': 55 casos en abril con 27% de cierre (umbral &lt;40% con volumen &gt;=20).</t>
-        </is>
-      </c>
-    </row>
-    <row r="22">
-      <c r="A22" s="3" t="inlineStr">
-        <is>
-          <t>NUEVA</t>
-        </is>
-      </c>
-      <c r="B22" s="3" t="inlineStr">
-        <is>
-          <t>Abr-2026</t>
-        </is>
-      </c>
-      <c r="C22" s="3" t="inlineStr">
-        <is>
-          <t>Transito</t>
-        </is>
-      </c>
-      <c r="D22" s="3" t="inlineStr">
-        <is>
-          <t>Muestra encuesta insuficiente</t>
-        </is>
-      </c>
-      <c r="E22" s="3" t="inlineStr">
-        <is>
-          <t>Tasa 4.4%</t>
-        </is>
-      </c>
-      <c r="F22" s="3" t="inlineStr">
         <is>
           <t>Tasa de respuesta encuesta 4.4% (24 respuestas sobre 550 incidentes). Datos de satisfaccion no representativos.</t>
         </is>

</xml_diff>

<commit_message>
Tablas_Stock vigente v2 - May-2026
</commit_message>
<xml_diff>
--- a/Tablas/Tablas_Stock.xlsx
+++ b/Tablas/Tablas_Stock.xlsx
@@ -458,7 +458,7 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>Total 5077 incidentes en abril (+9% vs marzo). RESIDUOS Y LIMPIEZA concentra 60% del volumen (3046 casos, +9%). TRANSITO sube +21% por reparacion de semaforo (+115%).</t>
+          <t>Total 4556 incidentes en mayo (-10% vs abril, 5072). RESIDUOS Y LIMPIEZA concentra 59% del volumen (2691 casos, -11%). Bajas generalizadas: ALUMBRADO -18%, ARBOLADO -21%.</t>
         </is>
       </c>
     </row>
@@ -470,7 +470,7 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>Cierre global 74% (+6.5pp vs marzo). CALLES Y VEREDAS colapsa a 7% (-25pp). ARBOLADO persiste en 35%. ALUMBRADO 84% y RESIDUOS 85% lideran. Cancelado total 1%.</t>
+          <t>Cierre global 74% (+0.0pp vs abril). CALLES Y VEREDAS en 15%, ARBOLADO 50%. ALUMBRADO 85% y RESIDUOS 81% lideran. Cancelado sobre cerrados alto en ARBOLADO 32%, TRANSITO 24%, CALLES 24%.</t>
         </is>
       </c>
     </row>
@@ -482,7 +482,7 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>SLA global 41% (-9.6pp). CTRL ACT COMERCIALES persiste en 4% (peor del municipio). CTRL ESPACIO PUBLICO 19%. RESIDUOS baja a 33%. ALUMBRADO lidera con 69%. Promedio 4.3 dias.</t>
+          <t>SLA global 45% (+4.0pp vs abril). CTRL ACT COMERCIALES 23% y CTRL ESPACIO PUBLICO 26% bajos. ALUMBRADO lidera con 71%, TRANSITO 58%. Promedio 3 dias.</t>
         </is>
       </c>
     </row>
@@ -494,7 +494,7 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>Satisfaccion global 63% (+1.6pp). ALUMBRADO 79% y TRANSITO 79%. Criticos: CTRL ACT COMERCIALES 18%, CALLES Y VEREDAS 25% (muestra insuficiente), ARBOLADO 25%. Tasa respuesta 17%.</t>
+          <t>Satisfaccion global 64% (+1.0pp vs abril). ARBOLADO 75% lidera. Mas bajos: CALLES Y VEREDAS 50%, CTRL ESPACIO PUBLICO 53%. Tasa respuesta 12%.</t>
         </is>
       </c>
     </row>
@@ -536,7 +536,7 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>Cierre 84% sobre 621 incidentes; 'Luminaria superior e inferior apagada du' lidera con 402 casos (88% cierre). Gestion interna 51%.</t>
+          <t>Cierre 85% sobre 503 incidentes; 'Luminaria superior e inferior apagada du' lidera con 342 casos (87% cierre). Gestion interna 53%.</t>
         </is>
       </c>
     </row>
@@ -548,7 +548,7 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>Cierre bajo 35% sobre 148 incidentes; 'Árbol obstruye semáforo/luminaria/cartel' lidera con 65 casos (22% cierre). SLA 37%, sat 25%.</t>
+          <t>Cierre moderado 50% sobre 120 incidentes; 'Árbol obstruye semáforo/luminaria/cartel' lidera con 47 casos (49% cierre). Sat 75% (muestra insuficiente).</t>
         </is>
       </c>
     </row>
@@ -560,7 +560,7 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>Cierre critico 7% sobre 282 incidentes; 'Bache en calle de asfalto' lidera con 104 casos (10% cierre). Sat 25% (muestra insuficiente).</t>
+          <t>Cierre critico 15% sobre 290 incidentes; 'Bache en calle de asfalto' lidera con 101 casos (19% cierre). Sat 50% (muestra insuficiente).</t>
         </is>
       </c>
     </row>
@@ -572,7 +572,7 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>Cierre moderado 58% sobre 89 incidentes; 'Otros ruidos molestos' lidera con 27 casos (48% cierre). SLA 4% critico.</t>
+          <t>Cierre moderado 60% sobre 88 incidentes; 'Otros ruidos molestos' lidera con 28 casos (54% cierre). SLA 23% bajo.</t>
         </is>
       </c>
     </row>
@@ -584,7 +584,7 @@
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>Cierre moderado 61% sobre 348 incidentes; 'Roedores en espacio público' lidera con 168 casos (92% cierre). SLA 19% bajo.</t>
+          <t>Cierre 72% sobre 350 incidentes; 'Roedores en espacio público' lidera con 214 casos (95% cierre). SLA 26% bajo.</t>
         </is>
       </c>
     </row>
@@ -596,7 +596,7 @@
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>Cierre 85% sobre 3046 incidentes; 'Falta de barrido o barrido deficiente' lidera con 822 casos (79% cierre). SLA 33%, sat 61%.</t>
+          <t>Cierre 81% sobre 2691 incidentes; 'Falta de barrido o barrido deficiente' lidera con 998 casos (73% cierre). SLA 40%, sat 65%.</t>
         </is>
       </c>
     </row>
@@ -608,7 +608,7 @@
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>Cierre 71% sobre 551 incidentes; 'Vehículos Abandonados' lidera con 369 casos (79% cierre). Sat 79% (muestra insuficiente).</t>
+          <t>Cierre moderado 69% sobre 514 incidentes; 'Vehículos Abandonados' lidera con 346 casos (79% cierre). Sat 67% (muestra insuficiente).</t>
         </is>
       </c>
     </row>
@@ -623,7 +623,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F20"/>
+  <dimension ref="A1:F18"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -674,27 +674,27 @@
       </c>
       <c r="B2" s="2" t="inlineStr">
         <is>
-          <t>Mar-2026</t>
+          <t>Feb-2026</t>
         </is>
       </c>
       <c r="C2" s="2" t="inlineStr">
         <is>
-          <t>RESIDUOS Y LIMPIEZA</t>
+          <t>Arbolado y Plazas</t>
         </is>
       </c>
       <c r="D2" s="2" t="inlineStr">
         <is>
-          <t>Falta barrido +39%</t>
+          <t>Cierre colapsado</t>
         </is>
       </c>
       <c r="E2" s="2" t="inlineStr">
         <is>
-          <t>822 casos, 79% cierre</t>
+          <t>35%-&gt;50%</t>
         </is>
       </c>
       <c r="F2" s="2" t="inlineStr">
         <is>
-          <t>Falta de barrido: 540-&gt;822 casos (marzo-&gt;abril), cierre 43%-&gt;79%. Mejora marcada del cierre; el tipo se normaliza en gestion aunque el volumen sigue alto.</t>
+          <t>Cierre del area sube de 35% a 50% (Abr-2026 a May-2026). Recuperacion significativa.</t>
         </is>
       </c>
     </row>
@@ -711,22 +711,22 @@
       </c>
       <c r="C3" s="2" t="inlineStr">
         <is>
-          <t>RESIDUOS Y LIMPIEZA</t>
+          <t>Arbolado y Plazas</t>
         </is>
       </c>
       <c r="D3" s="2" t="inlineStr">
         <is>
-          <t>Falta recoleccion organicos cierre critico</t>
+          <t>Arbol obstruye cierre critico</t>
         </is>
       </c>
       <c r="E3" s="2" t="inlineStr">
         <is>
-          <t>206 casos, 87% cierre</t>
+          <t>47 casos, 49% cierre</t>
         </is>
       </c>
       <c r="F3" s="2" t="inlineStr">
         <is>
-          <t>Falta de recoleccion de residuos organicos/humedos: 259-&gt;206 casos, cierre 11%-&gt;87%. Mejora marcada en cierre, volumen estable.</t>
+          <t>Arbol obstruye semaforo/luminaria/cartel: 47 casos con cierre 22%-&gt;49% (Abr-2026 a May-2026). Recuperacion marcada del cierre.</t>
         </is>
       </c>
     </row>
@@ -738,27 +738,27 @@
       </c>
       <c r="B4" s="2" t="inlineStr">
         <is>
-          <t>Mar-2026</t>
+          <t>Abr-2026</t>
         </is>
       </c>
       <c r="C4" s="2" t="inlineStr">
         <is>
-          <t>RESIDUOS Y LIMPIEZA</t>
+          <t>Arbolado y Plazas</t>
         </is>
       </c>
       <c r="D4" s="2" t="inlineStr">
         <is>
-          <t>Retiro restos poda arbolado +104%</t>
+          <t>Dias promedio alto</t>
         </is>
       </c>
       <c r="E4" s="2" t="inlineStr">
         <is>
-          <t>150 casos, 81% cierre</t>
+          <t>7 dias</t>
         </is>
       </c>
       <c r="F4" s="2" t="inlineStr">
         <is>
-          <t>Retiro de restos de poda/arbolado publico: 155-&gt;150 casos, cierre 36%-&gt;81%. Mejora marcada del cierre, volumen estable.</t>
+          <t>Tiempo promedio de resolucion baja a 7 dias en May-2026 (tablero). Vuelve a parametro habitual.</t>
         </is>
       </c>
     </row>
@@ -770,91 +770,91 @@
       </c>
       <c r="B5" s="2" t="inlineStr">
         <is>
-          <t>Mar-2026</t>
+          <t>Abr-2026</t>
         </is>
       </c>
       <c r="C5" s="2" t="inlineStr">
         <is>
-          <t>TRANSITO</t>
+          <t>Control de Actividades Comerciales</t>
         </is>
       </c>
       <c r="D5" s="2" t="inlineStr">
         <is>
-          <t>Reparacion semaforo cierre critico</t>
+          <t>Dias promedio alto</t>
         </is>
       </c>
       <c r="E5" s="2" t="inlineStr">
         <is>
-          <t>118 casos, 64% cierre</t>
+          <t>5 dias</t>
         </is>
       </c>
       <c r="F5" s="2" t="inlineStr">
         <is>
-          <t>Reparacion de semaforo: 57-&gt;118 casos (+107%), cierre 26%-&gt;64%. Mejora marcada del cierre, aunque el volumen subio fuerte.</t>
+          <t>Tiempo promedio de resolucion baja a 5 dias en May-2026 (tablero). Vuelve a parametro habitual.</t>
         </is>
       </c>
     </row>
     <row r="6">
-      <c r="A6" s="3" t="inlineStr">
-        <is>
-          <t>PERSISTE</t>
-        </is>
-      </c>
-      <c r="B6" s="3" t="inlineStr">
-        <is>
-          <t>Feb-2026</t>
-        </is>
-      </c>
-      <c r="C6" s="3" t="inlineStr">
-        <is>
-          <t>ARBOLADO Y PLAZAS</t>
-        </is>
-      </c>
-      <c r="D6" s="3" t="inlineStr">
-        <is>
-          <t>Cierre colapsado</t>
-        </is>
-      </c>
-      <c r="E6" s="3" t="inlineStr">
-        <is>
-          <t>29%-&gt;35%</t>
-        </is>
-      </c>
-      <c r="F6" s="3" t="inlineStr">
-        <is>
-          <t>Cierre del area 29%-&gt;35% (marzo a abril). Persiste debajo del umbral 50%. Cumplido real 31%, Cancelado 34% sobre cerrados.</t>
+      <c r="A6" s="2" t="inlineStr">
+        <is>
+          <t>RESUELTA</t>
+        </is>
+      </c>
+      <c r="B6" s="2" t="inlineStr">
+        <is>
+          <t>Abr-2026</t>
+        </is>
+      </c>
+      <c r="C6" s="2" t="inlineStr">
+        <is>
+          <t>Control del Espacio Publico</t>
+        </is>
+      </c>
+      <c r="D6" s="2" t="inlineStr">
+        <is>
+          <t>Cierre bajo - Cable cortado</t>
+        </is>
+      </c>
+      <c r="E6" s="2" t="inlineStr">
+        <is>
+          <t>4%-&gt;72%</t>
+        </is>
+      </c>
+      <c r="F6" s="2" t="inlineStr">
+        <is>
+          <t>Cierre del area sube de 4% a 72% (Abr-2026 a May-2026). Recuperacion significativa.</t>
         </is>
       </c>
     </row>
     <row r="7">
-      <c r="A7" s="3" t="inlineStr">
-        <is>
-          <t>PERSISTE</t>
-        </is>
-      </c>
-      <c r="B7" s="3" t="inlineStr">
-        <is>
-          <t>Feb-2026</t>
-        </is>
-      </c>
-      <c r="C7" s="3" t="inlineStr">
-        <is>
-          <t>ARBOLADO Y PLAZAS</t>
-        </is>
-      </c>
-      <c r="D7" s="3" t="inlineStr">
-        <is>
-          <t>% Cancelado &gt;10%</t>
-        </is>
-      </c>
-      <c r="E7" s="3" t="inlineStr">
-        <is>
-          <t>34% (sobre cerrados)</t>
-        </is>
-      </c>
-      <c r="F7" s="3" t="inlineStr">
-        <is>
-          <t>Cancelado 34% de los cerrados en abril (donut Cierres por Estado). Sigue por encima del 10% de referencia.</t>
+      <c r="A7" s="2" t="inlineStr">
+        <is>
+          <t>RESUELTA</t>
+        </is>
+      </c>
+      <c r="B7" s="2" t="inlineStr">
+        <is>
+          <t>Abr-2026</t>
+        </is>
+      </c>
+      <c r="C7" s="2" t="inlineStr">
+        <is>
+          <t>Residuos y Limpieza</t>
+        </is>
+      </c>
+      <c r="D7" s="2" t="inlineStr">
+        <is>
+          <t>Cierre bajo - Falta de recolección de residuos reciclables (Pr</t>
+        </is>
+      </c>
+      <c r="E7" s="2" t="inlineStr">
+        <is>
+          <t>27%-&gt;81%</t>
+        </is>
+      </c>
+      <c r="F7" s="2" t="inlineStr">
+        <is>
+          <t>Cierre del area sube de 27% a 81% (Abr-2026 a May-2026). Recuperacion significativa.</t>
         </is>
       </c>
     </row>
@@ -866,27 +866,27 @@
       </c>
       <c r="B8" s="3" t="inlineStr">
         <is>
-          <t>Mar-2026</t>
+          <t>Feb-2026</t>
         </is>
       </c>
       <c r="C8" s="3" t="inlineStr">
         <is>
-          <t>ARBOLADO Y PLAZAS</t>
+          <t>Arbolado y Plazas</t>
         </is>
       </c>
       <c r="D8" s="3" t="inlineStr">
         <is>
-          <t>Arbol obstruye cierre critico</t>
+          <t>% Cancelado &gt;10%</t>
         </is>
       </c>
       <c r="E8" s="3" t="inlineStr">
         <is>
-          <t>65 casos, 22% cierre</t>
+          <t>32% (sobre cerrados)</t>
         </is>
       </c>
       <c r="F8" s="3" t="inlineStr">
         <is>
-          <t>Arbol obstruye semaforo/luminaria: 65 casos con 22% cierre en abril (era 14% en marzo). Tipo dominante del area con cierre por debajo del umbral.</t>
+          <t>Cancelado 32% de los cerrados en May-2026 (donut Cierres por Estado). Proporcion elevada que persiste.</t>
         </is>
       </c>
     </row>
@@ -903,7 +903,7 @@
       </c>
       <c r="C9" s="3" t="inlineStr">
         <is>
-          <t>CALLES Y VEREDAS</t>
+          <t>Calles y Veredas</t>
         </is>
       </c>
       <c r="D9" s="3" t="inlineStr">
@@ -913,12 +913,12 @@
       </c>
       <c r="E9" s="3" t="inlineStr">
         <is>
-          <t>32%-&gt;7%</t>
+          <t>7%-&gt;15%</t>
         </is>
       </c>
       <c r="F9" s="3" t="inlineStr">
         <is>
-          <t>Cierre del area 32%-&gt;7% (marzo a abril). Persiste debajo del umbral 50%. Cumplido real 6%, Cancelado 21% sobre cerrados.</t>
+          <t>Cierre del area 7%-&gt;15% (Abr-2026 a May-2026). Sigue en zona critica. Cancelado 24% sobre cerrados.</t>
         </is>
       </c>
     </row>
@@ -935,7 +935,7 @@
       </c>
       <c r="C10" s="3" t="inlineStr">
         <is>
-          <t>CONTROL DE ACT. COMERCIALES</t>
+          <t>Control de Actividades Comerciales</t>
         </is>
       </c>
       <c r="D10" s="3" t="inlineStr">
@@ -945,12 +945,12 @@
       </c>
       <c r="E10" s="3" t="inlineStr">
         <is>
-          <t>4%</t>
+          <t>23%</t>
         </is>
       </c>
       <c r="F10" s="3" t="inlineStr">
         <is>
-          <t>SLA 4% en abril (tablero), persiste debajo del umbral 30%.</t>
+          <t>SLA 23% en May-2026 (tablero), persiste en niveles bajos.</t>
         </is>
       </c>
     </row>
@@ -967,7 +967,7 @@
       </c>
       <c r="C11" s="3" t="inlineStr">
         <is>
-          <t>CONTROL DEL ESPACIO PUBLICO</t>
+          <t>Control del Espacio Publico</t>
         </is>
       </c>
       <c r="D11" s="3" t="inlineStr">
@@ -977,12 +977,12 @@
       </c>
       <c r="E11" s="3" t="inlineStr">
         <is>
-          <t>19%</t>
+          <t>26%</t>
         </is>
       </c>
       <c r="F11" s="3" t="inlineStr">
         <is>
-          <t>SLA 19% en abril (tablero), persiste debajo del umbral 30%.</t>
+          <t>SLA 26% en May-2026 (tablero), persiste en niveles bajos.</t>
         </is>
       </c>
     </row>
@@ -994,34 +994,34 @@
       </c>
       <c r="B12" s="3" t="inlineStr">
         <is>
-          <t>Feb-2026</t>
+          <t>Abr-2026</t>
         </is>
       </c>
       <c r="C12" s="3" t="inlineStr">
         <is>
-          <t>TRANSITO</t>
+          <t>Calles y Veredas</t>
         </is>
       </c>
       <c r="D12" s="3" t="inlineStr">
         <is>
-          <t>% Cancelado excesivo</t>
+          <t>Cancelado alto en cerrados</t>
         </is>
       </c>
       <c r="E12" s="3" t="inlineStr">
         <is>
-          <t>26% (sobre cerrados)</t>
+          <t>24% (sobre cerrados)</t>
         </is>
       </c>
       <c r="F12" s="3" t="inlineStr">
         <is>
-          <t>Cancelado 26% de los cerrados en abril (donut Cierres por Estado). Sigue por encima del 10% de referencia.</t>
+          <t>Cancelado 24% de los cerrados en May-2026 (donut Cierres por Estado). Proporcion elevada que persiste.</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" s="3" t="inlineStr">
         <is>
-          <t>NUEVA</t>
+          <t>PERSISTE</t>
         </is>
       </c>
       <c r="B13" s="3" t="inlineStr">
@@ -1031,29 +1031,29 @@
       </c>
       <c r="C13" s="3" t="inlineStr">
         <is>
-          <t>Arbolado y Plazas</t>
+          <t>Calles y Veredas</t>
         </is>
       </c>
       <c r="D13" s="3" t="inlineStr">
         <is>
-          <t>Dias promedio alto</t>
+          <t>Muestra encuesta insuficiente</t>
         </is>
       </c>
       <c r="E13" s="3" t="inlineStr">
         <is>
-          <t>8 dias</t>
+          <t>Tasa 2.1%</t>
         </is>
       </c>
       <c r="F13" s="3" t="inlineStr">
         <is>
-          <t>Tiempo promedio de resolucion 8 dias en abril (tablero, umbral &gt;7).</t>
+          <t>Tasa de respuesta encuesta 2.1% (6 respuestas sobre 290 incidentes) en May-2026. Datos de satisfaccion no representativos.</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" s="3" t="inlineStr">
         <is>
-          <t>NUEVA</t>
+          <t>PERSISTE</t>
         </is>
       </c>
       <c r="B14" s="3" t="inlineStr">
@@ -1063,7 +1063,7 @@
       </c>
       <c r="C14" s="3" t="inlineStr">
         <is>
-          <t>Calles y Veredas</t>
+          <t>Control del Espacio Publico</t>
         </is>
       </c>
       <c r="D14" s="3" t="inlineStr">
@@ -1073,51 +1073,51 @@
       </c>
       <c r="E14" s="3" t="inlineStr">
         <is>
-          <t>21% (sobre cerrados)</t>
+          <t>12% (sobre cerrados)</t>
         </is>
       </c>
       <c r="F14" s="3" t="inlineStr">
         <is>
-          <t>21% de los cerrados son Cancelados (donut Cierres por Estado, umbral &gt;10%). Revisar calidad de cierre.</t>
+          <t>Cancelado 12% de los cerrados en May-2026 (donut Cierres por Estado). Proporcion elevada que persiste.</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" s="3" t="inlineStr">
         <is>
-          <t>NUEVA</t>
+          <t>PERSISTE</t>
         </is>
       </c>
       <c r="B15" s="3" t="inlineStr">
         <is>
-          <t>Abr-2026</t>
+          <t>Feb-2026</t>
         </is>
       </c>
       <c r="C15" s="3" t="inlineStr">
         <is>
-          <t>Calles y Veredas</t>
+          <t>Transito</t>
         </is>
       </c>
       <c r="D15" s="3" t="inlineStr">
         <is>
-          <t>Muestra encuesta insuficiente</t>
+          <t>% Cancelado excesivo</t>
         </is>
       </c>
       <c r="E15" s="3" t="inlineStr">
         <is>
-          <t>Tasa 1.4%</t>
+          <t>24% (sobre cerrados)</t>
         </is>
       </c>
       <c r="F15" s="3" t="inlineStr">
         <is>
-          <t>Tasa de respuesta encuesta 1.4% (4 respuestas sobre 282 incidentes). Datos de satisfaccion no representativos.</t>
+          <t>Cancelado 24% de los cerrados en May-2026 (donut Cierres por Estado). Proporcion elevada que persiste.</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" s="3" t="inlineStr">
         <is>
-          <t>NUEVA</t>
+          <t>PERSISTE</t>
         </is>
       </c>
       <c r="B16" s="3" t="inlineStr">
@@ -1127,22 +1127,22 @@
       </c>
       <c r="C16" s="3" t="inlineStr">
         <is>
-          <t>Control de Actividades Comerciales</t>
+          <t>Transito</t>
         </is>
       </c>
       <c r="D16" s="3" t="inlineStr">
         <is>
-          <t>Dias promedio alto</t>
+          <t>Muestra encuesta insuficiente</t>
         </is>
       </c>
       <c r="E16" s="3" t="inlineStr">
         <is>
-          <t>9 dias</t>
+          <t>Tasa 4.1%</t>
         </is>
       </c>
       <c r="F16" s="3" t="inlineStr">
         <is>
-          <t>Tiempo promedio de resolucion 9 dias en abril (tablero, umbral &gt;7).</t>
+          <t>Tasa de respuesta encuesta 4.1% (21 respuestas sobre 514 incidentes) en May-2026. Datos de satisfaccion no representativos.</t>
         </is>
       </c>
     </row>
@@ -1154,27 +1154,27 @@
       </c>
       <c r="B17" s="3" t="inlineStr">
         <is>
-          <t>Abr-2026</t>
+          <t>May-2026</t>
         </is>
       </c>
       <c r="C17" s="3" t="inlineStr">
         <is>
-          <t>Control del Espacio Publico</t>
+          <t>Arbolado y Plazas</t>
         </is>
       </c>
       <c r="D17" s="3" t="inlineStr">
         <is>
-          <t>Cancelado alto en cerrados</t>
+          <t>Muestra encuesta insuficiente</t>
         </is>
       </c>
       <c r="E17" s="3" t="inlineStr">
         <is>
-          <t>15% (sobre cerrados)</t>
+          <t>Tasa 3.3%</t>
         </is>
       </c>
       <c r="F17" s="3" t="inlineStr">
         <is>
-          <t>15% de los cerrados son Cancelados (donut Cierres por Estado, umbral &gt;10%). Revisar calidad de cierre.</t>
+          <t>Tasa de respuesta encuesta 3.3% (4 respuestas sobre 120 incidentes). Datos de satisfaccion no representativos.</t>
         </is>
       </c>
     </row>
@@ -1186,91 +1186,27 @@
       </c>
       <c r="B18" s="3" t="inlineStr">
         <is>
-          <t>Abr-2026</t>
+          <t>May-2026</t>
         </is>
       </c>
       <c r="C18" s="3" t="inlineStr">
         <is>
-          <t>Control del Espacio Publico</t>
+          <t>Transito</t>
         </is>
       </c>
       <c r="D18" s="3" t="inlineStr">
         <is>
-          <t>Cierre bajo - Cable cortado</t>
+          <t>Cierre bajo - Vehículo mal estacionado</t>
         </is>
       </c>
       <c r="E18" s="3" t="inlineStr">
         <is>
-          <t>4% (55 casos)</t>
+          <t>0% (22 casos)</t>
         </is>
       </c>
       <c r="F18" s="3" t="inlineStr">
         <is>
-          <t>Tipo 'Cable cortado': 55 casos en abril con 4% de cierre (tablero, umbral &lt;40% con volumen &gt;=20).</t>
-        </is>
-      </c>
-    </row>
-    <row r="19">
-      <c r="A19" s="3" t="inlineStr">
-        <is>
-          <t>NUEVA</t>
-        </is>
-      </c>
-      <c r="B19" s="3" t="inlineStr">
-        <is>
-          <t>Abr-2026</t>
-        </is>
-      </c>
-      <c r="C19" s="3" t="inlineStr">
-        <is>
-          <t>Residuos y Limpieza</t>
-        </is>
-      </c>
-      <c r="D19" s="3" t="inlineStr">
-        <is>
-          <t>Cierre bajo - Falta de recolección de residuos reciclables (Pr</t>
-        </is>
-      </c>
-      <c r="E19" s="3" t="inlineStr">
-        <is>
-          <t>27% (55 casos)</t>
-        </is>
-      </c>
-      <c r="F19" s="3" t="inlineStr">
-        <is>
-          <t>Tipo 'Falta de recolección de residuos reciclables (Programa Día Verde)': 55 casos en abril con 27% de cierre (tablero, umbral &lt;40% con volumen &gt;=20).</t>
-        </is>
-      </c>
-    </row>
-    <row r="20">
-      <c r="A20" s="3" t="inlineStr">
-        <is>
-          <t>NUEVA</t>
-        </is>
-      </c>
-      <c r="B20" s="3" t="inlineStr">
-        <is>
-          <t>Abr-2026</t>
-        </is>
-      </c>
-      <c r="C20" s="3" t="inlineStr">
-        <is>
-          <t>Transito</t>
-        </is>
-      </c>
-      <c r="D20" s="3" t="inlineStr">
-        <is>
-          <t>Muestra encuesta insuficiente</t>
-        </is>
-      </c>
-      <c r="E20" s="3" t="inlineStr">
-        <is>
-          <t>Tasa 4.4%</t>
-        </is>
-      </c>
-      <c r="F20" s="3" t="inlineStr">
-        <is>
-          <t>Tasa de respuesta encuesta 4.4% (24 respuestas sobre 550 incidentes). Datos de satisfaccion no representativos.</t>
+          <t>Tipo 'Vehículo mal estacionado': 22 casos en May-2026 con 0% de cierre (tablero). Cierre muy por debajo del resto del area.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Tablas_Stock vigente v2 - Jun-2026
</commit_message>
<xml_diff>
--- a/Tablas/Tablas_Stock.xlsx
+++ b/Tablas/Tablas_Stock.xlsx
@@ -458,7 +458,7 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>Total 4556 incidentes en mayo (-10% vs abril, 5072). RESIDUOS Y LIMPIEZA concentra 59% del volumen (2691 casos, -11%). Bajas generalizadas: ALUMBRADO -18%, ARBOLADO -21%.</t>
+          <t>Total 4309 incidentes en junio (-5% vs mayo, 4555). RESIDUOS Y LIMPIEZA concentra 57% del volumen (2457 casos, -9%). Subas: CTRL ACTIVIDADES +45%, CALLES +15%; baja CTRL ESPACIO -24%.</t>
         </is>
       </c>
     </row>
@@ -470,7 +470,7 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>Cierre global 74% (+0.0pp vs abril). CALLES Y VEREDAS en 15%, ARBOLADO 50%. ALUMBRADO 85% y RESIDUOS 81% lideran. Cancelado sobre cerrados alto en ARBOLADO 32%, CALLES 25%, TRANSITO 24%.</t>
+          <t>Cierre global 79% (+5pp vs mayo). ALUMBRADO 89%, RESIDUOS 89% y CTRL ACTIVIDADES 86% lideran. Criticos: CALLES 23% y ARBOLADO 40%. Cancelado sobre cerrados bajo en todas las areas (max TRANSITO 9%).</t>
         </is>
       </c>
     </row>
@@ -482,7 +482,7 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>SLA global 44% (+3.0pp vs abril). TRANSITO 31% y CTRL ACT COMERCIALES 30% bajos. ALUMBRADO lidera con 71%, RESIDUOS 40%, ARBOLADO 45%. Promedio 3 dias.</t>
+          <t>SLA global 38% (-6pp vs mayo). ARBOLADO 76% y CTRL ESPACIO 61% lideran; ALUMBRADO 55%. Mas bajos: RESIDUOS 31% y TRANSITO 38%. Promedio 4 dias para cerrados.</t>
         </is>
       </c>
     </row>
@@ -494,7 +494,7 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>Satisfaccion global 64% (+1.0pp vs abril). ARBOLADO 75% lidera. Mas bajos: CALLES Y VEREDAS 50%, CTRL ESPACIO PUBLICO 53%. Tasa respuesta 12%.</t>
+          <t>Satisfaccion global 70% (+6pp vs mayo). Muestra en maduracion: tasa de respuesta 3.5% (149 respuestas), las 7 areas por debajo del 5%. Dato publicado con reserva por representatividad.</t>
         </is>
       </c>
     </row>
@@ -536,7 +536,7 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>Cierre 85% sobre 503 incidentes; 'Luminaria superior e inferior apagada du' lidera con 342 casos (87% cierre). Gestion interna 53%.</t>
+          <t>Cierre 89% sobre 493 incidentes; 'Luminaria superior e inferior apagada du' lidera con 303 casos (88% cierre). Gestion interna 56%.</t>
         </is>
       </c>
     </row>
@@ -548,7 +548,7 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>Cierre moderado 50% sobre 120 incidentes; 'Árbol obstruye semáforo/luminaria/cartel' lidera con 47 casos (49% cierre). Sat 75% (muestra insuficiente).</t>
+          <t>Cierre bajo 40% sobre 124 incidentes; 'Árbol obstruye semáforo/luminaria/cartel' lidera con 46 casos (39% cierre). Sat 50% (muestra insuficiente).</t>
         </is>
       </c>
     </row>
@@ -560,7 +560,7 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>Cierre critico 15% sobre 292 incidentes; 'Bache en calle de asfalto' lidera con 101 casos (19% cierre). Sat 50% (muestra insuficiente).</t>
+          <t>Cierre bajo 23% sobre 332 incidentes; 'Bache en calle de asfalto' lidera con 129 casos (24% cierre). Dias prom 9.0 elevado.</t>
         </is>
       </c>
     </row>
@@ -572,7 +572,7 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>Cierre moderado 60% sobre 88 incidentes; 'Otros ruidos molestos' lidera con 28 casos (54% cierre). SLA 30%, sat 67%.</t>
+          <t>Cierre 86% sobre 128 incidentes; 'Otros ruidos molestos' lidera con 54 casos (87% cierre). Sat 20% (muestra insuficiente).</t>
         </is>
       </c>
     </row>
@@ -584,7 +584,7 @@
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>Cierre 72% sobre 348 incidentes; 'Roedores en espacio público' lidera con 214 casos (95% cierre). SLA 50%, sat 53%.</t>
+          <t>Cierre 75% sobre 263 incidentes; 'Roedores en espacio público' lidera con 97 casos (95% cierre). Sat 40% (muestra insuficiente).</t>
         </is>
       </c>
     </row>
@@ -596,7 +596,7 @@
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>Cierre 81% sobre 2691 incidentes; 'Falta de barrido o barrido deficiente' lidera con 998 casos (73% cierre). SLA 40%, sat 65%.</t>
+          <t>Cierre 89% sobre 2457 incidentes; 'Falta de barrido o barrido deficiente' lidera con 930 casos (92% cierre). Sat 72% (muestra insuficiente).</t>
         </is>
       </c>
     </row>
@@ -608,7 +608,7 @@
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>Cierre moderado 69% sobre 514 incidentes; 'Vehículos Abandonados' lidera con 346 casos (79% cierre). Sat 67% (muestra insuficiente).</t>
+          <t>Cierre moderado 67% sobre 512 incidentes; 'Vehículos Abandonados' lidera con 405 casos (75% cierre). Sat 100% (muestra insuficiente).</t>
         </is>
       </c>
     </row>
@@ -623,7 +623,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F18"/>
+  <dimension ref="A1:F14"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -684,17 +684,17 @@
       </c>
       <c r="D2" s="2" t="inlineStr">
         <is>
-          <t>Cierre colapsado</t>
+          <t>% Cancelado &gt;10%</t>
         </is>
       </c>
       <c r="E2" s="2" t="inlineStr">
         <is>
-          <t>35%-&gt;50%</t>
+          <t>4% (sobre cerrados)</t>
         </is>
       </c>
       <c r="F2" s="2" t="inlineStr">
         <is>
-          <t>Cierre del area sube de 35% a 50% (Abr-2026 a May-2026). Recuperacion significativa.</t>
+          <t>Cancelado baja a 4% de los cerrados en Jun-2026 (donut Cierres por Estado), dentro del rango operativo.</t>
         </is>
       </c>
     </row>
@@ -706,7 +706,7 @@
       </c>
       <c r="B3" s="2" t="inlineStr">
         <is>
-          <t>Mar-2026</t>
+          <t>May-2026</t>
         </is>
       </c>
       <c r="C3" s="2" t="inlineStr">
@@ -716,17 +716,17 @@
       </c>
       <c r="D3" s="2" t="inlineStr">
         <is>
-          <t>Arbol obstruye cierre critico</t>
+          <t>Muestra encuesta insuficiente</t>
         </is>
       </c>
       <c r="E3" s="2" t="inlineStr">
         <is>
-          <t>47 casos, 49% cierre</t>
+          <t>consolidada</t>
         </is>
       </c>
       <c r="F3" s="2" t="inlineStr">
         <is>
-          <t>Arbol obstruye cierre critico: 47 casos, cierre 22%-&gt;49% (Abr-2026 a May-2026). Recuperacion del cierre.</t>
+          <t>Alerta de muestra por area consolidada en la alerta global de tasa de respuesta de encuesta (Jun-2026).</t>
         </is>
       </c>
     </row>
@@ -743,22 +743,22 @@
       </c>
       <c r="C4" s="2" t="inlineStr">
         <is>
-          <t>Arbolado y Plazas</t>
+          <t>Calles y Veredas</t>
         </is>
       </c>
       <c r="D4" s="2" t="inlineStr">
         <is>
-          <t>Dias promedio alto</t>
+          <t>Cancelado alto en cerrados</t>
         </is>
       </c>
       <c r="E4" s="2" t="inlineStr">
         <is>
-          <t>7 dias</t>
+          <t>4% (sobre cerrados)</t>
         </is>
       </c>
       <c r="F4" s="2" t="inlineStr">
         <is>
-          <t>Tiempo promedio de resolucion baja a 7 dias en May-2026 (tablero). Vuelve a parametro habitual.</t>
+          <t>Cancelado baja a 4% de los cerrados en Jun-2026 (donut Cierres por Estado), dentro del rango operativo.</t>
         </is>
       </c>
     </row>
@@ -770,27 +770,27 @@
       </c>
       <c r="B5" s="2" t="inlineStr">
         <is>
-          <t>Feb-2026</t>
+          <t>Abr-2026</t>
         </is>
       </c>
       <c r="C5" s="2" t="inlineStr">
         <is>
-          <t>Control de Actividades Comerciales</t>
+          <t>Calles y Veredas</t>
         </is>
       </c>
       <c r="D5" s="2" t="inlineStr">
         <is>
-          <t>SLA critico</t>
+          <t>Muestra encuesta insuficiente</t>
         </is>
       </c>
       <c r="E5" s="2" t="inlineStr">
         <is>
-          <t>30%</t>
+          <t>consolidada</t>
         </is>
       </c>
       <c r="F5" s="2" t="inlineStr">
         <is>
-          <t>SLA sube a 30% en May-2026 (tablero), sale de zona critica.</t>
+          <t>Alerta de muestra por area consolidada en la alerta global de tasa de respuesta de encuesta (Jun-2026).</t>
         </is>
       </c>
     </row>
@@ -802,7 +802,7 @@
       </c>
       <c r="B6" s="2" t="inlineStr">
         <is>
-          <t>Feb-2026</t>
+          <t>Abr-2026</t>
         </is>
       </c>
       <c r="C6" s="2" t="inlineStr">
@@ -812,17 +812,17 @@
       </c>
       <c r="D6" s="2" t="inlineStr">
         <is>
-          <t>SLA por area</t>
+          <t>Cancelado alto en cerrados</t>
         </is>
       </c>
       <c r="E6" s="2" t="inlineStr">
         <is>
-          <t>50%</t>
+          <t>1% (sobre cerrados)</t>
         </is>
       </c>
       <c r="F6" s="2" t="inlineStr">
         <is>
-          <t>SLA sube a 50% en May-2026 (tablero), sale de zona critica.</t>
+          <t>Cancelado baja a 1% de los cerrados en Jun-2026 (donut Cierres por Estado), dentro del rango operativo.</t>
         </is>
       </c>
     </row>
@@ -834,27 +834,27 @@
       </c>
       <c r="B7" s="2" t="inlineStr">
         <is>
-          <t>Abr-2026</t>
+          <t>Feb-2026</t>
         </is>
       </c>
       <c r="C7" s="2" t="inlineStr">
         <is>
-          <t>Control de Actividades Comerciales</t>
+          <t>Transito</t>
         </is>
       </c>
       <c r="D7" s="2" t="inlineStr">
         <is>
-          <t>Dias promedio alto</t>
+          <t>% Cancelado excesivo</t>
         </is>
       </c>
       <c r="E7" s="2" t="inlineStr">
         <is>
-          <t>5 dias</t>
+          <t>9% (sobre cerrados)</t>
         </is>
       </c>
       <c r="F7" s="2" t="inlineStr">
         <is>
-          <t>Tiempo promedio de resolucion baja a 5 dias en May-2026 (tablero). Vuelve a parametro habitual.</t>
+          <t>Cancelado baja a 9% de los cerrados en Jun-2026 (donut Cierres por Estado), dentro del rango operativo.</t>
         </is>
       </c>
     </row>
@@ -871,22 +871,22 @@
       </c>
       <c r="C8" s="2" t="inlineStr">
         <is>
-          <t>Control del Espacio Publico</t>
+          <t>Transito</t>
         </is>
       </c>
       <c r="D8" s="2" t="inlineStr">
         <is>
-          <t>Cierre bajo - Cable cortado</t>
+          <t>Muestra encuesta insuficiente</t>
         </is>
       </c>
       <c r="E8" s="2" t="inlineStr">
         <is>
-          <t>4%-&gt;72%</t>
+          <t>consolidada</t>
         </is>
       </c>
       <c r="F8" s="2" t="inlineStr">
         <is>
-          <t>Cierre del area sube de 4% a 72% (Abr-2026 a May-2026). Recuperacion significativa.</t>
+          <t>Alerta de muestra por area consolidada en la alerta global de tasa de respuesta de encuesta (Jun-2026).</t>
         </is>
       </c>
     </row>
@@ -898,27 +898,27 @@
       </c>
       <c r="B9" s="2" t="inlineStr">
         <is>
-          <t>Abr-2026</t>
+          <t>May-2026</t>
         </is>
       </c>
       <c r="C9" s="2" t="inlineStr">
         <is>
-          <t>Residuos y Limpieza</t>
+          <t>Transito</t>
         </is>
       </c>
       <c r="D9" s="2" t="inlineStr">
         <is>
-          <t>Cierre bajo - Falta de recolección de residuos reciclables (Pr</t>
+          <t>Cierre bajo - Vehiculo mal estacionado</t>
         </is>
       </c>
       <c r="E9" s="2" t="inlineStr">
         <is>
-          <t>27%-&gt;81%</t>
+          <t>67%</t>
         </is>
       </c>
       <c r="F9" s="2" t="inlineStr">
         <is>
-          <t>Cierre del area sube de 27% a 81% (Abr-2026 a May-2026). Recuperacion significativa.</t>
+          <t>Cierre del area sube de 0% a 67% (May-2026 a Jun-2026). Recuperacion significativa.</t>
         </is>
       </c>
     </row>
@@ -930,71 +930,71 @@
       </c>
       <c r="B10" s="3" t="inlineStr">
         <is>
-          <t>Feb-2026</t>
+          <t>Mar-2026</t>
         </is>
       </c>
       <c r="C10" s="3" t="inlineStr">
         <is>
-          <t>Arbolado y Plazas</t>
+          <t>Calles y Veredas</t>
         </is>
       </c>
       <c r="D10" s="3" t="inlineStr">
         <is>
-          <t>% Cancelado &gt;10%</t>
+          <t>Cierre colapsado</t>
         </is>
       </c>
       <c r="E10" s="3" t="inlineStr">
         <is>
-          <t>32% (sobre cerrados)</t>
+          <t>15%-&gt;23%</t>
         </is>
       </c>
       <c r="F10" s="3" t="inlineStr">
         <is>
-          <t>Cancelado 32% de los cerrados en May-2026 (donut Cierres por Estado). Proporcion elevada que persiste.</t>
+          <t>Cierre del area 15%-&gt;23% (May-2026 a Jun-2026). Sigue en zona critica. Cancelado 4% sobre cerrados.</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" s="3" t="inlineStr">
         <is>
-          <t>PERSISTE</t>
+          <t>NUEVA</t>
         </is>
       </c>
       <c r="B11" s="3" t="inlineStr">
         <is>
-          <t>Mar-2026</t>
+          <t>Jun-2026</t>
         </is>
       </c>
       <c r="C11" s="3" t="inlineStr">
         <is>
-          <t>Calles y Veredas</t>
+          <t>Arbolado y Plazas</t>
         </is>
       </c>
       <c r="D11" s="3" t="inlineStr">
         <is>
-          <t>Cierre colapsado</t>
+          <t>Cierre bajo (area)</t>
         </is>
       </c>
       <c r="E11" s="3" t="inlineStr">
         <is>
-          <t>7%-&gt;15%</t>
+          <t>40%</t>
         </is>
       </c>
       <c r="F11" s="3" t="inlineStr">
         <is>
-          <t>Cierre del area 7%-&gt;15% (Abr-2026 a May-2026). Sigue en zona critica. Cancelado 25% sobre cerrados.</t>
+          <t>Cierre del area 40% en Jun-2026 (tablero). Cancelado 4% sobre cerrados.</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" s="3" t="inlineStr">
         <is>
-          <t>PERSISTE</t>
+          <t>NUEVA</t>
         </is>
       </c>
       <c r="B12" s="3" t="inlineStr">
         <is>
-          <t>Abr-2026</t>
+          <t>Jun-2026</t>
         </is>
       </c>
       <c r="C12" s="3" t="inlineStr">
@@ -1004,209 +1004,81 @@
       </c>
       <c r="D12" s="3" t="inlineStr">
         <is>
-          <t>Cancelado alto en cerrados</t>
+          <t>Dias promedio alto</t>
         </is>
       </c>
       <c r="E12" s="3" t="inlineStr">
         <is>
-          <t>25% (sobre cerrados)</t>
+          <t>9 dias</t>
         </is>
       </c>
       <c r="F12" s="3" t="inlineStr">
         <is>
-          <t>Cancelado 25% de los cerrados en May-2026 (donut Cierres por Estado). Proporcion elevada que persiste.</t>
+          <t>Tiempo promedio de resolucion 9 dias en Jun-2026 (tablero). Por encima del tiempo habitual.</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" s="3" t="inlineStr">
         <is>
-          <t>PERSISTE</t>
+          <t>NUEVA</t>
         </is>
       </c>
       <c r="B13" s="3" t="inlineStr">
         <is>
-          <t>Abr-2026</t>
+          <t>Jun-2026</t>
         </is>
       </c>
       <c r="C13" s="3" t="inlineStr">
         <is>
-          <t>Calles y Veredas</t>
+          <t>GENERAL</t>
         </is>
       </c>
       <c r="D13" s="3" t="inlineStr">
         <is>
-          <t>Muestra encuesta insuficiente</t>
+          <t>Muestra de encuesta insuficiente (municipio)</t>
         </is>
       </c>
       <c r="E13" s="3" t="inlineStr">
         <is>
-          <t>Tasa 2.1%</t>
+          <t>Tasa 3.5% (7/7 areas &lt;5%)</t>
         </is>
       </c>
       <c r="F13" s="3" t="inlineStr">
         <is>
-          <t>Tasa de respuesta encuesta 2.1% (6 respuestas sobre 292 incidentes) en May-2026. Datos de satisfaccion no representativos.</t>
+          <t>Tasa de respuesta de encuesta 3.5% en Jun-2026 (149 respuestas sobre 4309 incidentes); las 7 areas del monitor quedan por debajo del 5%. La baja responde a la maduracion de la encuesta (las respuestas de Jun-2026 aun no se acumularon al corte), no a una caida de satisfaccion. La satisfaccion por area se publica con la marca '(muestra insuficiente)'.</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" s="3" t="inlineStr">
         <is>
-          <t>PERSISTE</t>
+          <t>NUEVA</t>
         </is>
       </c>
       <c r="B14" s="3" t="inlineStr">
         <is>
-          <t>Abr-2026</t>
+          <t>Jun-2026</t>
         </is>
       </c>
       <c r="C14" s="3" t="inlineStr">
         <is>
-          <t>Control del Espacio Publico</t>
+          <t>Residuos y Limpieza</t>
         </is>
       </c>
       <c r="D14" s="3" t="inlineStr">
         <is>
-          <t>Cancelado alto en cerrados</t>
+          <t>Cierre bajo - Falta de recolección de residuos reciclables (Pr</t>
         </is>
       </c>
       <c r="E14" s="3" t="inlineStr">
         <is>
-          <t>12% (sobre cerrados)</t>
+          <t>22% (40 casos)</t>
         </is>
       </c>
       <c r="F14" s="3" t="inlineStr">
         <is>
-          <t>Cancelado 12% de los cerrados en May-2026 (donut Cierres por Estado). Proporcion elevada que persiste.</t>
-        </is>
-      </c>
-    </row>
-    <row r="15">
-      <c r="A15" s="3" t="inlineStr">
-        <is>
-          <t>PERSISTE</t>
-        </is>
-      </c>
-      <c r="B15" s="3" t="inlineStr">
-        <is>
-          <t>Feb-2026</t>
-        </is>
-      </c>
-      <c r="C15" s="3" t="inlineStr">
-        <is>
-          <t>Transito</t>
-        </is>
-      </c>
-      <c r="D15" s="3" t="inlineStr">
-        <is>
-          <t>% Cancelado excesivo</t>
-        </is>
-      </c>
-      <c r="E15" s="3" t="inlineStr">
-        <is>
-          <t>24% (sobre cerrados)</t>
-        </is>
-      </c>
-      <c r="F15" s="3" t="inlineStr">
-        <is>
-          <t>Cancelado 24% de los cerrados en May-2026 (donut Cierres por Estado). Proporcion elevada que persiste.</t>
-        </is>
-      </c>
-    </row>
-    <row r="16">
-      <c r="A16" s="3" t="inlineStr">
-        <is>
-          <t>PERSISTE</t>
-        </is>
-      </c>
-      <c r="B16" s="3" t="inlineStr">
-        <is>
-          <t>Abr-2026</t>
-        </is>
-      </c>
-      <c r="C16" s="3" t="inlineStr">
-        <is>
-          <t>Transito</t>
-        </is>
-      </c>
-      <c r="D16" s="3" t="inlineStr">
-        <is>
-          <t>Muestra encuesta insuficiente</t>
-        </is>
-      </c>
-      <c r="E16" s="3" t="inlineStr">
-        <is>
-          <t>Tasa 4.1%</t>
-        </is>
-      </c>
-      <c r="F16" s="3" t="inlineStr">
-        <is>
-          <t>Tasa de respuesta encuesta 4.1% (21 respuestas sobre 514 incidentes) en May-2026. Datos de satisfaccion no representativos.</t>
-        </is>
-      </c>
-    </row>
-    <row r="17">
-      <c r="A17" s="3" t="inlineStr">
-        <is>
-          <t>NUEVA</t>
-        </is>
-      </c>
-      <c r="B17" s="3" t="inlineStr">
-        <is>
-          <t>May-2026</t>
-        </is>
-      </c>
-      <c r="C17" s="3" t="inlineStr">
-        <is>
-          <t>Arbolado y Plazas</t>
-        </is>
-      </c>
-      <c r="D17" s="3" t="inlineStr">
-        <is>
-          <t>Muestra encuesta insuficiente</t>
-        </is>
-      </c>
-      <c r="E17" s="3" t="inlineStr">
-        <is>
-          <t>Tasa 3.3%</t>
-        </is>
-      </c>
-      <c r="F17" s="3" t="inlineStr">
-        <is>
-          <t>Tasa de respuesta encuesta 3.3% (4 respuestas sobre 120 incidentes). Datos de satisfaccion no representativos.</t>
-        </is>
-      </c>
-    </row>
-    <row r="18">
-      <c r="A18" s="3" t="inlineStr">
-        <is>
-          <t>NUEVA</t>
-        </is>
-      </c>
-      <c r="B18" s="3" t="inlineStr">
-        <is>
-          <t>May-2026</t>
-        </is>
-      </c>
-      <c r="C18" s="3" t="inlineStr">
-        <is>
-          <t>Transito</t>
-        </is>
-      </c>
-      <c r="D18" s="3" t="inlineStr">
-        <is>
-          <t>Cierre bajo - Vehiculo mal estacionado</t>
-        </is>
-      </c>
-      <c r="E18" s="3" t="inlineStr">
-        <is>
-          <t>22 casos, 0% cierre</t>
-        </is>
-      </c>
-      <c r="F18" s="3" t="inlineStr">
-        <is>
-          <t>Tipo 'Vehiculo mal estacionado': 22 casos en May-2026 que se registran en estado 'Sin asignar' (no se cierran), igual que en abril. Tipo implementado desde marzo 2026. No es demora operativa: revisar con el area si se estan siguiendo los protocolos de implementacion del proceso para tratar este tipo de reclamos.</t>
+          <t>Tipo 'Falta de recolección de residuos reciclables (Programa Día Verde)': 40 casos en Jun-2026 con 22% de cierre (tablero). Cierre muy por debajo del resto del area.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Corrige Stock junio 2026: dias (Calles/global), alerta falsa, muestreo consolidado, Alumbrado sin truncar
</commit_message>
<xml_diff>
--- a/Tablas/Tablas_Stock.xlsx
+++ b/Tablas/Tablas_Stock.xlsx
@@ -31,7 +31,7 @@
       <b val="1"/>
     </font>
   </fonts>
-  <fills count="4">
+  <fills count="6">
     <fill>
       <patternFill/>
     </fill>
@@ -48,6 +48,18 @@
         <fgColor rgb="00FCE4D6"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00E2EFDA"/>
+        <bgColor rgb="00E2EFDA"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00FCE4D6"/>
+        <bgColor rgb="00FCE4D6"/>
+      </patternFill>
+    </fill>
   </fills>
   <borders count="1">
     <border>
@@ -61,11 +73,13 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="4">
+  <cellXfs count="6">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="3" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="4" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="5" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -482,7 +496,7 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>SLA global 38% (-6pp vs mayo). ARBOLADO 76% y CTRL ESPACIO 61% lideran; ALUMBRADO 55%. Mas bajos: RESIDUOS 31% y TRANSITO 38%. Promedio 4 dias para cerrados.</t>
+          <t>SLA global 38% (-6pp vs mayo). ARBOLADO 76% y CTRL ESPACIO 61% lideran; ALUMBRADO 55%. Mas bajos: RESIDUOS 31% y TRANSITO 38%. Promedio 5 dias para cerrados.</t>
         </is>
       </c>
     </row>
@@ -494,7 +508,7 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>Satisfaccion global 70% (+6pp vs mayo). (*) Muestra escasa: en junio se registraron inconvenientes tecnicos en la toma de encuestas, sumado a la maduracion natural de respuestas. Tasa 3.5% (149 resp.), 7 areas &lt;5%. Dato con reserva.</t>
+          <t>Satisfaccion global 70% (+6pp vs mayo). La baja tasa de respuesta (3.5%, 7/7 areas bajo 5%) se debe a la caida de la app que envia la encuesta al cierre del reclamo, mas la maduracion de respuestas. No refleja caida real; dato con reserva.</t>
         </is>
       </c>
     </row>
@@ -536,7 +550,7 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>Cierre 89% sobre 493 incidentes; 'Luminaria superior e inferior apagada du' lidera con 303 casos (88% cierre). Gestion interna 56%.</t>
+          <t>Cierre 89% sobre 493 incidentes; 'Luminaria sup. e inf. apagada de noche' lidera con 303 casos (88% cierre). Gestion interna 56%.</t>
         </is>
       </c>
     </row>
@@ -548,7 +562,7 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>Cierre bajo 40% sobre 124 incidentes; 'Árbol obstruye semáforo/luminaria/cartel' lidera con 46 casos (39% cierre). Sat 50% (muestra insuficiente).</t>
+          <t>Cierre bajo 40% sobre 124 incidentes; 'Arbol obstruye semaforo/luminaria/cartel' lidera con 46 casos (39% cierre). Sat 50% (muestra insuficiente).</t>
         </is>
       </c>
     </row>
@@ -560,7 +574,7 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>Cierre bajo 23% sobre 332 incidentes; 'Bache en calle de asfalto' lidera con 129 casos (24% cierre). Dias prom 9.0 elevado.</t>
+          <t>Cierre bajo 23% sobre 332 incidentes; 'Bache en calle de asfalto' lidera con 129 casos (24% cierre). Sat 62% (muestra insuficiente).</t>
         </is>
       </c>
     </row>
@@ -584,7 +598,7 @@
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>Cierre 75% sobre 263 incidentes; 'Roedores en espacio público' lidera con 97 casos (95% cierre). Sat 40% (muestra insuficiente).</t>
+          <t>Cierre 75% sobre 263 incidentes; 'Roedores en espacio publico' lidera con 97 casos (95% cierre). Sat 40% (muestra insuficiente).</t>
         </is>
       </c>
     </row>
@@ -608,7 +622,7 @@
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>Cierre moderado 67% sobre 512 incidentes; 'Vehículos Abandonados' lidera con 405 casos (75% cierre). Sat 100% (muestra insuficiente).</t>
+          <t>Cierre moderado 67% sobre 512 incidentes; 'Vehiculos Abandonados' lidera con 405 casos (75% cierre). Sat 100% (muestra insuficiente).</t>
         </is>
       </c>
     </row>
@@ -623,7 +637,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F14"/>
+  <dimension ref="A1:F10"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -667,418 +681,290 @@
       </c>
     </row>
     <row r="2">
-      <c r="A2" s="2" t="inlineStr">
+      <c r="A2" s="4" t="inlineStr">
         <is>
           <t>RESUELTA</t>
         </is>
       </c>
-      <c r="B2" s="2" t="inlineStr">
+      <c r="B2" s="4" t="inlineStr">
         <is>
           <t>Feb-2026</t>
         </is>
       </c>
-      <c r="C2" s="2" t="inlineStr">
+      <c r="C2" s="4" t="inlineStr">
         <is>
           <t>Arbolado y Plazas</t>
         </is>
       </c>
-      <c r="D2" s="2" t="inlineStr">
-        <is>
-          <t>% Cancelado &gt;10%</t>
-        </is>
-      </c>
-      <c r="E2" s="2" t="inlineStr">
-        <is>
-          <t>4% (sobre cerrados)</t>
-        </is>
-      </c>
-      <c r="F2" s="2" t="inlineStr">
-        <is>
-          <t>Cancelado baja a 4% de los cerrados en Jun-2026 (donut Cierres por Estado), dentro del rango operativo.</t>
+      <c r="D2" s="4" t="inlineStr">
+        <is>
+          <t>Cancelado alto en cerrados</t>
+        </is>
+      </c>
+      <c r="E2" s="4" t="inlineStr">
+        <is>
+          <t>4%</t>
+        </is>
+      </c>
+      <c r="F2" s="4" t="inlineStr">
+        <is>
+          <t>El cancelado baja a 4% de los cerrados en junio, dentro del rango operativo.</t>
         </is>
       </c>
     </row>
     <row r="3">
-      <c r="A3" s="2" t="inlineStr">
+      <c r="A3" s="4" t="inlineStr">
         <is>
           <t>RESUELTA</t>
         </is>
       </c>
-      <c r="B3" s="2" t="inlineStr">
+      <c r="B3" s="4" t="inlineStr">
+        <is>
+          <t>Abr-2026</t>
+        </is>
+      </c>
+      <c r="C3" s="4" t="inlineStr">
+        <is>
+          <t>Calles y Veredas</t>
+        </is>
+      </c>
+      <c r="D3" s="4" t="inlineStr">
+        <is>
+          <t>Cancelado alto en cerrados</t>
+        </is>
+      </c>
+      <c r="E3" s="4" t="inlineStr">
+        <is>
+          <t>4%</t>
+        </is>
+      </c>
+      <c r="F3" s="4" t="inlineStr">
+        <is>
+          <t>El cancelado baja a 4% de los cerrados en junio, dentro del rango operativo.</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="4" t="inlineStr">
+        <is>
+          <t>RESUELTA</t>
+        </is>
+      </c>
+      <c r="B4" s="4" t="inlineStr">
+        <is>
+          <t>Abr-2026</t>
+        </is>
+      </c>
+      <c r="C4" s="4" t="inlineStr">
+        <is>
+          <t>Control del Espacio Publico</t>
+        </is>
+      </c>
+      <c r="D4" s="4" t="inlineStr">
+        <is>
+          <t>Cancelado alto en cerrados</t>
+        </is>
+      </c>
+      <c r="E4" s="4" t="inlineStr">
+        <is>
+          <t>1%</t>
+        </is>
+      </c>
+      <c r="F4" s="4" t="inlineStr">
+        <is>
+          <t>El cancelado baja a 1% de los cerrados en junio, dentro del rango operativo.</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="4" t="inlineStr">
+        <is>
+          <t>RESUELTA</t>
+        </is>
+      </c>
+      <c r="B5" s="4" t="inlineStr">
+        <is>
+          <t>Feb-2026</t>
+        </is>
+      </c>
+      <c r="C5" s="4" t="inlineStr">
+        <is>
+          <t>Transito</t>
+        </is>
+      </c>
+      <c r="D5" s="4" t="inlineStr">
+        <is>
+          <t>Cancelado excesivo</t>
+        </is>
+      </c>
+      <c r="E5" s="4" t="inlineStr">
+        <is>
+          <t>9%</t>
+        </is>
+      </c>
+      <c r="F5" s="4" t="inlineStr">
+        <is>
+          <t>El cancelado baja a 9% de los cerrados en junio, dentro del rango operativo.</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="4" t="inlineStr">
+        <is>
+          <t>RESUELTA</t>
+        </is>
+      </c>
+      <c r="B6" s="4" t="inlineStr">
         <is>
           <t>May-2026</t>
         </is>
       </c>
-      <c r="C3" s="2" t="inlineStr">
+      <c r="C6" s="4" t="inlineStr">
+        <is>
+          <t>Transito</t>
+        </is>
+      </c>
+      <c r="D6" s="4" t="inlineStr">
+        <is>
+          <t>Cierre bajo en Vehiculo mal estacionado</t>
+        </is>
+      </c>
+      <c r="E6" s="4" t="inlineStr">
+        <is>
+          <t>67%</t>
+        </is>
+      </c>
+      <c r="F6" s="4" t="inlineStr">
+        <is>
+          <t>El cierre del tipo sube de 0% a 67% entre mayo y junio.</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="5" t="inlineStr">
+        <is>
+          <t>PERSISTE</t>
+        </is>
+      </c>
+      <c r="B7" s="5" t="inlineStr">
+        <is>
+          <t>Mar-2026</t>
+        </is>
+      </c>
+      <c r="C7" s="5" t="inlineStr">
+        <is>
+          <t>Calles y Veredas</t>
+        </is>
+      </c>
+      <c r="D7" s="5" t="inlineStr">
+        <is>
+          <t>Cierre colapsado</t>
+        </is>
+      </c>
+      <c r="E7" s="5" t="inlineStr">
+        <is>
+          <t>15% a 23%</t>
+        </is>
+      </c>
+      <c r="F7" s="5" t="inlineStr">
+        <is>
+          <t>El cierre del area sube de 15% a 23% entre mayo y junio; se mantiene en zona critica.</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="5" t="inlineStr">
+        <is>
+          <t>NUEVA</t>
+        </is>
+      </c>
+      <c r="B8" s="5" t="inlineStr">
+        <is>
+          <t>Jun-2026</t>
+        </is>
+      </c>
+      <c r="C8" s="5" t="inlineStr">
         <is>
           <t>Arbolado y Plazas</t>
         </is>
       </c>
-      <c r="D3" s="2" t="inlineStr">
-        <is>
-          <t>Muestra encuesta insuficiente</t>
-        </is>
-      </c>
-      <c r="E3" s="2" t="inlineStr">
-        <is>
-          <t>consolidada</t>
-        </is>
-      </c>
-      <c r="F3" s="2" t="inlineStr">
-        <is>
-          <t>Alerta de muestra por area consolidada en la alerta global de tasa de respuesta de encuesta (Jun-2026).</t>
-        </is>
-      </c>
-    </row>
-    <row r="4">
-      <c r="A4" s="2" t="inlineStr">
-        <is>
-          <t>RESUELTA</t>
-        </is>
-      </c>
-      <c r="B4" s="2" t="inlineStr">
-        <is>
-          <t>Abr-2026</t>
-        </is>
-      </c>
-      <c r="C4" s="2" t="inlineStr">
-        <is>
-          <t>Calles y Veredas</t>
-        </is>
-      </c>
-      <c r="D4" s="2" t="inlineStr">
-        <is>
-          <t>Cancelado alto en cerrados</t>
-        </is>
-      </c>
-      <c r="E4" s="2" t="inlineStr">
-        <is>
-          <t>4% (sobre cerrados)</t>
-        </is>
-      </c>
-      <c r="F4" s="2" t="inlineStr">
-        <is>
-          <t>Cancelado baja a 4% de los cerrados en Jun-2026 (donut Cierres por Estado), dentro del rango operativo.</t>
-        </is>
-      </c>
-    </row>
-    <row r="5">
-      <c r="A5" s="2" t="inlineStr">
-        <is>
-          <t>RESUELTA</t>
-        </is>
-      </c>
-      <c r="B5" s="2" t="inlineStr">
-        <is>
-          <t>Abr-2026</t>
-        </is>
-      </c>
-      <c r="C5" s="2" t="inlineStr">
-        <is>
-          <t>Calles y Veredas</t>
-        </is>
-      </c>
-      <c r="D5" s="2" t="inlineStr">
-        <is>
-          <t>Muestra encuesta insuficiente</t>
-        </is>
-      </c>
-      <c r="E5" s="2" t="inlineStr">
-        <is>
-          <t>consolidada</t>
-        </is>
-      </c>
-      <c r="F5" s="2" t="inlineStr">
-        <is>
-          <t>Alerta de muestra por area consolidada en la alerta global de tasa de respuesta de encuesta (Jun-2026).</t>
-        </is>
-      </c>
-    </row>
-    <row r="6">
-      <c r="A6" s="2" t="inlineStr">
-        <is>
-          <t>RESUELTA</t>
-        </is>
-      </c>
-      <c r="B6" s="2" t="inlineStr">
-        <is>
-          <t>Abr-2026</t>
-        </is>
-      </c>
-      <c r="C6" s="2" t="inlineStr">
-        <is>
-          <t>Control del Espacio Publico</t>
-        </is>
-      </c>
-      <c r="D6" s="2" t="inlineStr">
-        <is>
-          <t>Cancelado alto en cerrados</t>
-        </is>
-      </c>
-      <c r="E6" s="2" t="inlineStr">
-        <is>
-          <t>1% (sobre cerrados)</t>
-        </is>
-      </c>
-      <c r="F6" s="2" t="inlineStr">
-        <is>
-          <t>Cancelado baja a 1% de los cerrados en Jun-2026 (donut Cierres por Estado), dentro del rango operativo.</t>
-        </is>
-      </c>
-    </row>
-    <row r="7">
-      <c r="A7" s="2" t="inlineStr">
-        <is>
-          <t>RESUELTA</t>
-        </is>
-      </c>
-      <c r="B7" s="2" t="inlineStr">
-        <is>
-          <t>Feb-2026</t>
-        </is>
-      </c>
-      <c r="C7" s="2" t="inlineStr">
-        <is>
-          <t>Transito</t>
-        </is>
-      </c>
-      <c r="D7" s="2" t="inlineStr">
-        <is>
-          <t>% Cancelado excesivo</t>
-        </is>
-      </c>
-      <c r="E7" s="2" t="inlineStr">
-        <is>
-          <t>9% (sobre cerrados)</t>
-        </is>
-      </c>
-      <c r="F7" s="2" t="inlineStr">
-        <is>
-          <t>Cancelado baja a 9% de los cerrados en Jun-2026 (donut Cierres por Estado), dentro del rango operativo.</t>
-        </is>
-      </c>
-    </row>
-    <row r="8">
-      <c r="A8" s="2" t="inlineStr">
-        <is>
-          <t>RESUELTA</t>
-        </is>
-      </c>
-      <c r="B8" s="2" t="inlineStr">
-        <is>
-          <t>Abr-2026</t>
-        </is>
-      </c>
-      <c r="C8" s="2" t="inlineStr">
-        <is>
-          <t>Transito</t>
-        </is>
-      </c>
-      <c r="D8" s="2" t="inlineStr">
-        <is>
-          <t>Muestra encuesta insuficiente</t>
-        </is>
-      </c>
-      <c r="E8" s="2" t="inlineStr">
-        <is>
-          <t>consolidada</t>
-        </is>
-      </c>
-      <c r="F8" s="2" t="inlineStr">
-        <is>
-          <t>Alerta de muestra por area consolidada en la alerta global de tasa de respuesta de encuesta (Jun-2026).</t>
+      <c r="D8" s="5" t="inlineStr">
+        <is>
+          <t>Cierre bajo del area</t>
+        </is>
+      </c>
+      <c r="E8" s="5" t="inlineStr">
+        <is>
+          <t>40%</t>
+        </is>
+      </c>
+      <c r="F8" s="5" t="inlineStr">
+        <is>
+          <t>El cierre del area se ubica en 40% en junio, el mas bajo despues de Calles y Veredas.</t>
         </is>
       </c>
     </row>
     <row r="9">
-      <c r="A9" s="2" t="inlineStr">
-        <is>
-          <t>RESUELTA</t>
-        </is>
-      </c>
-      <c r="B9" s="2" t="inlineStr">
-        <is>
-          <t>May-2026</t>
-        </is>
-      </c>
-      <c r="C9" s="2" t="inlineStr">
-        <is>
-          <t>Transito</t>
-        </is>
-      </c>
-      <c r="D9" s="2" t="inlineStr">
-        <is>
-          <t>Cierre bajo - Vehiculo mal estacionado</t>
-        </is>
-      </c>
-      <c r="E9" s="2" t="inlineStr">
-        <is>
-          <t>67%</t>
-        </is>
-      </c>
-      <c r="F9" s="2" t="inlineStr">
-        <is>
-          <t>Cierre del area sube de 0% a 67% (May-2026 a Jun-2026). Recuperacion significativa.</t>
+      <c r="A9" s="5" t="inlineStr">
+        <is>
+          <t>NUEVA</t>
+        </is>
+      </c>
+      <c r="B9" s="5" t="inlineStr">
+        <is>
+          <t>Jun-2026</t>
+        </is>
+      </c>
+      <c r="C9" s="5" t="inlineStr">
+        <is>
+          <t>GENERAL</t>
+        </is>
+      </c>
+      <c r="D9" s="5" t="inlineStr">
+        <is>
+          <t>Muestra de encuesta insuficiente (municipio)</t>
+        </is>
+      </c>
+      <c r="E9" s="5" t="inlineStr">
+        <is>
+          <t>Tasa 3.5%</t>
+        </is>
+      </c>
+      <c r="F9" s="5" t="inlineStr">
+        <is>
+          <t>La tasa de respuesta de encuesta de junio es 3.5%, con 149 respuestas sobre 4309 incidentes, y las 7 areas del monitor quedan por debajo del 5%. La causa principal es una caida de la aplicacion que envia la encuesta al cierre de cada reclamo, por lo que a muchos vecinos no se les envio la encuesta; a esto se suma la maduracion natural de las respuestas, que al corte aun no se habian acumulado. No refleja una caida real de la satisfaccion. Por eso la satisfaccion por area se publica con la marca (muestra insuficiente) y con reserva.</t>
         </is>
       </c>
     </row>
     <row r="10">
-      <c r="A10" s="3" t="inlineStr">
-        <is>
-          <t>PERSISTE</t>
-        </is>
-      </c>
-      <c r="B10" s="3" t="inlineStr">
-        <is>
-          <t>Mar-2026</t>
-        </is>
-      </c>
-      <c r="C10" s="3" t="inlineStr">
-        <is>
-          <t>Calles y Veredas</t>
-        </is>
-      </c>
-      <c r="D10" s="3" t="inlineStr">
-        <is>
-          <t>Cierre colapsado</t>
-        </is>
-      </c>
-      <c r="E10" s="3" t="inlineStr">
-        <is>
-          <t>15%-&gt;23%</t>
-        </is>
-      </c>
-      <c r="F10" s="3" t="inlineStr">
-        <is>
-          <t>Cierre del area 15%-&gt;23% (May-2026 a Jun-2026). Sigue en zona critica. Cancelado 4% sobre cerrados.</t>
-        </is>
-      </c>
-    </row>
-    <row r="11">
-      <c r="A11" s="3" t="inlineStr">
+      <c r="A10" s="5" t="inlineStr">
         <is>
           <t>NUEVA</t>
         </is>
       </c>
-      <c r="B11" s="3" t="inlineStr">
+      <c r="B10" s="5" t="inlineStr">
         <is>
           <t>Jun-2026</t>
         </is>
       </c>
-      <c r="C11" s="3" t="inlineStr">
-        <is>
-          <t>Arbolado y Plazas</t>
-        </is>
-      </c>
-      <c r="D11" s="3" t="inlineStr">
-        <is>
-          <t>Cierre bajo (area)</t>
-        </is>
-      </c>
-      <c r="E11" s="3" t="inlineStr">
-        <is>
-          <t>40%</t>
-        </is>
-      </c>
-      <c r="F11" s="3" t="inlineStr">
-        <is>
-          <t>Cierre del area 40% en Jun-2026 (tablero). Cancelado 4% sobre cerrados.</t>
-        </is>
-      </c>
-    </row>
-    <row r="12">
-      <c r="A12" s="3" t="inlineStr">
-        <is>
-          <t>NUEVA</t>
-        </is>
-      </c>
-      <c r="B12" s="3" t="inlineStr">
-        <is>
-          <t>Jun-2026</t>
-        </is>
-      </c>
-      <c r="C12" s="3" t="inlineStr">
-        <is>
-          <t>Calles y Veredas</t>
-        </is>
-      </c>
-      <c r="D12" s="3" t="inlineStr">
-        <is>
-          <t>Dias promedio alto</t>
-        </is>
-      </c>
-      <c r="E12" s="3" t="inlineStr">
-        <is>
-          <t>9 dias</t>
-        </is>
-      </c>
-      <c r="F12" s="3" t="inlineStr">
-        <is>
-          <t>Tiempo promedio de resolucion 9 dias en Jun-2026 (tablero). Por encima del tiempo habitual.</t>
-        </is>
-      </c>
-    </row>
-    <row r="13">
-      <c r="A13" s="3" t="inlineStr">
-        <is>
-          <t>NUEVA</t>
-        </is>
-      </c>
-      <c r="B13" s="3" t="inlineStr">
-        <is>
-          <t>Jun-2026</t>
-        </is>
-      </c>
-      <c r="C13" s="3" t="inlineStr">
-        <is>
-          <t>GENERAL</t>
-        </is>
-      </c>
-      <c r="D13" s="3" t="inlineStr">
-        <is>
-          <t>Muestra de encuesta insuficiente (municipio)</t>
-        </is>
-      </c>
-      <c r="E13" s="3" t="inlineStr">
-        <is>
-          <t>Tasa 3.5% (7/7 areas &lt;5%)</t>
-        </is>
-      </c>
-      <c r="F13" s="3" t="inlineStr">
-        <is>
-          <t>Tasa de respuesta de encuesta 3.5% en Jun-2026 (149 respuestas sobre 4309 incidentes); las 7 areas del monitor quedan por debajo del 5%. Dos causas: inconvenientes tecnicos en la toma de encuestas durante Jun-2026 y la maduracion natural de las respuestas (las cargadas en Jun-2026 aun no se acumularon al corte). No refleja caida de satisfaccion. La satisfaccion por area se publica con la marca '(muestra insuficiente)'.</t>
-        </is>
-      </c>
-    </row>
-    <row r="14">
-      <c r="A14" s="3" t="inlineStr">
-        <is>
-          <t>NUEVA</t>
-        </is>
-      </c>
-      <c r="B14" s="3" t="inlineStr">
-        <is>
-          <t>Jun-2026</t>
-        </is>
-      </c>
-      <c r="C14" s="3" t="inlineStr">
+      <c r="C10" s="5" t="inlineStr">
         <is>
           <t>Residuos y Limpieza</t>
         </is>
       </c>
-      <c r="D14" s="3" t="inlineStr">
-        <is>
-          <t>Cierre bajo - Falta de recolección de residuos reciclables (Pr</t>
-        </is>
-      </c>
-      <c r="E14" s="3" t="inlineStr">
-        <is>
-          <t>22% (40 casos)</t>
-        </is>
-      </c>
-      <c r="F14" s="3" t="inlineStr">
-        <is>
-          <t>Tipo 'Falta de recolección de residuos reciclables (Programa Día Verde)': 40 casos en Jun-2026 con 22% de cierre (tablero). Cierre muy por debajo del resto del area.</t>
+      <c r="D10" s="5" t="inlineStr">
+        <is>
+          <t>Cierre bajo en Falta de recoleccion de residuos reciclables</t>
+        </is>
+      </c>
+      <c r="E10" s="5" t="inlineStr">
+        <is>
+          <t>22%</t>
+        </is>
+      </c>
+      <c r="F10" s="5" t="inlineStr">
+        <is>
+          <t>El tipo del Programa Dia Verde tiene 40 casos con 22% de cierre en junio, muy por debajo del resto del area.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Tablas_Stock vigente v2 - Jul-2026
</commit_message>
<xml_diff>
--- a/Tablas/Tablas_Stock.xlsx
+++ b/Tablas/Tablas_Stock.xlsx
@@ -31,7 +31,7 @@
       <b val="1"/>
     </font>
   </fonts>
-  <fills count="6">
+  <fills count="4">
     <fill>
       <patternFill/>
     </fill>
@@ -48,18 +48,6 @@
         <fgColor rgb="00FCE4D6"/>
       </patternFill>
     </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="00E2EFDA"/>
-        <bgColor rgb="00E2EFDA"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="00FCE4D6"/>
-        <bgColor rgb="00FCE4D6"/>
-      </patternFill>
-    </fill>
   </fills>
   <borders count="1">
     <border>
@@ -73,13 +61,11 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="6">
+  <cellXfs count="4">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="3" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="0" fillId="4" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="0" fillId="5" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -472,7 +458,7 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>Total 4309 incidentes en junio (-5% vs mayo, 4555). RESIDUOS Y LIMPIEZA concentra 57% del volumen (2457 casos, -9%). Subas: CTRL ACTIVIDADES +45%, CALLES +15%; baja CTRL ESPACIO -24%.</t>
+          <t>Total 2947 incidentes en julio (-31% vs junio, 4311). Caida generalizada: ARBOLADO -61%, CTRL ACTIVIDADES -47%, RESIDUOS -41% (1450 casos, 49% del volumen). Unica suba: CTRL ESPACIO +6%.</t>
         </is>
       </c>
     </row>
@@ -484,7 +470,7 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>Cierre global 79% (+5pp vs mayo). ALUMBRADO 89%, RESIDUOS 89% y CTRL ACTIVIDADES 86% lideran. Criticos: CALLES 23% y ARBOLADO 40%. Cancelado sobre cerrados bajo en todas las areas (max TRANSITO 9%).</t>
+          <t>Cierre global 76% (-3pp vs junio). RESIDUOS 88%, ALUMBRADO 81% y CTRL ACTIVIDADES 78% lideran; ARBOLADO recupera a 60%. Critico: CALLES 13%, quinto mes en zona critica. Cancelado sobre cerrados: CALLES 35% y TRANSITO 11%; resto &lt;=4%.</t>
         </is>
       </c>
     </row>
@@ -496,7 +482,7 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>SLA global 38% (-6pp vs mayo). ARBOLADO 76% y CTRL ESPACIO 61% lideran; ALUMBRADO 55%. Mas bajos: RESIDUOS 31% y TRANSITO 38%. Promedio 5 dias para cerrados.</t>
+          <t>SLA global 44% (+6pp vs junio). ALUMBRADO 61% lidera; CALLES y CTRL ACTIVIDADES 54%. Mas bajos: TRANSITO 31% y CTRL ESPACIO 39%. Promedio 6 dias para cerrados; ARBOLADO sube a 9 dias.</t>
         </is>
       </c>
     </row>
@@ -508,7 +494,7 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>Satisfaccion global 70% (+6pp vs mayo). La baja tasa de respuesta (3.5%, 7/7 areas bajo 5%) se debe a la caida de la app que envia la encuesta al cierre del reclamo, mas la maduracion de respuestas. No refleja caida real; dato con reserva.</t>
+          <t>Satisfaccion global 67% (-3pp vs junio). Encuesta normalizada: 476 respuestas, tasa 16.2% del total (21% s/incidentes con email). RESIDUOS 73% y ALUMBRADO 62%; CTRL ACTIVIDADES 10%. CALLES y TRANSITO con muestra insuficiente.</t>
         </is>
       </c>
     </row>
@@ -550,7 +536,7 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>Cierre 89% sobre 493 incidentes; 'Luminaria sup. e inf. apagada de noche' lidera con 303 casos (88% cierre). Gestion interna 56%.</t>
+          <t>Cierre 81% sobre 401 incidentes; 'Luminaria superior e inferior apagada du' lidera con 262 casos (82% cierre). Gestion interna 56%.</t>
         </is>
       </c>
     </row>
@@ -562,7 +548,7 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>Cierre bajo 40% sobre 124 incidentes; 'Arbol obstruye semaforo/luminaria/cartel' lidera con 46 casos (39% cierre). Sat 50% (muestra insuficiente).</t>
+          <t>Cierre moderado 60% sobre 47 incidentes; 'Inconvenientes con intervenciones de arb' lidera con 19 casos (84% cierre). Dias prom 9.0 elevado.</t>
         </is>
       </c>
     </row>
@@ -574,7 +560,7 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>Cierre bajo 23% sobre 332 incidentes; 'Bache en calle de asfalto' lidera con 129 casos (24% cierre). Sat 62% (muestra insuficiente).</t>
+          <t>Cierre critico 13% sobre 295 incidentes; 'Bache en calle de asfalto' lidera con 109 casos (10% cierre). Sat 50% (muestra insuficiente).</t>
         </is>
       </c>
     </row>
@@ -586,7 +572,7 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>Cierre 86% sobre 128 incidentes; 'Otros ruidos molestos' lidera con 54 casos (87% cierre). Sat 20% (muestra insuficiente).</t>
+          <t>Cierre 78% sobre 67 incidentes; 'Falta de Habilitación - Actividad no dec' lidera con 22 casos (82% cierre). SLA 54%, sat 10%.</t>
         </is>
       </c>
     </row>
@@ -598,7 +584,7 @@
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>Cierre 75% sobre 263 incidentes; 'Roedores en espacio publico' lidera con 97 casos (95% cierre). Sat 40% (muestra insuficiente).</t>
+          <t>Cierre 74% sobre 262 incidentes; 'Cable cortado' lidera con 115 casos (71% cierre). SLA 39%, sat 56%.</t>
         </is>
       </c>
     </row>
@@ -610,7 +596,7 @@
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>Cierre 89% sobre 2457 incidentes; 'Falta de barrido o barrido deficiente' lidera con 930 casos (92% cierre). Sat 72% (muestra insuficiente).</t>
+          <t>Cierre 88% sobre 1450 incidentes; 'Retiro de escombros y/o restos de obra' lidera con 437 casos (90% cierre). SLA 43%, sat 73%.</t>
         </is>
       </c>
     </row>
@@ -622,7 +608,7 @@
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>Cierre moderado 67% sobre 512 incidentes; 'Vehiculos Abandonados' lidera con 405 casos (75% cierre). Sat 100% (muestra insuficiente).</t>
+          <t>Cierre 75% sobre 425 incidentes; 'Vehículos Abandonados' lidera con 333 casos (81% cierre). Sat 56% (muestra insuficiente).</t>
         </is>
       </c>
     </row>
@@ -637,7 +623,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F10"/>
+  <dimension ref="A1:F9"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -681,290 +667,258 @@
       </c>
     </row>
     <row r="2">
-      <c r="A2" s="4" t="inlineStr">
+      <c r="A2" s="2" t="inlineStr">
         <is>
           <t>RESUELTA</t>
         </is>
       </c>
-      <c r="B2" s="4" t="inlineStr">
-        <is>
-          <t>Feb-2026</t>
-        </is>
-      </c>
-      <c r="C2" s="4" t="inlineStr">
+      <c r="B2" s="2" t="inlineStr">
+        <is>
+          <t>Jun-2026</t>
+        </is>
+      </c>
+      <c r="C2" s="2" t="inlineStr">
         <is>
           <t>Arbolado y Plazas</t>
         </is>
       </c>
-      <c r="D2" s="4" t="inlineStr">
+      <c r="D2" s="2" t="inlineStr">
+        <is>
+          <t>Cierre bajo del area</t>
+        </is>
+      </c>
+      <c r="E2" s="2" t="inlineStr">
+        <is>
+          <t>40%-&gt;60%</t>
+        </is>
+      </c>
+      <c r="F2" s="2" t="inlineStr">
+        <is>
+          <t>Cierre del area sube de 40% a 60% (Jun-2026 a Jul-2026). Recuperacion significativa.</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="2" t="inlineStr">
+        <is>
+          <t>RESUELTA</t>
+        </is>
+      </c>
+      <c r="B3" s="2" t="inlineStr">
+        <is>
+          <t>Jun-2026</t>
+        </is>
+      </c>
+      <c r="C3" s="2" t="inlineStr">
+        <is>
+          <t>GENERAL</t>
+        </is>
+      </c>
+      <c r="D3" s="2" t="inlineStr">
+        <is>
+          <t>Muestra de encuesta insuficiente (municipio)</t>
+        </is>
+      </c>
+      <c r="E3" s="2" t="inlineStr">
+        <is>
+          <t>Tasa 16.2% (476 resp.)</t>
+        </is>
+      </c>
+      <c r="F3" s="2" t="inlineStr">
+        <is>
+          <t>La tasa de respuesta de encuesta se recupera en julio: 476 respuestas sobre 2947 incidentes (16.2% del total; 21% sobre incidentes con email segun tablero), tras los inconvenientes tecnicos de junio. Solo Calles y Veredas (2.7%) y Transito (2.1%) permanecen debajo del 5%; su satisfaccion se publica con la marca (muestra insuficiente).</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="2" t="inlineStr">
+        <is>
+          <t>RESUELTA</t>
+        </is>
+      </c>
+      <c r="B4" s="2" t="inlineStr">
+        <is>
+          <t>Jun-2026</t>
+        </is>
+      </c>
+      <c r="C4" s="2" t="inlineStr">
+        <is>
+          <t>Residuos y Limpieza</t>
+        </is>
+      </c>
+      <c r="D4" s="2" t="inlineStr">
+        <is>
+          <t>Cierre bajo en Falta de recoleccion de residuos reciclables</t>
+        </is>
+      </c>
+      <c r="E4" s="2" t="inlineStr">
+        <is>
+          <t>37 casos, 100% cierre</t>
+        </is>
+      </c>
+      <c r="F4" s="2" t="inlineStr">
+        <is>
+          <t>Cierre bajo en Falta de recoleccion de residuos reciclables: 37 casos, cierre 22%-&gt;100% (Jun-2026 a Jul-2026). Recuperacion del cierre.</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="3" t="inlineStr">
+        <is>
+          <t>PERSISTE</t>
+        </is>
+      </c>
+      <c r="B5" s="3" t="inlineStr">
+        <is>
+          <t>Mar-2026</t>
+        </is>
+      </c>
+      <c r="C5" s="3" t="inlineStr">
+        <is>
+          <t>Calles y Veredas</t>
+        </is>
+      </c>
+      <c r="D5" s="3" t="inlineStr">
+        <is>
+          <t>Cierre colapsado</t>
+        </is>
+      </c>
+      <c r="E5" s="3" t="inlineStr">
+        <is>
+          <t>23%-&gt;13%</t>
+        </is>
+      </c>
+      <c r="F5" s="3" t="inlineStr">
+        <is>
+          <t>Cierre del area 23%-&gt;13% (Jun-2026 a Jul-2026). Sigue en zona critica. Cancelado 35% sobre cerrados.</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="3" t="inlineStr">
+        <is>
+          <t>NUEVA</t>
+        </is>
+      </c>
+      <c r="B6" s="3" t="inlineStr">
+        <is>
+          <t>Jul-2026</t>
+        </is>
+      </c>
+      <c r="C6" s="3" t="inlineStr">
+        <is>
+          <t>Arbolado y Plazas</t>
+        </is>
+      </c>
+      <c r="D6" s="3" t="inlineStr">
+        <is>
+          <t>Dias promedio alto</t>
+        </is>
+      </c>
+      <c r="E6" s="3" t="inlineStr">
+        <is>
+          <t>9 dias</t>
+        </is>
+      </c>
+      <c r="F6" s="3" t="inlineStr">
+        <is>
+          <t>Tiempo promedio de resolucion 9 dias en Jul-2026 (tablero). Por encima del tiempo habitual.</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="3" t="inlineStr">
+        <is>
+          <t>NUEVA</t>
+        </is>
+      </c>
+      <c r="B7" s="3" t="inlineStr">
+        <is>
+          <t>Jul-2026</t>
+        </is>
+      </c>
+      <c r="C7" s="3" t="inlineStr">
+        <is>
+          <t>Calles y Veredas</t>
+        </is>
+      </c>
+      <c r="D7" s="3" t="inlineStr">
         <is>
           <t>Cancelado alto en cerrados</t>
         </is>
       </c>
-      <c r="E2" s="4" t="inlineStr">
-        <is>
-          <t>4%</t>
-        </is>
-      </c>
-      <c r="F2" s="4" t="inlineStr">
-        <is>
-          <t>El cancelado baja a 4% de los cerrados en junio, dentro del rango operativo.</t>
-        </is>
-      </c>
-    </row>
-    <row r="3">
-      <c r="A3" s="4" t="inlineStr">
-        <is>
-          <t>RESUELTA</t>
-        </is>
-      </c>
-      <c r="B3" s="4" t="inlineStr">
-        <is>
-          <t>Abr-2026</t>
-        </is>
-      </c>
-      <c r="C3" s="4" t="inlineStr">
-        <is>
-          <t>Calles y Veredas</t>
-        </is>
-      </c>
-      <c r="D3" s="4" t="inlineStr">
+      <c r="E7" s="3" t="inlineStr">
+        <is>
+          <t>35% (sobre cerrados)</t>
+        </is>
+      </c>
+      <c r="F7" s="3" t="inlineStr">
+        <is>
+          <t>35% de los cerrados son Cancelados en Jul-2026 (donut Cierres por Estado). Revisar calidad de cierre.</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="3" t="inlineStr">
+        <is>
+          <t>NUEVA</t>
+        </is>
+      </c>
+      <c r="B8" s="3" t="inlineStr">
+        <is>
+          <t>Jul-2026</t>
+        </is>
+      </c>
+      <c r="C8" s="3" t="inlineStr">
+        <is>
+          <t>Control de Actividades Comerciales</t>
+        </is>
+      </c>
+      <c r="D8" s="3" t="inlineStr">
+        <is>
+          <t>Brecha cierre-satisfaccion</t>
+        </is>
+      </c>
+      <c r="E8" s="3" t="inlineStr">
+        <is>
+          <t>Cierre 78% / Sat 10%</t>
+        </is>
+      </c>
+      <c r="F8" s="3" t="inlineStr">
+        <is>
+          <t>Cierre 78% con satisfaccion 10%. Vecinos no perciben resolucion efectiva.</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="3" t="inlineStr">
+        <is>
+          <t>NUEVA</t>
+        </is>
+      </c>
+      <c r="B9" s="3" t="inlineStr">
+        <is>
+          <t>Jul-2026</t>
+        </is>
+      </c>
+      <c r="C9" s="3" t="inlineStr">
+        <is>
+          <t>Transito</t>
+        </is>
+      </c>
+      <c r="D9" s="3" t="inlineStr">
         <is>
           <t>Cancelado alto en cerrados</t>
         </is>
       </c>
-      <c r="E3" s="4" t="inlineStr">
-        <is>
-          <t>4%</t>
-        </is>
-      </c>
-      <c r="F3" s="4" t="inlineStr">
-        <is>
-          <t>El cancelado baja a 4% de los cerrados en junio, dentro del rango operativo.</t>
-        </is>
-      </c>
-    </row>
-    <row r="4">
-      <c r="A4" s="4" t="inlineStr">
-        <is>
-          <t>RESUELTA</t>
-        </is>
-      </c>
-      <c r="B4" s="4" t="inlineStr">
-        <is>
-          <t>Abr-2026</t>
-        </is>
-      </c>
-      <c r="C4" s="4" t="inlineStr">
-        <is>
-          <t>Control del Espacio Publico</t>
-        </is>
-      </c>
-      <c r="D4" s="4" t="inlineStr">
-        <is>
-          <t>Cancelado alto en cerrados</t>
-        </is>
-      </c>
-      <c r="E4" s="4" t="inlineStr">
-        <is>
-          <t>1%</t>
-        </is>
-      </c>
-      <c r="F4" s="4" t="inlineStr">
-        <is>
-          <t>El cancelado baja a 1% de los cerrados en junio, dentro del rango operativo.</t>
-        </is>
-      </c>
-    </row>
-    <row r="5">
-      <c r="A5" s="4" t="inlineStr">
-        <is>
-          <t>RESUELTA</t>
-        </is>
-      </c>
-      <c r="B5" s="4" t="inlineStr">
-        <is>
-          <t>Feb-2026</t>
-        </is>
-      </c>
-      <c r="C5" s="4" t="inlineStr">
-        <is>
-          <t>Transito</t>
-        </is>
-      </c>
-      <c r="D5" s="4" t="inlineStr">
-        <is>
-          <t>Cancelado excesivo</t>
-        </is>
-      </c>
-      <c r="E5" s="4" t="inlineStr">
-        <is>
-          <t>9%</t>
-        </is>
-      </c>
-      <c r="F5" s="4" t="inlineStr">
-        <is>
-          <t>El cancelado baja a 9% de los cerrados en junio, dentro del rango operativo.</t>
-        </is>
-      </c>
-    </row>
-    <row r="6">
-      <c r="A6" s="4" t="inlineStr">
-        <is>
-          <t>RESUELTA</t>
-        </is>
-      </c>
-      <c r="B6" s="4" t="inlineStr">
-        <is>
-          <t>May-2026</t>
-        </is>
-      </c>
-      <c r="C6" s="4" t="inlineStr">
-        <is>
-          <t>Transito</t>
-        </is>
-      </c>
-      <c r="D6" s="4" t="inlineStr">
-        <is>
-          <t>Cierre bajo en Vehiculo mal estacionado</t>
-        </is>
-      </c>
-      <c r="E6" s="4" t="inlineStr">
-        <is>
-          <t>67%</t>
-        </is>
-      </c>
-      <c r="F6" s="4" t="inlineStr">
-        <is>
-          <t>El cierre del tipo sube de 0% a 67% entre mayo y junio.</t>
-        </is>
-      </c>
-    </row>
-    <row r="7">
-      <c r="A7" s="5" t="inlineStr">
-        <is>
-          <t>PERSISTE</t>
-        </is>
-      </c>
-      <c r="B7" s="5" t="inlineStr">
-        <is>
-          <t>Mar-2026</t>
-        </is>
-      </c>
-      <c r="C7" s="5" t="inlineStr">
-        <is>
-          <t>Calles y Veredas</t>
-        </is>
-      </c>
-      <c r="D7" s="5" t="inlineStr">
-        <is>
-          <t>Cierre colapsado</t>
-        </is>
-      </c>
-      <c r="E7" s="5" t="inlineStr">
-        <is>
-          <t>15% a 23%</t>
-        </is>
-      </c>
-      <c r="F7" s="5" t="inlineStr">
-        <is>
-          <t>El cierre del area sube de 15% a 23% entre mayo y junio; se mantiene en zona critica.</t>
-        </is>
-      </c>
-    </row>
-    <row r="8">
-      <c r="A8" s="5" t="inlineStr">
-        <is>
-          <t>NUEVA</t>
-        </is>
-      </c>
-      <c r="B8" s="5" t="inlineStr">
-        <is>
-          <t>Jun-2026</t>
-        </is>
-      </c>
-      <c r="C8" s="5" t="inlineStr">
-        <is>
-          <t>Arbolado y Plazas</t>
-        </is>
-      </c>
-      <c r="D8" s="5" t="inlineStr">
-        <is>
-          <t>Cierre bajo del area</t>
-        </is>
-      </c>
-      <c r="E8" s="5" t="inlineStr">
-        <is>
-          <t>40%</t>
-        </is>
-      </c>
-      <c r="F8" s="5" t="inlineStr">
-        <is>
-          <t>El cierre del area se ubica en 40% en junio, el mas bajo despues de Calles y Veredas.</t>
-        </is>
-      </c>
-    </row>
-    <row r="9">
-      <c r="A9" s="5" t="inlineStr">
-        <is>
-          <t>NUEVA</t>
-        </is>
-      </c>
-      <c r="B9" s="5" t="inlineStr">
-        <is>
-          <t>Jun-2026</t>
-        </is>
-      </c>
-      <c r="C9" s="5" t="inlineStr">
-        <is>
-          <t>GENERAL</t>
-        </is>
-      </c>
-      <c r="D9" s="5" t="inlineStr">
-        <is>
-          <t>Muestra de encuesta insuficiente (municipio)</t>
-        </is>
-      </c>
-      <c r="E9" s="5" t="inlineStr">
-        <is>
-          <t>Tasa 3.5%</t>
-        </is>
-      </c>
-      <c r="F9" s="5" t="inlineStr">
-        <is>
-          <t>La tasa de respuesta de encuesta de junio es 3.5%, con 149 respuestas sobre 4309 incidentes, y las 7 areas del monitor quedan por debajo del 5%. La causa principal es una caida de la aplicacion que envia la encuesta al cierre de cada reclamo, por lo que a muchos vecinos no se les envio la encuesta; a esto se suma la maduracion natural de las respuestas, que al corte aun no se habian acumulado. No refleja una caida real de la satisfaccion. Por eso la satisfaccion por area se publica con la marca (muestra insuficiente) y con reserva.</t>
-        </is>
-      </c>
-    </row>
-    <row r="10">
-      <c r="A10" s="5" t="inlineStr">
-        <is>
-          <t>NUEVA</t>
-        </is>
-      </c>
-      <c r="B10" s="5" t="inlineStr">
-        <is>
-          <t>Jun-2026</t>
-        </is>
-      </c>
-      <c r="C10" s="5" t="inlineStr">
-        <is>
-          <t>Residuos y Limpieza</t>
-        </is>
-      </c>
-      <c r="D10" s="5" t="inlineStr">
-        <is>
-          <t>Cierre bajo en Falta de recoleccion de residuos reciclables</t>
-        </is>
-      </c>
-      <c r="E10" s="5" t="inlineStr">
-        <is>
-          <t>22%</t>
-        </is>
-      </c>
-      <c r="F10" s="5" t="inlineStr">
-        <is>
-          <t>El tipo del Programa Dia Verde tiene 40 casos con 22% de cierre en junio, muy por debajo del resto del area.</t>
+      <c r="E9" s="3" t="inlineStr">
+        <is>
+          <t>11% (sobre cerrados)</t>
+        </is>
+      </c>
+      <c r="F9" s="3" t="inlineStr">
+        <is>
+          <t>11% de los cerrados son Cancelados en Jul-2026 (donut Cierres por Estado). Revisar calidad de cierre.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Tablas_Stock vigente v2 - Ago-2026
</commit_message>
<xml_diff>
--- a/Tablas/Tablas_Stock.xlsx
+++ b/Tablas/Tablas_Stock.xlsx
@@ -458,7 +458,7 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>Total 2947 incidentes en julio (-31% vs junio, 4311). Caida generalizada: ARBOLADO -61%, CTRL ACTIVIDADES -47%, RESIDUOS -41% (1450 casos, 49% del volumen). Unica suba: CTRL ESPACIO +6%.</t>
+          <t>Total 3559 incidentes en agosto (20% vs julio, 2947). Suba en las SIETE areas: ARBOLADO +123%, CTRL ACTIVIDADES +55%, ALUMBRADO +42%, CALLES +25%, RESIDUOS +14% (1657 casos, 47% del volumen). Mayor movimiento por tipo: Luminaria apagada 262 a 398 (+136).</t>
         </is>
       </c>
     </row>
@@ -470,7 +470,7 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>Cierre global 76% (-3pp vs junio). RESIDUOS 88%, ALUMBRADO 81% y CTRL ACTIVIDADES 78% lideran; ARBOLADO recupera a 60%. Critico: CALLES 13%, quinto mes en zona critica. Cancelado sobre cerrados: CALLES 35% y TRANSITO 11%; resto &lt;=4%.</t>
+          <t>Cierre global 73% (-3pp vs julio). ALUMBRADO 89%, RESIDUOS 86% y CTRL ACTIVIDADES 78% lideran. Critico: CALLES 20% (sexto mes en zona critica) y ARBOLADO cae a 49%. Cancelado sobre cerrados: ninguna area supera el 10% (maximo TRANSITO y ARBOLADO 8%).</t>
         </is>
       </c>
     </row>
@@ -482,7 +482,7 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>SLA global 44% (+6pp vs junio). ALUMBRADO 61% lidera; CALLES y CTRL ACTIVIDADES 54%. Mas bajos: TRANSITO 31% y CTRL ESPACIO 39%. Promedio 6 dias para cerrados; ARBOLADO sube a 9 dias.</t>
+          <t>SLA global 51% (+7pp vs julio). ARBOLADO 77% y CTRL ESPACIO 76% lideran; ALUMBRADO 62%. Mas bajos: TRANSITO y CALLES 31%. Promedio 5 dias para cerrados; CALLES sube a 9 dias.</t>
         </is>
       </c>
     </row>
@@ -494,7 +494,7 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>Satisfaccion global 67% (-3pp vs junio). Encuesta normalizada: 476 respuestas, tasa 16.2% del total (21% s/incidentes con email). RESIDUOS 73% y ALUMBRADO 62%; CTRL ACTIVIDADES 10%. CALLES y TRANSITO con muestra insuficiente.</t>
+          <t>Satisfaccion global 69% (+2pp vs julio). 526 respuestas, tasa 14.8% del total (18% s/incidentes con email). RESIDUOS 73%, ALUMBRADO 72% y TRANSITO 71%; CTRL ACTIVIDADES 33%. CALLES y TRANSITO con muestra insuficiente.</t>
         </is>
       </c>
     </row>
@@ -536,7 +536,7 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>Cierre 81% sobre 401 incidentes; 'Luminaria superior e inferior apagada du' lidera con 262 casos (82% cierre). Gestion interna 56%.</t>
+          <t>Cierre 89% sobre 565 incidentes; 'Luminaria superior e inferior apagada du' lidera con 398 casos (91% cierre). Gestion interna 50%.</t>
         </is>
       </c>
     </row>
@@ -548,7 +548,7 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>Cierre moderado 60% sobre 47 incidentes; 'Inconvenientes con intervenciones de arb' lidera con 19 casos (84% cierre). Dias prom 9.0 elevado.</t>
+          <t>Cierre bajo 49% sobre 98 incidentes; 'Inconvenientes con intervenciones de arb' lidera con 33 casos (88% cierre). SLA 77%, sat 54%.</t>
         </is>
       </c>
     </row>
@@ -560,7 +560,7 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>Cierre critico 13% sobre 295 incidentes; 'Bache en calle de asfalto' lidera con 109 casos (10% cierre). Sat 50% (muestra insuficiente).</t>
+          <t>Cierre bajo 20% sobre 405 incidentes; 'Bache en calle de asfalto' lidera con 178 casos (19% cierre). Dias prom 9.0 elevado.</t>
         </is>
       </c>
     </row>
@@ -572,7 +572,7 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>Cierre 78% sobre 67 incidentes; 'Falta de Habilitación - Actividad no dec' lidera con 22 casos (82% cierre). SLA 54%, sat 10%.</t>
+          <t>Cierre 78% sobre 101 incidentes; 'Falta de Habilitación - Actividad no dec' lidera con 37 casos (89% cierre). SLA 52%, sat 33%.</t>
         </is>
       </c>
     </row>
@@ -584,7 +584,7 @@
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>Cierre 74% sobre 262 incidentes; 'Cable cortado' lidera con 115 casos (71% cierre). SLA 39%, sat 56%.</t>
+          <t>Cierre moderado 55% sobre 275 incidentes; 'Cable cortado' lidera con 77 casos (12% cierre). SLA 76%, sat 47%.</t>
         </is>
       </c>
     </row>
@@ -596,7 +596,7 @@
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>Cierre 88% sobre 1450 incidentes; 'Retiro de escombros y/o restos de obra' lidera con 437 casos (90% cierre). SLA 43%, sat 73%.</t>
+          <t>Cierre 86% sobre 1657 incidentes; 'Retiro de escombros y/o restos de obra' lidera con 468 casos (91% cierre). SLA 50%, sat 73%.</t>
         </is>
       </c>
     </row>
@@ -608,7 +608,7 @@
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>Cierre 75% sobre 425 incidentes; 'Vehículos Abandonados' lidera con 333 casos (81% cierre). Sat 56% (muestra insuficiente).</t>
+          <t>Cierre 70% sobre 458 incidentes; 'Vehículos Abandonados' lidera con 346 casos (76% cierre). Sat 71% (muestra insuficiente).</t>
         </is>
       </c>
     </row>
@@ -623,7 +623,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F9"/>
+  <dimension ref="A1:F10"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -674,7 +674,7 @@
       </c>
       <c r="B2" s="2" t="inlineStr">
         <is>
-          <t>Jun-2026</t>
+          <t>Jul-2026</t>
         </is>
       </c>
       <c r="C2" s="2" t="inlineStr">
@@ -684,17 +684,17 @@
       </c>
       <c r="D2" s="2" t="inlineStr">
         <is>
-          <t>Cierre bajo del area</t>
+          <t>Dias promedio alto</t>
         </is>
       </c>
       <c r="E2" s="2" t="inlineStr">
         <is>
-          <t>40%-&gt;60%</t>
+          <t>4 dias</t>
         </is>
       </c>
       <c r="F2" s="2" t="inlineStr">
         <is>
-          <t>Cierre del area sube de 40% a 60% (Jun-2026 a Jul-2026). Recuperacion significativa.</t>
+          <t>Tiempo promedio de resolucion baja a 4 dias en Ago-2026 (tablero). Vuelve a parametro habitual.</t>
         </is>
       </c>
     </row>
@@ -706,27 +706,27 @@
       </c>
       <c r="B3" s="2" t="inlineStr">
         <is>
-          <t>Jun-2026</t>
+          <t>Jul-2026</t>
         </is>
       </c>
       <c r="C3" s="2" t="inlineStr">
         <is>
-          <t>GENERAL</t>
+          <t>Calles y Veredas</t>
         </is>
       </c>
       <c r="D3" s="2" t="inlineStr">
         <is>
-          <t>Muestra de encuesta insuficiente (municipio)</t>
+          <t>Cancelado alto en cerrados</t>
         </is>
       </c>
       <c r="E3" s="2" t="inlineStr">
         <is>
-          <t>Tasa 16.2% (476 resp.)</t>
+          <t>5% (sobre cerrados)</t>
         </is>
       </c>
       <c r="F3" s="2" t="inlineStr">
         <is>
-          <t>La tasa de respuesta de encuesta se recupera en julio: 476 respuestas sobre 2947 incidentes (16.2% del total; 21% sobre incidentes con email segun tablero), tras los inconvenientes tecnicos de junio. Solo Calles y Veredas (2.7%) y Transito (2.1%) permanecen debajo del 5%; su satisfaccion se publica con la marca (muestra insuficiente).</t>
+          <t>Cancelado baja a 5% de los cerrados en Ago-2026 (donut Cierres por Estado), dentro del rango operativo.</t>
         </is>
       </c>
     </row>
@@ -738,27 +738,27 @@
       </c>
       <c r="B4" s="2" t="inlineStr">
         <is>
-          <t>Jun-2026</t>
+          <t>Jul-2026</t>
         </is>
       </c>
       <c r="C4" s="2" t="inlineStr">
         <is>
-          <t>Residuos y Limpieza</t>
+          <t>Transito</t>
         </is>
       </c>
       <c r="D4" s="2" t="inlineStr">
         <is>
-          <t>Cierre bajo en Falta de recoleccion de residuos reciclables</t>
+          <t>Cancelado alto en cerrados</t>
         </is>
       </c>
       <c r="E4" s="2" t="inlineStr">
         <is>
-          <t>37 casos, 100% cierre</t>
+          <t>8% (sobre cerrados)</t>
         </is>
       </c>
       <c r="F4" s="2" t="inlineStr">
         <is>
-          <t>Cierre bajo en Falta de recoleccion de residuos reciclables: 37 casos, cierre 22%-&gt;100% (Jun-2026 a Jul-2026). Recuperacion del cierre.</t>
+          <t>Cancelado baja a 8% de los cerrados en Ago-2026 (donut Cierres por Estado), dentro del rango operativo.</t>
         </is>
       </c>
     </row>
@@ -785,19 +785,19 @@
       </c>
       <c r="E5" s="3" t="inlineStr">
         <is>
-          <t>23%-&gt;13%</t>
+          <t>13%-&gt;20%</t>
         </is>
       </c>
       <c r="F5" s="3" t="inlineStr">
         <is>
-          <t>Cierre del area 23%-&gt;13% (Jun-2026 a Jul-2026). Sigue en zona critica. Cancelado 35% sobre cerrados.</t>
+          <t>Cierre del area 13%-&gt;20% (Jul-2026 a Ago-2026). Sigue en zona critica. Cancelado 5% sobre cerrados.</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" s="3" t="inlineStr">
         <is>
-          <t>NUEVA</t>
+          <t>PERSISTE</t>
         </is>
       </c>
       <c r="B6" s="3" t="inlineStr">
@@ -807,22 +807,22 @@
       </c>
       <c r="C6" s="3" t="inlineStr">
         <is>
-          <t>Arbolado y Plazas</t>
+          <t>Control de Actividades Comerciales</t>
         </is>
       </c>
       <c r="D6" s="3" t="inlineStr">
         <is>
-          <t>Dias promedio alto</t>
+          <t>Brecha cierre-satisfaccion</t>
         </is>
       </c>
       <c r="E6" s="3" t="inlineStr">
         <is>
-          <t>9 dias</t>
+          <t>Cierre 78% / Sat 33%</t>
         </is>
       </c>
       <c r="F6" s="3" t="inlineStr">
         <is>
-          <t>Tiempo promedio de resolucion 9 dias en Jul-2026 (tablero). Por encima del tiempo habitual.</t>
+          <t>Cierre 78% con satisfaccion 33% en Ago-2026 (tablero). La brecha entre gestion cerrada y percepcion del vecino se mantiene.</t>
         </is>
       </c>
     </row>
@@ -834,27 +834,27 @@
       </c>
       <c r="B7" s="3" t="inlineStr">
         <is>
-          <t>Jul-2026</t>
+          <t>Ago-2026</t>
         </is>
       </c>
       <c r="C7" s="3" t="inlineStr">
         <is>
-          <t>Calles y Veredas</t>
+          <t>Arbolado y Plazas</t>
         </is>
       </c>
       <c r="D7" s="3" t="inlineStr">
         <is>
-          <t>Cancelado alto en cerrados</t>
+          <t>Cierre bajo (area)</t>
         </is>
       </c>
       <c r="E7" s="3" t="inlineStr">
         <is>
-          <t>35% (sobre cerrados)</t>
+          <t>49%</t>
         </is>
       </c>
       <c r="F7" s="3" t="inlineStr">
         <is>
-          <t>35% de los cerrados son Cancelados en Jul-2026 (donut Cierres por Estado). Revisar calidad de cierre.</t>
+          <t>Cierre del area 49% en Ago-2026 (tablero). Cancelado 8% sobre cerrados.</t>
         </is>
       </c>
     </row>
@@ -866,27 +866,27 @@
       </c>
       <c r="B8" s="3" t="inlineStr">
         <is>
-          <t>Jul-2026</t>
+          <t>Ago-2026</t>
         </is>
       </c>
       <c r="C8" s="3" t="inlineStr">
         <is>
-          <t>Control de Actividades Comerciales</t>
+          <t>Calles y Veredas</t>
         </is>
       </c>
       <c r="D8" s="3" t="inlineStr">
         <is>
-          <t>Brecha cierre-satisfaccion</t>
+          <t>Dias promedio alto</t>
         </is>
       </c>
       <c r="E8" s="3" t="inlineStr">
         <is>
-          <t>Cierre 78% / Sat 10%</t>
+          <t>9 dias</t>
         </is>
       </c>
       <c r="F8" s="3" t="inlineStr">
         <is>
-          <t>Cierre 78% con satisfaccion 10%. Vecinos no perciben resolucion efectiva.</t>
+          <t>Tiempo promedio de resolucion 9 dias en Ago-2026 (tablero). Por encima del tiempo habitual.</t>
         </is>
       </c>
     </row>
@@ -898,27 +898,59 @@
       </c>
       <c r="B9" s="3" t="inlineStr">
         <is>
-          <t>Jul-2026</t>
+          <t>Ago-2026</t>
         </is>
       </c>
       <c r="C9" s="3" t="inlineStr">
         <is>
-          <t>Transito</t>
+          <t>Control del Espacio Publico</t>
         </is>
       </c>
       <c r="D9" s="3" t="inlineStr">
         <is>
-          <t>Cancelado alto en cerrados</t>
+          <t>Cierre bajo - Cable cortado</t>
         </is>
       </c>
       <c r="E9" s="3" t="inlineStr">
         <is>
-          <t>11% (sobre cerrados)</t>
+          <t>12% (77 casos)</t>
         </is>
       </c>
       <c r="F9" s="3" t="inlineStr">
         <is>
-          <t>11% de los cerrados son Cancelados en Jul-2026 (donut Cierres por Estado). Revisar calidad de cierre.</t>
+          <t>Tipo 'Cable cortado': 77 casos en Ago-2026 con 12% de cierre (tablero). Cierre muy por debajo del resto del area.</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="3" t="inlineStr">
+        <is>
+          <t>NUEVA</t>
+        </is>
+      </c>
+      <c r="B10" s="3" t="inlineStr">
+        <is>
+          <t>Ago-2026</t>
+        </is>
+      </c>
+      <c r="C10" s="3" t="inlineStr">
+        <is>
+          <t>Control del Espacio Publico</t>
+        </is>
+      </c>
+      <c r="D10" s="3" t="inlineStr">
+        <is>
+          <t>Cierre bajo - Poste en mal estado/sin mantenimiento</t>
+        </is>
+      </c>
+      <c r="E10" s="3" t="inlineStr">
+        <is>
+          <t>22% (23 casos)</t>
+        </is>
+      </c>
+      <c r="F10" s="3" t="inlineStr">
+        <is>
+          <t>Tipo 'Poste en mal estado/sin mantenimiento': 23 casos en Ago-2026 con 22% de cierre (tablero). Cierre muy por debajo del resto del area.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Stock_KPIs agosto 2026 - textos con tildes (coherencia con Stock_Areas)
</commit_message>
<xml_diff>
--- a/Tablas/Tablas_Stock.xlsx
+++ b/Tablas/Tablas_Stock.xlsx
@@ -458,7 +458,7 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>Demanda del vecino 3559 casos: sube 20% vs julio pero sigue 22% por debajo del promedio 2026 (4.580) y es el 2do mes mas bajo del ano. La carga baja 30% desde el pico de abril (5.074): mejora sostenida. Excepcion: CALLES Y VEREDAS 405, maximo de toda la serie y en alza todo el ano.</t>
+          <t>Demanda del vecino 3.559 casos: sube 20% vs julio pero sigue 22% por debajo del promedio 2026 (4.580) y es el 2do mes más bajo del año. La carga baja 30% desde el pico de abril (5.074): mejora sostenida. Excepción: CALLES Y VEREDAS 405, máximo de toda la serie y en alza todo el año.</t>
         </is>
       </c>
     </row>
@@ -470,7 +470,7 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>Cierre global 73% (-3pp vs julio). ALUMBRADO 89%, RESIDUOS 86% y CTRL ACTIVIDADES 78% lideran. Critico: CALLES 20% (sexto mes en zona critica) y ARBOLADO cae a 49%. Cancelado sobre cerrados: ninguna area supera el 10% (maximo TRANSITO y ARBOLADO 8%).</t>
+          <t>Cierre global 73% (-3pp vs julio). ALUMBRADO 89%, RESIDUOS 86% y CTRL ACTIVIDADES 78% lideran. Crítico: CALLES 20% (sexto mes en zona crítica) y ARBOLADO cae a 49%. Cancelado sobre cerrados: ninguna área supera el 10% (máximo TRÁNSITO y ARBOLADO 8%).</t>
         </is>
       </c>
     </row>
@@ -482,7 +482,7 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>SLA global 51% (+7pp vs julio). ARBOLADO 77% y CTRL ESPACIO 76% lideran; ALUMBRADO 62%. Mas bajos: TRANSITO y CALLES 31%. Promedio 5 dias para cerrados; CALLES sube a 9 dias.</t>
+          <t>SLA global 51% (+7pp vs julio). ARBOLADO 77% y CTRL ESPACIO 76% lideran; ALUMBRADO 62%. Más bajos: TRÁNSITO y CALLES 31%. Promedio 5 días para cerrados; CALLES sube a 9 días.</t>
         </is>
       </c>
     </row>
@@ -494,7 +494,7 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>Satisfaccion global 69% (+2pp vs julio). 526 respuestas, tasa 14.8% del total (18% s/incidentes con email). RESIDUOS 73%, ALUMBRADO 72% y TRANSITO 71%; CTRL ACTIVIDADES 33%. CALLES y TRANSITO con muestra insuficiente.</t>
+          <t>Satisfacción global 69% (+2pp vs julio). 526 respuestas, tasa 14.8% del total (18% s/incidentes con email). RESIDUOS 73%, ALUMBRADO 72% y TRÁNSITO 71%; CTRL ACTIVIDADES 33%. CALLES y TRÁNSITO con muestra insuficiente.</t>
         </is>
       </c>
     </row>

</xml_diff>